<commit_message>
V5 daily refresh 2026-09-14
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3">
@@ -868,7 +868,7 @@
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>35.73</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -964,7 +964,7 @@
         <v>73.94</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -1012,7 +1012,7 @@
         <v>27.21</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -1060,7 +1060,7 @@
         <v>7.91</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1108,7 +1108,7 @@
         <v>170.46</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1156,7 +1156,7 @@
         <v>13.22</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1204,7 +1204,7 @@
         <v>92.48999999999999</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1252,7 +1252,7 @@
         <v>92.61</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1300,7 +1300,7 @@
         <v>25.79</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1348,7 +1348,7 @@
         <v>24.01</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1396,7 +1396,7 @@
         <v>47.59</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1444,7 +1444,7 @@
         <v>73.94</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -6073,7 +6073,7 @@
         <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8295373652737494</v>
+        <v>0.8291526291099833</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6111,7 +6111,7 @@
         <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8127752712428832</v>
+        <v>0.8131066356774276</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6146,10 +6146,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8347597307265371</v>
+        <v>0.8350077117716462</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6187,7 +6187,7 @@
         <v>6.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.782817524259677</v>
+        <v>0.7826973787084026</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6225,7 +6225,7 @@
         <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7818942242274501</v>
+        <v>0.7814046796594026</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6263,7 +6263,7 @@
         <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7937161170193719</v>
+        <v>0.7931820120260992</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6301,7 +6301,7 @@
         <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7754404339886132</v>
+        <v>0.7755400017058296</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6339,7 +6339,7 @@
         <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7690704336305368</v>
+        <v>0.7690043640809132</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6377,7 +6377,7 @@
         <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7695744261825473</v>
+        <v>0.7691356774276088</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6415,7 +6415,7 @@
         <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7697217746267053</v>
+        <v>0.7696504470695268</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6453,7 +6453,7 @@
         <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7736752963082322</v>
+        <v>0.7739665515231637</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6491,7 +6491,7 @@
         <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7780409639417052</v>
+        <v>0.778033178387138</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6529,7 +6529,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.773216779460737</v>
+        <v>0.772761987007264</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6567,7 +6567,7 @@
         <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7718695169549181</v>
+        <v>0.7714159807809857</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -6605,7 +6605,7 @@
         <v>6.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7688973036846063</v>
+        <v>0.7690201785435057</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-15
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 11 Sep 2026</t>
+          <t>As of Tue 15 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹201,910</t>
+          <t>₹199,656</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-771  (-0.38%)</t>
+          <t>₹-2,254  (-1.12%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.95%</t>
+          <t>-0.17%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-2.03%</t>
+          <t>-3.13%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹80,236</t>
+          <t>₹97,028</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹120,198</t>
+          <t>₹102,599</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹121,674</t>
+          <t>₹102,628</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹+541</t>
+          <t>₹-285</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8836</v>
+        <v>8714</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8836</v>
+        <v>8714</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-81.5</v>
+        <v>-203.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.009139332772638072</v>
+        <v>-0.02282029716848893</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03382299683114538</v>
+        <v>0.02029607528115683</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>8813</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1226.4</v>
+        <v>1213.6</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>8584.800000000001</v>
+        <v>8495.199999999999</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-228.1999999999994</v>
+        <v>-317.8000000000006</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02589356632247809</v>
+        <v>-0.03606036536934082</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1182.47</v>
@@ -910,13 +910,13 @@
         <v>1182.47</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.03582028701891721</v>
+        <v>0.02565095583388257</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>35.73</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9029.5</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1968.5</v>
+        <v>1932.4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9842.5</v>
+        <v>9662</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>812.9999999999995</v>
+        <v>632.5</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.0900382080956863</v>
+        <v>0.07004817542499585</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1605.14</v>
@@ -958,115 +958,115 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07577198011538891</v>
+        <v>0.05850607682526555</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>721.55</v>
+        <v>333.9</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>8658.6</v>
+        <v>9015.299999999999</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>705.45</v>
+        <v>336.2</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>8465.400000000001</v>
+        <v>9077.4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>-193.1999999999989</v>
+        <v>62.10000000000031</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-0.02231307601690792</v>
+        <v>0.006888289907157866</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>664.91</v>
+        <v>317.56</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>685.5</v>
+        <v>327.8214285714286</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.0282798213906018</v>
+        <v>0.02492139032888571</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>27.21</v>
+        <v>7.91</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>333.9</v>
+        <v>9239</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>9015.299999999999</v>
+        <v>9239</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>344.5</v>
+        <v>9198</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9301.5</v>
+        <v>9198</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>286.2000000000006</v>
+        <v>-41</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.03174603174603181</v>
+        <v>-0.004437709708842948</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>317.56</v>
+        <v>8902.93</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>327.8214285714286</v>
+        <v>8902.93</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04841385030064264</v>
+        <v>0.03207979995651225</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>7.91</v>
+        <v>170.46</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1075,94 +1075,94 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>9239</v>
+        <v>702</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>9239</v>
+        <v>9126</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>9322</v>
+        <v>715</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9322</v>
+        <v>9295</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>83</v>
+        <v>169</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.008983656239852799</v>
+        <v>0.01851851851851852</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>8902.93</v>
+        <v>683.88</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>8902.93</v>
+        <v>701.55</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.04495494529071012</v>
+        <v>0.01881118881118888</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>170.46</v>
+        <v>13.22</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>702</v>
+        <v>4884.8</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>9126</v>
+        <v>4884.8</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>718.5</v>
+        <v>4695</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>9340.5</v>
+        <v>4695</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>214.5</v>
+        <v>-189.8000000000002</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.0235042735042735</v>
+        <v>-0.03885522436947268</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>683.88</v>
+        <v>4669.86</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>701.55</v>
+        <v>4669.86</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.02359081419624224</v>
+        <v>0.005354632587859494</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>13.22</v>
+        <v>92.61</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,46 +1171,46 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>4470</v>
+        <v>690</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>8940</v>
+        <v>8970</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4368.1</v>
+        <v>684</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8736.200000000001</v>
+        <v>8892</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-203.7999999999993</v>
+        <v>-78</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.0227964205816554</v>
+        <v>-0.008695652173913044</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>4302.67</v>
+        <v>627</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>4302.67</v>
+        <v>627</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.01497905267736551</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>92.48999999999999</v>
+        <v>25.79</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -1219,46 +1219,46 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>4884.8</v>
+        <v>844.5</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>4884.8</v>
+        <v>9289.5</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4905</v>
+        <v>872.6</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4905</v>
+        <v>9598.6</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>20.19999999999982</v>
+        <v>309.1000000000003</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.004135276776940677</v>
+        <v>0.03327412670219067</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>4669.86</v>
+        <v>801.9400000000001</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>4669.86</v>
+        <v>805.1999999999999</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.04793883792048936</v>
+        <v>0.07724043089617245</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>92.61</v>
+        <v>24.01</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1267,46 +1267,46 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>690</v>
+        <v>1474.1</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>8970</v>
+        <v>8844.6</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>691.75</v>
+        <v>1418.1</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8992.75</v>
+        <v>8508.599999999999</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>22.75</v>
+        <v>-336</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.002536231884057971</v>
+        <v>-0.03798928159554983</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>627</v>
+        <v>1378.14</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>627</v>
+        <v>1378.14</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.09360318033971811</v>
+        <v>0.02817854876242847</v>
       </c>
       <c r="M12" s="13" t="n">
-        <v>25.79</v>
+        <v>47.59</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1315,140 +1315,44 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>844.5</v>
+        <v>2306.1</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>9289.5</v>
+        <v>9224.4</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>909.3</v>
+        <v>2311.7</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>10002.3</v>
+        <v>9246.799999999999</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>712.7999999999995</v>
+        <v>22.39999999999964</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.07673179396092357</v>
+        <v>0.00242834222280036</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>801.9400000000001</v>
+        <v>2152.33</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>805.1999999999999</v>
+        <v>2152.33</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.1144836687561861</v>
+        <v>0.06894060648007955</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>24.01</v>
+        <v>73.94</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>MEDANTA</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>1474.1</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>8844.6</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>1447.2</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>8683.200000000001</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>-161.3999999999992</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>-0.01824842276643366</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>1378.14</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>1378.14</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>0.04771973466003313</v>
-      </c>
-      <c r="M14" s="13" t="n">
-        <v>47.59</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>SJS</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>2306.1</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>9224.4</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>2354</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>9416</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>191.6000000000004</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0.02077099865573917</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>2152.33</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>2152.33</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>0.08567119796091761</v>
-      </c>
-      <c r="M15" s="13" t="n">
-        <v>73.94</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H15">
+  <conditionalFormatting sqref="H2:H13">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1466,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1542,7 +1446,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -1551,18 +1455,18 @@
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>1849</v>
+        <v>721.55</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>1765.23</v>
+        <v>685.5</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1570,42 +1474,42 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-449.58</v>
+        <v>-461.33</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0486</v>
+        <v>-0.0533</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-1.07</v>
+        <v>-0.68</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>1902.4</v>
+        <v>4470</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>1886.44</v>
+        <v>4302.67</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1613,42 +1517,42 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-89.47</v>
+        <v>-364.46</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0118</v>
+        <v>-0.0408</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-0.38</v>
+        <v>-1.09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>830</v>
+        <v>1849</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>820</v>
+        <v>1765.23</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1656,22 +1560,22 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-140.73</v>
+        <v>-449.58</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0154</v>
+        <v>-0.0486</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-0.48</v>
+        <v>-1.07</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
@@ -1680,18 +1584,18 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1800</v>
+        <v>1902.4</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>1819.38</v>
+        <v>1886.44</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1699,42 +1603,42 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>96.89</v>
+        <v>-89.47</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.0108</v>
+        <v>-0.0118</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>0.28</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>856.5</v>
+        <v>830</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>816</v>
+        <v>820</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1742,22 +1646,22 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-405</v>
+        <v>-140.73</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0473</v>
+        <v>-0.0154</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.85</v>
+        <v>-0.48</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1766,10 +1670,10 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>817.6</v>
+        <v>1800</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
@@ -1777,7 +1681,7 @@
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>773.4</v>
+        <v>1819.38</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1788,39 +1692,39 @@
         <v>9</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>-486.2</v>
+        <v>96.89</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>-0.0541</v>
+        <v>0.0108</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>-0.96</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>UNITDSPR</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1510</v>
+        <v>856.5</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>1459</v>
+        <v>816</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1828,85 +1732,85 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-306</v>
+        <v>-405</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0338</v>
+        <v>-0.0473</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.89</v>
+        <v>-0.85</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>1412.6</v>
+        <v>817.6</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>1472.2</v>
+        <v>773.4</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>178.8</v>
+        <v>-486.2</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>0.0422</v>
+        <v>-0.0541</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>0.72</v>
+        <v>-0.96</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>UNITDSPR</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1478.7</v>
+        <v>1510</v>
       </c>
       <c r="D10" s="16" t="n">
         <v>6</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1448.3</v>
+        <v>1459</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1914,65 +1818,65 @@
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-182.4</v>
+        <v>-306</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0206</v>
+        <v>-0.0338</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-0.44</v>
+        <v>-0.89</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1423.8</v>
+        <v>1412.6</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>1414.5</v>
+        <v>1472.2</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>-55.8</v>
+        <v>178.8</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>-0.0065</v>
+        <v>0.0422</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>-0.17</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -1981,18 +1885,18 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>2058</v>
+        <v>1478.7</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>2021.3</v>
+        <v>1448.3</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -2000,108 +1904,108 @@
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-146.8</v>
+        <v>-182.4</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0178</v>
+        <v>-0.0206</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1624.8</v>
+        <v>1423.8</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>1802</v>
+        <v>1414.5</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>531.6</v>
+        <v>-55.8</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.1091</v>
+        <v>-0.0065</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>1.69</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>1588.9</v>
+        <v>2058</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>1649</v>
+        <v>2021.3</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>180.3</v>
+        <v>-146.8</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>0.0378</v>
+        <v>-0.0178</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>0.67</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2110,10 +2014,10 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>728.8</v>
+        <v>1624.8</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
@@ -2121,7 +2025,7 @@
         </is>
       </c>
       <c r="F15" s="15" t="n">
-        <v>817.6</v>
+        <v>1802</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -2132,19 +2036,19 @@
         <v>25</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>621.6</v>
+        <v>531.6</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.1218</v>
+        <v>0.1091</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>1.7</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -2153,10 +2057,10 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>4120</v>
+        <v>1588.9</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
@@ -2164,7 +2068,7 @@
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>4639.8</v>
+        <v>1649</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -2175,19 +2079,19 @@
         <v>25</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>519.8</v>
+        <v>180.3</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.1262</v>
+        <v>0.0378</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>2.66</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2196,10 +2100,10 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>862</v>
+        <v>728.8</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
@@ -2207,7 +2111,7 @@
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>849.25</v>
+        <v>817.6</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -2218,19 +2122,19 @@
         <v>25</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>-76.5</v>
+        <v>621.6</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>-0.0148</v>
+        <v>0.1218</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>-0.33</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2239,147 +2143,147 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>1412.6</v>
+        <v>4120</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>1417.16</v>
+        <v>4639.8</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>13.69</v>
+        <v>519.8</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>0.0032</v>
+        <v>0.1262</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>0.07000000000000001</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>507</v>
+        <v>862</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>471.54</v>
+        <v>849.25</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-638.28</v>
+        <v>-76.5</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0699</v>
+        <v>-0.0148</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-1</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>8847</v>
+        <v>1412.6</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>9240</v>
+        <v>1417.16</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>393</v>
+        <v>13.69</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>0.0444</v>
+        <v>0.0032</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>0.74</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>1948.5</v>
+        <v>507</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>1922.5</v>
+        <v>471.54</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -2387,85 +2291,85 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-52</v>
+        <v>-638.28</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0133</v>
+        <v>-0.0699</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-0.36</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>4568</v>
+        <v>8847</v>
       </c>
       <c r="D22" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>4460</v>
+        <v>9240</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>-108</v>
+        <v>393</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>-0.0236</v>
+        <v>0.0444</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>-0.49</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1550</v>
+        <v>1948.5</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>1470.07</v>
+        <v>1922.5</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2473,22 +2377,22 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-239.79</v>
+        <v>-52</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0516</v>
+        <v>-0.0133</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.77</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2497,18 +2401,18 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>1713.4</v>
+        <v>4568</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1650</v>
+        <v>4460</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -2516,42 +2420,42 @@
         </is>
       </c>
       <c r="H24" s="14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I24" s="17" t="n">
-        <v>-190.2</v>
+        <v>-108</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.037</v>
+        <v>-0.0236</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.65</v>
+        <v>-0.49</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>2360</v>
+        <v>1550</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>2250.39</v>
+        <v>1470.07</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -2559,42 +2463,42 @@
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-548.05</v>
+        <v>-239.79</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0464</v>
+        <v>-0.0516</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-1</v>
+        <v>-0.77</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>8945</v>
+        <v>1713.4</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>8673.639999999999</v>
+        <v>1650</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2602,171 +2506,171 @@
         </is>
       </c>
       <c r="H26" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>-271.36</v>
+        <v>-190.2</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>-0.0303</v>
+        <v>-0.037</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>-1</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>2218</v>
+        <v>2360</v>
       </c>
       <c r="D27" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>2250.39</v>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="F27" s="15" t="n">
-        <v>2132.81</v>
-      </c>
-      <c r="G27" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H27" s="14" t="n">
-        <v>7</v>
-      </c>
       <c r="I27" s="17" t="n">
-        <v>-170.37</v>
+        <v>-548.05</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>-0.0384</v>
+        <v>-0.0464</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>-0.76</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>1269</v>
+        <v>8945</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>1365.2</v>
+        <v>8673.639999999999</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>673.4</v>
+        <v>-271.36</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>0.07580000000000001</v>
+        <v>-0.0303</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>1.11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>7579.5</v>
+        <v>2218</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>7567.5</v>
+        <v>2132.81</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H29" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>-12</v>
+        <v>-170.37</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>-0.0016</v>
+        <v>-0.0384</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>-0.03</v>
+        <v>-0.76</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>1798.5</v>
+        <v>1269</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>1747.8</v>
+        <v>1365.2</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -2777,125 +2681,125 @@
         <v>25</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>-253.5</v>
+        <v>673.4</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>-0.0282</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>-0.43</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>5438</v>
+        <v>7579.5</v>
       </c>
       <c r="D31" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>5381</v>
+        <v>7567.5</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-57</v>
+        <v>-12</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.0105</v>
+        <v>-0.0016</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>1784</v>
+        <v>1798.5</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1752.1</v>
+        <v>1747.8</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-63.8</v>
+        <v>-253.5</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0282</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>871.8</v>
+        <v>5438</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>830.15</v>
+        <v>5381</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -2903,108 +2807,108 @@
         </is>
       </c>
       <c r="H33" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-249.9</v>
+        <v>-57</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0105</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>420.3</v>
+        <v>1784</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>448.6</v>
+        <v>1752.1</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>622.6</v>
+        <v>-63.8</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0179</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>1465</v>
+        <v>871.8</v>
       </c>
       <c r="D35" s="16" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>1596.9</v>
+        <v>830.15</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>791.4</v>
+        <v>-249.9</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>0.09</v>
+        <v>-0.0478</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>1.32</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -3013,10 +2917,10 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>619.25</v>
+        <v>420.3</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
@@ -3024,7 +2928,7 @@
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>717.95</v>
+        <v>448.6</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -3035,19 +2939,19 @@
         <v>25</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>1480.5</v>
+        <v>622.6</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>0.1594</v>
+        <v>0.0673</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>3.55</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
@@ -3056,10 +2960,10 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>8700</v>
+        <v>1465</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
@@ -3067,7 +2971,7 @@
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>8805.5</v>
+        <v>1596.9</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
@@ -3078,31 +2982,31 @@
         <v>25</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>105.5</v>
+        <v>791.4</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.09</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>0.29</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>961.85</v>
+        <v>619.25</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
@@ -3110,42 +3014,42 @@
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>935.6</v>
+        <v>717.95</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H38" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>-236.25</v>
+        <v>1480.5</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.1594</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>-0.64</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>1560</v>
+        <v>8700</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
@@ -3153,50 +3057,50 @@
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>1547.4</v>
+        <v>8805.5</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H39" s="14" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>-63</v>
+        <v>105.5</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>-0.0081</v>
+        <v>0.0121</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>-0.23</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>900</v>
+        <v>961.85</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F40" s="15" t="n">
-        <v>887.1</v>
+        <v>935.6</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -3204,22 +3108,22 @@
         </is>
       </c>
       <c r="H40" s="14" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="I40" s="17" t="n">
-        <v>-129</v>
+        <v>-236.25</v>
       </c>
       <c r="J40" s="18" t="n">
-        <v>-0.0143</v>
+        <v>-0.0273</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>-0.2</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -3228,18 +3132,18 @@
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>880.8</v>
+        <v>1560</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F41" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>1547.4</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -3247,42 +3151,42 @@
         </is>
       </c>
       <c r="H41" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I41" s="17" t="n">
-        <v>-478.6</v>
+        <v>-63</v>
       </c>
       <c r="J41" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0081</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>-1</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>777</v>
+        <v>900</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F42" s="15" t="n">
-        <v>744.8</v>
+        <v>887.1</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
@@ -3290,42 +3194,42 @@
         </is>
       </c>
       <c r="H42" s="14" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="I42" s="17" t="n">
-        <v>-386.4</v>
+        <v>-129</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0143</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C43" s="15" t="n">
-        <v>1114.9</v>
+        <v>880.8</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E43" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F43" s="15" t="n">
-        <v>1050.57</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
@@ -3333,13 +3237,13 @@
         </is>
       </c>
       <c r="H43" s="14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I43" s="17" t="n">
-        <v>-514.64</v>
+        <v>-478.6</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0543</v>
       </c>
       <c r="K43" s="19" t="n">
         <v>-1</v>
@@ -3348,93 +3252,93 @@
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C44" s="15" t="n">
-        <v>790</v>
+        <v>777</v>
       </c>
       <c r="D44" s="16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E44" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F44" s="15" t="n">
-        <v>880.8</v>
+        <v>744.8</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H44" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I44" s="17" t="n">
-        <v>998.8</v>
+        <v>-386.4</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0414</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C45" s="15" t="n">
-        <v>3770</v>
+        <v>1114.9</v>
       </c>
       <c r="D45" s="16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E45" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F45" s="15" t="n">
-        <v>4097.9</v>
+        <v>1050.57</v>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H45" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I45" s="17" t="n">
-        <v>655.8</v>
+        <v>-514.64</v>
       </c>
       <c r="J45" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0577</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>1.98</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
@@ -3443,7 +3347,7 @@
         </is>
       </c>
       <c r="C46" s="15" t="n">
-        <v>821.05</v>
+        <v>790</v>
       </c>
       <c r="D46" s="16" t="n">
         <v>11</v>
@@ -3454,7 +3358,7 @@
         </is>
       </c>
       <c r="F46" s="15" t="n">
-        <v>844</v>
+        <v>880.8</v>
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
@@ -3465,19 +3369,19 @@
         <v>25</v>
       </c>
       <c r="I46" s="17" t="n">
-        <v>252.45</v>
+        <v>998.8</v>
       </c>
       <c r="J46" s="18" t="n">
-        <v>0.028</v>
+        <v>0.1149</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>0.6</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
@@ -3486,10 +3390,10 @@
         </is>
       </c>
       <c r="C47" s="15" t="n">
-        <v>2426.1</v>
+        <v>3770</v>
       </c>
       <c r="D47" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E47" s="14" t="inlineStr">
         <is>
@@ -3497,7 +3401,7 @@
         </is>
       </c>
       <c r="F47" s="15" t="n">
-        <v>2484.2</v>
+        <v>4097.9</v>
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
@@ -3508,39 +3412,39 @@
         <v>25</v>
       </c>
       <c r="I47" s="17" t="n">
-        <v>174.3</v>
+        <v>655.8</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K47" s="19" t="n">
-        <v>0.5</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C48" s="15" t="n">
-        <v>1410</v>
+        <v>821.05</v>
       </c>
       <c r="D48" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E48" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F48" s="15" t="n">
-        <v>1455.2</v>
+        <v>844</v>
       </c>
       <c r="G48" s="14" t="inlineStr">
         <is>
@@ -3551,39 +3455,39 @@
         <v>25</v>
       </c>
       <c r="I48" s="17" t="n">
-        <v>135.6</v>
+        <v>252.45</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.028</v>
       </c>
       <c r="K48" s="19" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C49" s="15" t="n">
-        <v>690</v>
+        <v>2426.1</v>
       </c>
       <c r="D49" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E49" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F49" s="15" t="n">
-        <v>660.45</v>
+        <v>2484.2</v>
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
@@ -3594,19 +3498,19 @@
         <v>25</v>
       </c>
       <c r="I49" s="17" t="n">
-        <v>-206.85</v>
+        <v>174.3</v>
       </c>
       <c r="J49" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.0239</v>
       </c>
       <c r="K49" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
@@ -3615,10 +3519,10 @@
         </is>
       </c>
       <c r="C50" s="15" t="n">
-        <v>1839</v>
+        <v>1410</v>
       </c>
       <c r="D50" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
@@ -3626,7 +3530,7 @@
         </is>
       </c>
       <c r="F50" s="15" t="n">
-        <v>1828.1</v>
+        <v>1455.2</v>
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
@@ -3637,19 +3541,19 @@
         <v>25</v>
       </c>
       <c r="I50" s="17" t="n">
-        <v>-21.8</v>
+        <v>135.6</v>
       </c>
       <c r="J50" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.0321</v>
       </c>
       <c r="K50" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B51" s="14" t="inlineStr">
@@ -3658,10 +3562,10 @@
         </is>
       </c>
       <c r="C51" s="15" t="n">
-        <v>1414</v>
+        <v>690</v>
       </c>
       <c r="D51" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E51" s="14" t="inlineStr">
         <is>
@@ -3669,7 +3573,7 @@
         </is>
       </c>
       <c r="F51" s="15" t="n">
-        <v>1537.8</v>
+        <v>660.45</v>
       </c>
       <c r="G51" s="14" t="inlineStr">
         <is>
@@ -3680,19 +3584,19 @@
         <v>25</v>
       </c>
       <c r="I51" s="17" t="n">
-        <v>371.4</v>
+        <v>-206.85</v>
       </c>
       <c r="J51" s="18" t="n">
-        <v>0.0876</v>
+        <v>-0.0428</v>
       </c>
       <c r="K51" s="19" t="n">
-        <v>1.38</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
@@ -3701,10 +3605,10 @@
         </is>
       </c>
       <c r="C52" s="15" t="n">
-        <v>1300</v>
+        <v>1839</v>
       </c>
       <c r="D52" s="16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E52" s="14" t="inlineStr">
         <is>
@@ -3712,7 +3616,7 @@
         </is>
       </c>
       <c r="F52" s="15" t="n">
-        <v>1389.1</v>
+        <v>1828.1</v>
       </c>
       <c r="G52" s="14" t="inlineStr">
         <is>
@@ -3723,19 +3627,19 @@
         <v>25</v>
       </c>
       <c r="I52" s="17" t="n">
-        <v>356.4</v>
+        <v>-21.8</v>
       </c>
       <c r="J52" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>-0.0059</v>
       </c>
       <c r="K52" s="19" t="n">
-        <v>0.63</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
@@ -3744,10 +3648,10 @@
         </is>
       </c>
       <c r="C53" s="15" t="n">
-        <v>276.45</v>
+        <v>1414</v>
       </c>
       <c r="D53" s="16" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E53" s="14" t="inlineStr">
         <is>
@@ -3755,7 +3659,7 @@
         </is>
       </c>
       <c r="F53" s="15" t="n">
-        <v>330.1</v>
+        <v>1537.8</v>
       </c>
       <c r="G53" s="14" t="inlineStr">
         <is>
@@ -3766,19 +3670,19 @@
         <v>25</v>
       </c>
       <c r="I53" s="17" t="n">
-        <v>1019.35</v>
+        <v>371.4</v>
       </c>
       <c r="J53" s="18" t="n">
-        <v>0.1941</v>
+        <v>0.0876</v>
       </c>
       <c r="K53" s="19" t="n">
-        <v>3.1</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
@@ -3787,10 +3691,10 @@
         </is>
       </c>
       <c r="C54" s="15" t="n">
-        <v>1462.5</v>
+        <v>1300</v>
       </c>
       <c r="D54" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E54" s="14" t="inlineStr">
         <is>
@@ -3798,7 +3702,7 @@
         </is>
       </c>
       <c r="F54" s="15" t="n">
-        <v>1564.7</v>
+        <v>1389.1</v>
       </c>
       <c r="G54" s="14" t="inlineStr">
         <is>
@@ -3809,19 +3713,19 @@
         <v>25</v>
       </c>
       <c r="I54" s="17" t="n">
-        <v>306.6</v>
+        <v>356.4</v>
       </c>
       <c r="J54" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K54" s="19" t="n">
-        <v>1.78</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B55" s="14" t="inlineStr">
@@ -3830,41 +3734,41 @@
         </is>
       </c>
       <c r="C55" s="15" t="n">
-        <v>798</v>
+        <v>276.45</v>
       </c>
       <c r="D55" s="16" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E55" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F55" s="15" t="n">
-        <v>750</v>
+        <v>330.1</v>
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H55" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I55" s="17" t="n">
-        <v>-288</v>
+        <v>1019.35</v>
       </c>
       <c r="J55" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.1941</v>
       </c>
       <c r="K55" s="19" t="n">
-        <v>-0.92</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
@@ -3873,53 +3777,53 @@
         </is>
       </c>
       <c r="C56" s="15" t="n">
-        <v>260.45</v>
+        <v>1462.5</v>
       </c>
       <c r="D56" s="16" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E56" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F56" s="15" t="n">
-        <v>257.85</v>
+        <v>1564.7</v>
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H56" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I56" s="17" t="n">
-        <v>-52.07</v>
+        <v>306.6</v>
       </c>
       <c r="J56" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.0699</v>
       </c>
       <c r="K56" s="19" t="n">
-        <v>-0.13</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C57" s="15" t="n">
-        <v>6500</v>
+        <v>798</v>
       </c>
       <c r="D57" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E57" s="14" t="inlineStr">
         <is>
@@ -3927,7 +3831,7 @@
         </is>
       </c>
       <c r="F57" s="15" t="n">
-        <v>6401.5</v>
+        <v>750</v>
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
@@ -3935,34 +3839,34 @@
         </is>
       </c>
       <c r="H57" s="14" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I57" s="17" t="n">
-        <v>-98.5</v>
+        <v>-288</v>
       </c>
       <c r="J57" s="18" t="n">
-        <v>-0.0152</v>
+        <v>-0.0602</v>
       </c>
       <c r="K57" s="19" t="n">
-        <v>-0.31</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C58" s="15" t="n">
-        <v>571.5</v>
+        <v>260.45</v>
       </c>
       <c r="D58" s="16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E58" s="14" t="inlineStr">
         <is>
@@ -3970,7 +3874,7 @@
         </is>
       </c>
       <c r="F58" s="15" t="n">
-        <v>571.1</v>
+        <v>257.85</v>
       </c>
       <c r="G58" s="14" t="inlineStr">
         <is>
@@ -3978,34 +3882,34 @@
         </is>
       </c>
       <c r="H58" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I58" s="17" t="n">
-        <v>-6.4</v>
+        <v>-52.07</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.01</v>
       </c>
       <c r="K58" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C59" s="15" t="n">
-        <v>965</v>
+        <v>6500</v>
       </c>
       <c r="D59" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E59" s="14" t="inlineStr">
         <is>
@@ -4013,7 +3917,7 @@
         </is>
       </c>
       <c r="F59" s="15" t="n">
-        <v>933</v>
+        <v>6401.5</v>
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
@@ -4021,22 +3925,22 @@
         </is>
       </c>
       <c r="H59" s="14" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="I59" s="17" t="n">
-        <v>-288</v>
+        <v>-98.5</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.0152</v>
       </c>
       <c r="K59" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B60" s="14" t="inlineStr">
@@ -4045,18 +3949,18 @@
         </is>
       </c>
       <c r="C60" s="15" t="n">
-        <v>5479</v>
+        <v>571.5</v>
       </c>
       <c r="D60" s="16" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E60" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F60" s="15" t="n">
-        <v>5424</v>
+        <v>571.1</v>
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
@@ -4064,42 +3968,42 @@
         </is>
       </c>
       <c r="H60" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I60" s="17" t="n">
-        <v>-55</v>
+        <v>-6.4</v>
       </c>
       <c r="J60" s="18" t="n">
+        <v>-0.0007</v>
+      </c>
+      <c r="K60" s="19" t="n">
         <v>-0.01</v>
-      </c>
-      <c r="K60" s="19" t="n">
-        <v>-0.18</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C61" s="15" t="n">
-        <v>960.1</v>
+        <v>965</v>
       </c>
       <c r="D61" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E61" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F61" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>933</v>
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
@@ -4107,42 +4011,42 @@
         </is>
       </c>
       <c r="H61" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I61" s="17" t="n">
-        <v>-516.79</v>
+        <v>-288</v>
       </c>
       <c r="J61" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0332</v>
       </c>
       <c r="K61" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C62" s="15" t="n">
-        <v>952.1</v>
+        <v>5479</v>
       </c>
       <c r="D62" s="16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E62" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F62" s="15" t="n">
-        <v>948.8</v>
+        <v>5424</v>
       </c>
       <c r="G62" s="14" t="inlineStr">
         <is>
@@ -4153,39 +4057,39 @@
         <v>1</v>
       </c>
       <c r="I62" s="17" t="n">
-        <v>-29.7</v>
+        <v>-55</v>
       </c>
       <c r="J62" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.01</v>
       </c>
       <c r="K62" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C63" s="15" t="n">
-        <v>1475</v>
+        <v>960.1</v>
       </c>
       <c r="D63" s="16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E63" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F63" s="15" t="n">
-        <v>1394.19</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
@@ -4193,42 +4097,42 @@
         </is>
       </c>
       <c r="H63" s="14" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I63" s="17" t="n">
-        <v>-484.86</v>
+        <v>-516.79</v>
       </c>
       <c r="J63" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.0598</v>
       </c>
       <c r="K63" s="19" t="n">
-        <v>-1</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C64" s="15" t="n">
-        <v>248.05</v>
+        <v>952.1</v>
       </c>
       <c r="D64" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E64" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F64" s="15" t="n">
-        <v>242.8</v>
+        <v>948.8</v>
       </c>
       <c r="G64" s="14" t="inlineStr">
         <is>
@@ -4236,42 +4140,42 @@
         </is>
       </c>
       <c r="H64" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I64" s="17" t="n">
-        <v>-110.25</v>
+        <v>-29.7</v>
       </c>
       <c r="J64" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0035</v>
       </c>
       <c r="K64" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C65" s="15" t="n">
-        <v>1039.2</v>
+        <v>1475</v>
       </c>
       <c r="D65" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E65" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F65" s="15" t="n">
-        <v>970</v>
+        <v>1394.19</v>
       </c>
       <c r="G65" s="14" t="inlineStr">
         <is>
@@ -4279,22 +4183,22 @@
         </is>
       </c>
       <c r="H65" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I65" s="17" t="n">
-        <v>-346</v>
+        <v>-484.86</v>
       </c>
       <c r="J65" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0548</v>
       </c>
       <c r="K65" s="19" t="n">
-        <v>-0.82</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
@@ -4303,10 +4207,10 @@
         </is>
       </c>
       <c r="C66" s="15" t="n">
-        <v>199.96</v>
+        <v>248.05</v>
       </c>
       <c r="D66" s="16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
@@ -4314,7 +4218,7 @@
         </is>
       </c>
       <c r="F66" s="15" t="n">
-        <v>193.31</v>
+        <v>242.8</v>
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
@@ -4325,19 +4229,19 @@
         <v>11</v>
       </c>
       <c r="I66" s="17" t="n">
-        <v>-172.9</v>
+        <v>-110.25</v>
       </c>
       <c r="J66" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0212</v>
       </c>
       <c r="K66" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
@@ -4346,7 +4250,7 @@
         </is>
       </c>
       <c r="C67" s="15" t="n">
-        <v>986.4</v>
+        <v>1039.2</v>
       </c>
       <c r="D67" s="16" t="n">
         <v>5</v>
@@ -4357,7 +4261,7 @@
         </is>
       </c>
       <c r="F67" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>970</v>
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
@@ -4368,17 +4272,103 @@
         <v>11</v>
       </c>
       <c r="I67" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J67" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K67" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D68" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E68" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F68" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G68" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H68" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I68" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J68" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K68" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D69" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F69" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G69" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H69" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I69" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J67" s="18" t="n">
+      <c r="J69" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K67" s="19" t="n">
+      <c r="K69" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I67">
+  <conditionalFormatting sqref="I2:I69">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -4396,7 +4386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5968,6 +5958,31 @@
       </c>
       <c r="G62" s="14" t="n">
         <v>14</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B63" s="20" t="n">
+        <v>199656</v>
+      </c>
+      <c r="C63" s="20" t="n">
+        <v>97027.8</v>
+      </c>
+      <c r="D63" s="20" t="n">
+        <v>102628.2</v>
+      </c>
+      <c r="E63" s="20" t="n">
+        <v>102599.2</v>
+      </c>
+      <c r="F63" s="20" t="n">
+        <v>-284.8</v>
+      </c>
+      <c r="G63" s="14" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -6050,18 +6065,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>909.3</v>
+        <v>4360</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>857.25</v>
+        <v>4168.96</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6070,10 +6085,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8291526291099833</v>
+        <v>0.8522804522752496</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6088,18 +6103,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>9322</v>
+        <v>790</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8865.639999999999</v>
+        <v>747.77</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6108,10 +6123,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8131066356774276</v>
+        <v>0.8204737791342952</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6126,18 +6141,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1909</v>
+        <v>872.6</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1810.1</v>
+        <v>815.5</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6149,7 +6164,7 @@
         <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8350077117716462</v>
+        <v>0.8099125971143174</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6164,18 +6179,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>NEULANDLAB</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>11763</v>
+        <v>22595</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>11117.57</v>
+        <v>21157.86</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6187,7 +6202,7 @@
         <v>6.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7826973787084026</v>
+        <v>0.8055788706992231</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6202,18 +6217,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1969</v>
+        <v>684</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1861.91</v>
+        <v>632.9400000000001</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6225,7 +6240,7 @@
         <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7814046796594026</v>
+        <v>0.7860831714761376</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6240,18 +6255,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>NEULANDLAB</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>23535</v>
+        <v>11803</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>22197.57</v>
+        <v>11152.86</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6260,10 +6275,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7931820120260992</v>
+        <v>0.7834298695893452</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6278,7 +6293,7 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -6286,10 +6301,10 @@
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>11678</v>
+        <v>11424</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>11212.43</v>
+        <v>10945.86</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6298,10 +6313,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7755400017058296</v>
+        <v>0.7807072003329634</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6316,18 +6331,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>EMCURE</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1585</v>
+        <v>1993</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1470.59</v>
+        <v>1898.37</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6336,10 +6351,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7690043640809132</v>
+        <v>0.8042712957824639</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6354,18 +6369,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>344.5</v>
+        <v>47070</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>329.21</v>
+        <v>44728.57</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6374,10 +6389,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7691356774276088</v>
+        <v>0.7781284683684796</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6392,18 +6407,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>VARROC</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>872</v>
+        <v>9198</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>798.95</v>
+        <v>8737.290000000001</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6412,10 +6427,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7696504470695268</v>
+        <v>0.7697957130965594</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6430,18 +6445,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>CORONA</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>2236.1</v>
+        <v>1906.4</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>2099.84</v>
+        <v>1810.24</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6453,7 +6468,7 @@
         <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7739665515231637</v>
+        <v>0.7734652469478357</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6468,18 +6483,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SIS</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>419.3</v>
+        <v>2311.7</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>398.44</v>
+        <v>2160.41</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -6488,10 +6503,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.778033178387138</v>
+        <v>0.7675447419533852</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6506,18 +6521,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>CORONA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1270</v>
+        <v>2217.9</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1185.54</v>
+        <v>2075.47</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -6529,7 +6544,7 @@
         <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.772761987007264</v>
+        <v>0.7727004716981132</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6544,18 +6559,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>BLSE</t>
+          <t>INNOVACAP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>312.8</v>
+        <v>1140.1</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>291.4</v>
+        <v>1038.86</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -6567,7 +6582,7 @@
         <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7714159807809857</v>
+        <v>0.7650874028856826</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -6582,18 +6597,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260911</v>
+        <v>20260915</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>EMCURE</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1978.9</v>
+        <v>480.05</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1883.63</v>
+        <v>450.86</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -6602,10 +6617,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7690201785435057</v>
+        <v>0.7797395255271921</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-16
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 15 Sep 2026</t>
+          <t>As of Wed 16 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹199,656</t>
+          <t>₹198,669</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-2,254  (-1.12%)</t>
+          <t>₹-987  (-0.49%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-0.17%</t>
+          <t>-0.67%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-3.13%</t>
+          <t>-3.60%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹97,028</t>
+          <t>₹118,761</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹102,599</t>
+          <t>₹79,886</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹102,628</t>
+          <t>₹79,908</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>₹-285</t>
+          <t>₹-1,275</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8714</v>
+        <v>8696.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8714</v>
+        <v>8696.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-203.5</v>
+        <v>-221</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.02282029716848893</v>
+        <v>-0.02478273058592655</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,19 +862,19 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.02029607528115683</v>
+        <v>0.01832461335019842</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -883,238 +883,238 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>1259</v>
+        <v>1805.9</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>8813</v>
+        <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1213.6</v>
+        <v>1950.7</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>8495.199999999999</v>
+        <v>9753.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-317.8000000000006</v>
+        <v>723.9999999999998</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.03606036536934082</v>
+        <v>0.08018162688963948</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>1182.47</v>
+        <v>1605.14</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1182.47</v>
+        <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.02565095583388257</v>
+        <v>0.0673384645804804</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>35.73</v>
+        <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1805.9</v>
+        <v>9239</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>9029.5</v>
+        <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1932.4</v>
+        <v>9158</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9662</v>
+        <v>9158</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>632.5</v>
+        <v>-81</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.07004817542499585</v>
+        <v>-0.008767182595518995</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>1605.14</v>
+        <v>8902.93</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1819.342857142857</v>
+        <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.05850607682526555</v>
+        <v>0.02785215112469968</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>73.94</v>
+        <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>333.9</v>
+        <v>702</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>9015.299999999999</v>
+        <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>336.2</v>
+        <v>713.4</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9077.4</v>
+        <v>9274.199999999999</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>62.10000000000031</v>
+        <v>148.1999999999997</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.006888289907157866</v>
+        <v>0.01623931623931621</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>317.56</v>
+        <v>683.88</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>327.8214285714286</v>
+        <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.02492139032888571</v>
+        <v>0.01661059714045419</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>7.91</v>
+        <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>9239</v>
+        <v>690</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>9239</v>
+        <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>9198</v>
+        <v>690.2</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9198</v>
+        <v>8972.6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-41</v>
+        <v>2.600000000000591</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.004437709708842948</v>
+        <v>0.000289855072463834</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>8902.93</v>
+        <v>627</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>8902.93</v>
+        <v>627</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.03207979995651225</v>
+        <v>0.09156766154737764</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>170.46</v>
+        <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>702</v>
+        <v>844.5</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>9126</v>
+        <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>715</v>
+        <v>835.6</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9295</v>
+        <v>9191.6</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>169</v>
+        <v>-97.89999999999975</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.01851851851851852</v>
+        <v>-0.01053878034339843</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>683.88</v>
+        <v>801.9400000000001</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>701.55</v>
+        <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.01881118881118888</v>
+        <v>0.0363810435615128</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>13.22</v>
+        <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1123,46 +1123,46 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>4884.8</v>
+        <v>1474.1</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>4884.8</v>
+        <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4695</v>
+        <v>1404.6</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4695</v>
+        <v>8427.599999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-189.8000000000002</v>
+        <v>-417</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.03885522436947268</v>
+        <v>-0.0471474119801913</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>4669.86</v>
+        <v>1378.14</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>4669.86</v>
+        <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.005354632587859494</v>
+        <v>0.01883810337462609</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>92.61</v>
+        <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1171,188 +1171,44 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>690</v>
+        <v>2306.1</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>8970</v>
+        <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>684</v>
+        <v>2297.2</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8892</v>
+        <v>9188.799999999999</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-78</v>
+        <v>-35.60000000000036</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.008695652173913044</v>
+        <v>-0.003859329604093531</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>627</v>
+        <v>2152.33</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>627</v>
+        <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.06306372975796617</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>25.79</v>
+        <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>GRANULES</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>844.5</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="E11" s="9" t="n">
-        <v>9289.5</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>872.6</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <v>9598.6</v>
-      </c>
-      <c r="H11" s="10" t="n">
-        <v>309.1000000000003</v>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>0.03327412670219067</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>801.9400000000001</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>805.1999999999999</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>0.07724043089617245</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <v>24.01</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>MEDANTA</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>1474.1</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>8844.6</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>1418.1</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>8508.599999999999</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <v>-336</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>-0.03798928159554983</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>1378.14</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>1378.14</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>0.02817854876242847</v>
-      </c>
-      <c r="M12" s="13" t="n">
-        <v>47.59</v>
-      </c>
-      <c r="N12" s="6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>SJS</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>2306.1</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>9224.4</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>2311.7</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>9246.799999999999</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>22.39999999999964</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0.00242834222280036</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>2152.33</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>2152.33</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>0.06894060648007955</v>
-      </c>
-      <c r="M13" s="13" t="n">
-        <v>73.94</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H13">
+  <conditionalFormatting sqref="H2:H10">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1370,7 +1226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1446,7 +1302,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -1455,18 +1311,18 @@
         </is>
       </c>
       <c r="C2" s="15" t="n">
-        <v>721.55</v>
+        <v>1259</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F2" s="15" t="n">
-        <v>685.5</v>
+        <v>1182.47</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -1474,42 +1330,42 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>-461.33</v>
+        <v>-564.84</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>-0.0533</v>
+        <v>-0.0641</v>
       </c>
       <c r="K2" s="19" t="n">
-        <v>-0.68</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C3" s="15" t="n">
-        <v>4470</v>
+        <v>333.9</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F3" s="15" t="n">
-        <v>4302.67</v>
+        <v>327.82</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -1517,42 +1373,42 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="I3" s="17" t="n">
-        <v>-364.46</v>
+        <v>-194.39</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>-0.0408</v>
+        <v>-0.0216</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>-1.09</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1849</v>
+        <v>4884.8</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F4" s="15" t="n">
-        <v>1765.23</v>
+        <v>4669.86</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -1560,42 +1416,42 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>-449.58</v>
+        <v>-231.18</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>-0.0486</v>
+        <v>-0.0473</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>-1.07</v>
+        <v>-1.08</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>1902.4</v>
+        <v>721.55</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F5" s="15" t="n">
-        <v>1886.44</v>
+        <v>685.5</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -1603,42 +1459,42 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="I5" s="17" t="n">
-        <v>-89.47</v>
+        <v>-461.33</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>-0.0118</v>
+        <v>-0.0533</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>-0.38</v>
+        <v>-0.68</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>830</v>
+        <v>4470</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F6" s="15" t="n">
-        <v>820</v>
+        <v>4302.67</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -1646,42 +1502,42 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I6" s="17" t="n">
-        <v>-140.73</v>
+        <v>-364.46</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>-0.0154</v>
+        <v>-0.0408</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>-0.48</v>
+        <v>-1.09</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>1800</v>
+        <v>1849</v>
       </c>
       <c r="D7" s="16" t="n">
         <v>5</v>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F7" s="15" t="n">
-        <v>1819.38</v>
+        <v>1765.23</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -1689,22 +1545,22 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>96.89</v>
+        <v>-449.58</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.0108</v>
+        <v>-0.0486</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>0.28</v>
+        <v>-1.07</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1713,18 +1569,18 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>856.5</v>
+        <v>1902.4</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
-        <v>816</v>
+        <v>1886.44</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -1732,42 +1588,42 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I8" s="17" t="n">
-        <v>-405</v>
+        <v>-89.47</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>-0.0473</v>
+        <v>-0.0118</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>-0.85</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>817.6</v>
+        <v>830</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>11</v>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
-        <v>773.4</v>
+        <v>820</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -1775,42 +1631,42 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>-486.2</v>
+        <v>-140.73</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>-0.0541</v>
+        <v>-0.0154</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>-0.96</v>
+        <v>-0.48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>UNITDSPR</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>1510</v>
+        <v>1800</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1459</v>
+        <v>1819.38</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -1818,65 +1674,65 @@
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>-306</v>
+        <v>96.89</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>-0.0338</v>
+        <v>0.0108</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>-0.89</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1412.6</v>
+        <v>856.5</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
-        <v>1472.2</v>
+        <v>816</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>178.8</v>
+        <v>-405</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>0.0422</v>
+        <v>-0.0473</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>0.72</v>
+        <v>-0.85</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -1885,18 +1741,18 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>1478.7</v>
+        <v>817.6</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F12" s="15" t="n">
-        <v>1448.3</v>
+        <v>773.4</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -1904,42 +1760,42 @@
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>-182.4</v>
+        <v>-486.2</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>-0.0206</v>
+        <v>-0.0541</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>-0.44</v>
+        <v>-0.96</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>UNITDSPR</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>1423.8</v>
+        <v>1510</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>6</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F13" s="15" t="n">
-        <v>1414.5</v>
+        <v>1459</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -1947,194 +1803,194 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>-55.8</v>
+        <v>-306</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>-0.0065</v>
+        <v>-0.0338</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>-0.17</v>
+        <v>-0.89</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>2058</v>
+        <v>1412.6</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F14" s="15" t="n">
-        <v>2021.3</v>
+        <v>1472.2</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>-146.8</v>
+        <v>178.8</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>-0.0178</v>
+        <v>0.0422</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>-0.3</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>1624.8</v>
+        <v>1478.7</v>
       </c>
       <c r="D15" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>1448.3</v>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="F15" s="15" t="n">
-        <v>1802</v>
-      </c>
-      <c r="G15" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H15" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I15" s="17" t="n">
-        <v>531.6</v>
+        <v>-182.4</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.1091</v>
+        <v>-0.0206</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>1.69</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>1588.9</v>
+        <v>1423.8</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F16" s="15" t="n">
-        <v>1649</v>
+        <v>1414.5</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>180.3</v>
+        <v>-55.8</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.0378</v>
+        <v>-0.0065</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>0.67</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>728.8</v>
+        <v>2058</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F17" s="15" t="n">
-        <v>817.6</v>
+        <v>2021.3</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>621.6</v>
+        <v>-146.8</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>0.1218</v>
+        <v>-0.0178</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>1.7</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2143,10 +1999,10 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>4120</v>
+        <v>1624.8</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
@@ -2154,7 +2010,7 @@
         </is>
       </c>
       <c r="F18" s="15" t="n">
-        <v>4639.8</v>
+        <v>1802</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -2165,19 +2021,19 @@
         <v>25</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>519.8</v>
+        <v>531.6</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>0.1262</v>
+        <v>0.1091</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>2.66</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2186,10 +2042,10 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>862</v>
+        <v>1588.9</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
@@ -2197,7 +2053,7 @@
         </is>
       </c>
       <c r="F19" s="15" t="n">
-        <v>849.25</v>
+        <v>1649</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -2208,19 +2064,19 @@
         <v>25</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>-76.5</v>
+        <v>180.3</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>-0.0148</v>
+        <v>0.0378</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>-0.33</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2229,104 +2085,104 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>1412.6</v>
+        <v>728.8</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="F20" s="15" t="n">
-        <v>1417.16</v>
+        <v>817.6</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>13.69</v>
+        <v>621.6</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>0.0032</v>
+        <v>0.1218</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>507</v>
+        <v>4120</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="F21" s="15" t="n">
-        <v>471.54</v>
+        <v>4639.8</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I21" s="17" t="n">
-        <v>-638.28</v>
+        <v>519.8</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>-0.0699</v>
+        <v>0.1262</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>-1</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>POLYCAB</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>8847</v>
+        <v>862</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="F22" s="15" t="n">
-        <v>9240</v>
+        <v>849.25</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -2337,19 +2193,19 @@
         <v>25</v>
       </c>
       <c r="I22" s="17" t="n">
-        <v>393</v>
+        <v>-76.5</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>0.0444</v>
+        <v>-0.0148</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>0.74</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2358,18 +2214,18 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1948.5</v>
+        <v>1412.6</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="F23" s="15" t="n">
-        <v>1922.5</v>
+        <v>1417.16</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -2377,128 +2233,128 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="I23" s="17" t="n">
-        <v>-52</v>
+        <v>13.69</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>-0.0133</v>
+        <v>0.0032</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>-0.36</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>4568</v>
+        <v>507</v>
       </c>
       <c r="D24" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>471.54</v>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="F24" s="15" t="n">
-        <v>4460</v>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>STOP_LOSS</t>
-        </is>
-      </c>
-      <c r="H24" s="14" t="n">
-        <v>10</v>
-      </c>
       <c r="I24" s="17" t="n">
-        <v>-108</v>
+        <v>-638.28</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>-0.0236</v>
+        <v>-0.0699</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>-0.49</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>POLYCAB</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>1550</v>
+        <v>8847</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="F25" s="15" t="n">
-        <v>1470.07</v>
+        <v>9240</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="I25" s="17" t="n">
-        <v>-239.79</v>
+        <v>393</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>-0.0516</v>
+        <v>0.0444</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>-0.77</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>1713.4</v>
+        <v>1948.5</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="F26" s="15" t="n">
-        <v>1650</v>
+        <v>1922.5</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -2506,42 +2362,42 @@
         </is>
       </c>
       <c r="H26" s="14" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="I26" s="17" t="n">
-        <v>-190.2</v>
+        <v>-52</v>
       </c>
       <c r="J26" s="18" t="n">
-        <v>-0.037</v>
+        <v>-0.0133</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>-0.65</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>2360</v>
+        <v>4568</v>
       </c>
       <c r="D27" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F27" s="15" t="n">
-        <v>2250.39</v>
+        <v>4460</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -2549,42 +2405,42 @@
         </is>
       </c>
       <c r="H27" s="14" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I27" s="17" t="n">
-        <v>-548.05</v>
+        <v>-108</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>-0.0464</v>
+        <v>-0.0236</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>-1</v>
+        <v>-0.49</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>8945</v>
+        <v>1550</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="F28" s="15" t="n">
-        <v>8673.639999999999</v>
+        <v>1470.07</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -2592,22 +2448,22 @@
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I28" s="17" t="n">
-        <v>-271.36</v>
+        <v>-239.79</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>-0.0303</v>
+        <v>-0.0516</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>-1</v>
+        <v>-0.77</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2616,18 +2472,18 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>2218</v>
+        <v>1713.4</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F29" s="15" t="n">
-        <v>2132.81</v>
+        <v>1650</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -2635,409 +2491,409 @@
         </is>
       </c>
       <c r="H29" s="14" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I29" s="17" t="n">
-        <v>-170.37</v>
+        <v>-190.2</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>-0.0384</v>
+        <v>-0.037</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>-0.76</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C30" s="15" t="n">
-        <v>1269</v>
+        <v>2360</v>
       </c>
       <c r="D30" s="16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F30" s="15" t="n">
-        <v>1365.2</v>
+        <v>2250.39</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H30" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I30" s="17" t="n">
-        <v>673.4</v>
+        <v>-548.05</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>0.07580000000000001</v>
+        <v>-0.0464</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>1.11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>7579.5</v>
+        <v>8945</v>
       </c>
       <c r="D31" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F31" s="15" t="n">
-        <v>7567.5</v>
+        <v>8673.639999999999</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I31" s="17" t="n">
-        <v>-12</v>
+        <v>-271.36</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>-0.0016</v>
+        <v>-0.0303</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>-0.03</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>1798.5</v>
+        <v>2218</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1747.8</v>
+        <v>2132.81</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I32" s="17" t="n">
-        <v>-253.5</v>
+        <v>-170.37</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>-0.0282</v>
+        <v>-0.0384</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>-0.43</v>
+        <v>-0.76</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>5438</v>
+        <v>1269</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F33" s="15" t="n">
-        <v>5381</v>
+        <v>1365.2</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H33" s="14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="I33" s="17" t="n">
-        <v>-57</v>
+        <v>673.4</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>-0.0105</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>-0.2</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>1784</v>
+        <v>7579.5</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F34" s="15" t="n">
-        <v>1752.1</v>
+        <v>7567.5</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I34" s="17" t="n">
-        <v>-63.8</v>
+        <v>-12</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>-0.0179</v>
+        <v>-0.0016</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>871.8</v>
+        <v>1798.5</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F35" s="15" t="n">
-        <v>830.15</v>
+        <v>1747.8</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I35" s="17" t="n">
-        <v>-249.9</v>
+        <v>-253.5</v>
       </c>
       <c r="J35" s="18" t="n">
-        <v>-0.0478</v>
+        <v>-0.0282</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>420.3</v>
+        <v>5438</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F36" s="15" t="n">
-        <v>448.6</v>
+        <v>5381</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="I36" s="17" t="n">
-        <v>622.6</v>
+        <v>-57</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>0.0673</v>
+        <v>-0.0105</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>0.84</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>1465</v>
+        <v>1784</v>
       </c>
       <c r="D37" s="16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F37" s="15" t="n">
-        <v>1596.9</v>
+        <v>1752.1</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H37" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I37" s="17" t="n">
-        <v>791.4</v>
+        <v>-63.8</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>0.09</v>
+        <v>-0.0179</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>1.32</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>619.25</v>
+        <v>871.8</v>
       </c>
       <c r="D38" s="16" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="F38" s="15" t="n">
-        <v>717.95</v>
+        <v>830.15</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H38" s="14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>1480.5</v>
+        <v>-249.9</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>0.1594</v>
+        <v>-0.0478</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>3.55</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
@@ -3046,10 +2902,10 @@
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>8700</v>
+        <v>420.3</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
@@ -3057,7 +2913,7 @@
         </is>
       </c>
       <c r="F39" s="15" t="n">
-        <v>8805.5</v>
+        <v>448.6</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -3068,31 +2924,31 @@
         <v>25</v>
       </c>
       <c r="I39" s="17" t="n">
-        <v>105.5</v>
+        <v>622.6</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>0.0121</v>
+        <v>0.0673</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>0.29</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C40" s="15" t="n">
-        <v>961.85</v>
+        <v>1465</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
@@ -3100,42 +2956,42 @@
         </is>
       </c>
       <c r="F40" s="15" t="n">
-        <v>935.6</v>
+        <v>1596.9</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H40" s="14" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I40" s="17" t="n">
-        <v>-236.25</v>
+        <v>791.4</v>
       </c>
       <c r="J40" s="18" t="n">
-        <v>-0.0273</v>
+        <v>0.09</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>-0.64</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>1560</v>
+        <v>619.25</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
@@ -3143,93 +2999,93 @@
         </is>
       </c>
       <c r="F41" s="15" t="n">
-        <v>1547.4</v>
+        <v>717.95</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H41" s="14" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I41" s="17" t="n">
-        <v>-63</v>
+        <v>1480.5</v>
       </c>
       <c r="J41" s="18" t="n">
-        <v>-0.0081</v>
+        <v>0.1594</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>-0.23</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>900</v>
+        <v>8700</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F42" s="15" t="n">
-        <v>887.1</v>
+        <v>8805.5</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H42" s="14" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I42" s="17" t="n">
-        <v>-129</v>
+        <v>105.5</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>-0.0143</v>
+        <v>0.0121</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>-0.2</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>FORTIS</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C43" s="15" t="n">
-        <v>880.8</v>
+        <v>961.85</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E43" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F43" s="15" t="n">
-        <v>832.9400000000001</v>
+        <v>935.6</v>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
@@ -3237,22 +3093,22 @@
         </is>
       </c>
       <c r="H43" s="14" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I43" s="17" t="n">
-        <v>-478.6</v>
+        <v>-236.25</v>
       </c>
       <c r="J43" s="18" t="n">
-        <v>-0.0543</v>
+        <v>-0.0273</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>-1</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -3261,18 +3117,18 @@
         </is>
       </c>
       <c r="C44" s="15" t="n">
-        <v>777</v>
+        <v>1560</v>
       </c>
       <c r="D44" s="16" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E44" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F44" s="15" t="n">
-        <v>744.8</v>
+        <v>1547.4</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
@@ -3280,42 +3136,42 @@
         </is>
       </c>
       <c r="H44" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I44" s="17" t="n">
-        <v>-386.4</v>
+        <v>-63</v>
       </c>
       <c r="J44" s="18" t="n">
-        <v>-0.0414</v>
+        <v>-0.0081</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>-1</v>
+        <v>-0.23</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>PREMIERENE</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C45" s="15" t="n">
-        <v>1114.9</v>
+        <v>900</v>
       </c>
       <c r="D45" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E45" s="14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="F45" s="15" t="n">
-        <v>1050.57</v>
+        <v>887.1</v>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
@@ -3323,16 +3179,16 @@
         </is>
       </c>
       <c r="H45" s="14" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="I45" s="17" t="n">
-        <v>-514.64</v>
+        <v>-129</v>
       </c>
       <c r="J45" s="18" t="n">
-        <v>-0.0577</v>
+        <v>-0.0143</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="46">
@@ -3343,131 +3199,131 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C46" s="15" t="n">
-        <v>790</v>
+        <v>880.8</v>
       </c>
       <c r="D46" s="16" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E46" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="F46" s="15" t="n">
-        <v>880.8</v>
+        <v>832.9400000000001</v>
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H46" s="14" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="I46" s="17" t="n">
-        <v>998.8</v>
+        <v>-478.6</v>
       </c>
       <c r="J46" s="18" t="n">
-        <v>0.1149</v>
+        <v>-0.0543</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>1.79</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C47" s="15" t="n">
-        <v>3770</v>
+        <v>777</v>
       </c>
       <c r="D47" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="F47" s="15" t="n">
+        <v>744.8</v>
+      </c>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H47" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="E47" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="F47" s="15" t="n">
-        <v>4097.9</v>
-      </c>
-      <c r="G47" s="14" t="inlineStr">
-        <is>
-          <t>TIME_STOP</t>
-        </is>
-      </c>
-      <c r="H47" s="14" t="n">
-        <v>25</v>
-      </c>
       <c r="I47" s="17" t="n">
-        <v>655.8</v>
+        <v>-386.4</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>0.08699999999999999</v>
+        <v>-0.0414</v>
       </c>
       <c r="K47" s="19" t="n">
-        <v>1.98</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>PREMIERENE</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="C48" s="15" t="n">
-        <v>821.05</v>
+        <v>1114.9</v>
       </c>
       <c r="D48" s="16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E48" s="14" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="F48" s="15" t="n">
-        <v>844</v>
+        <v>1050.57</v>
       </c>
       <c r="G48" s="14" t="inlineStr">
         <is>
-          <t>TIME_STOP</t>
+          <t>STOP_LOSS</t>
         </is>
       </c>
       <c r="H48" s="14" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I48" s="17" t="n">
-        <v>252.45</v>
+        <v>-514.64</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>0.028</v>
+        <v>-0.0577</v>
       </c>
       <c r="K48" s="19" t="n">
-        <v>0.6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
         <is>
-          <t>MANKIND</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
@@ -3476,10 +3332,10 @@
         </is>
       </c>
       <c r="C49" s="15" t="n">
-        <v>2426.1</v>
+        <v>790</v>
       </c>
       <c r="D49" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E49" s="14" t="inlineStr">
         <is>
@@ -3487,7 +3343,7 @@
         </is>
       </c>
       <c r="F49" s="15" t="n">
-        <v>2484.2</v>
+        <v>880.8</v>
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
@@ -3498,39 +3354,39 @@
         <v>25</v>
       </c>
       <c r="I49" s="17" t="n">
-        <v>174.3</v>
+        <v>998.8</v>
       </c>
       <c r="J49" s="18" t="n">
-        <v>0.0239</v>
+        <v>0.1149</v>
       </c>
       <c r="K49" s="19" t="n">
-        <v>0.5</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C50" s="15" t="n">
-        <v>1410</v>
+        <v>3770</v>
       </c>
       <c r="D50" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F50" s="15" t="n">
-        <v>1455.2</v>
+        <v>4097.9</v>
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
@@ -3541,39 +3397,39 @@
         <v>25</v>
       </c>
       <c r="I50" s="17" t="n">
-        <v>135.6</v>
+        <v>655.8</v>
       </c>
       <c r="J50" s="18" t="n">
-        <v>0.0321</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="K50" s="19" t="n">
-        <v>0.46</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>HSCL</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C51" s="15" t="n">
-        <v>690</v>
+        <v>821.05</v>
       </c>
       <c r="D51" s="16" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E51" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F51" s="15" t="n">
-        <v>660.45</v>
+        <v>844</v>
       </c>
       <c r="G51" s="14" t="inlineStr">
         <is>
@@ -3584,39 +3440,39 @@
         <v>25</v>
       </c>
       <c r="I51" s="17" t="n">
-        <v>-206.85</v>
+        <v>252.45</v>
       </c>
       <c r="J51" s="18" t="n">
-        <v>-0.0428</v>
+        <v>0.028</v>
       </c>
       <c r="K51" s="19" t="n">
-        <v>-0.38</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="14" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C52" s="15" t="n">
-        <v>1839</v>
+        <v>2426.1</v>
       </c>
       <c r="D52" s="16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E52" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="F52" s="15" t="n">
-        <v>1828.1</v>
+        <v>2484.2</v>
       </c>
       <c r="G52" s="14" t="inlineStr">
         <is>
@@ -3627,19 +3483,19 @@
         <v>25</v>
       </c>
       <c r="I52" s="17" t="n">
-        <v>-21.8</v>
+        <v>174.3</v>
       </c>
       <c r="J52" s="18" t="n">
-        <v>-0.0059</v>
+        <v>0.0239</v>
       </c>
       <c r="K52" s="19" t="n">
-        <v>-0.1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
@@ -3648,7 +3504,7 @@
         </is>
       </c>
       <c r="C53" s="15" t="n">
-        <v>1414</v>
+        <v>1410</v>
       </c>
       <c r="D53" s="16" t="n">
         <v>3</v>
@@ -3659,7 +3515,7 @@
         </is>
       </c>
       <c r="F53" s="15" t="n">
-        <v>1537.8</v>
+        <v>1455.2</v>
       </c>
       <c r="G53" s="14" t="inlineStr">
         <is>
@@ -3670,19 +3526,19 @@
         <v>25</v>
       </c>
       <c r="I53" s="17" t="n">
-        <v>371.4</v>
+        <v>135.6</v>
       </c>
       <c r="J53" s="18" t="n">
-        <v>0.0876</v>
+        <v>0.0321</v>
       </c>
       <c r="K53" s="19" t="n">
-        <v>1.38</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>HSCL</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
@@ -3691,10 +3547,10 @@
         </is>
       </c>
       <c r="C54" s="15" t="n">
-        <v>1300</v>
+        <v>690</v>
       </c>
       <c r="D54" s="16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E54" s="14" t="inlineStr">
         <is>
@@ -3702,7 +3558,7 @@
         </is>
       </c>
       <c r="F54" s="15" t="n">
-        <v>1389.1</v>
+        <v>660.45</v>
       </c>
       <c r="G54" s="14" t="inlineStr">
         <is>
@@ -3713,19 +3569,19 @@
         <v>25</v>
       </c>
       <c r="I54" s="17" t="n">
-        <v>356.4</v>
+        <v>-206.85</v>
       </c>
       <c r="J54" s="18" t="n">
-        <v>0.06850000000000001</v>
+        <v>-0.0428</v>
       </c>
       <c r="K54" s="19" t="n">
-        <v>0.63</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B55" s="14" t="inlineStr">
@@ -3734,10 +3590,10 @@
         </is>
       </c>
       <c r="C55" s="15" t="n">
-        <v>276.45</v>
+        <v>1839</v>
       </c>
       <c r="D55" s="16" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E55" s="14" t="inlineStr">
         <is>
@@ -3745,7 +3601,7 @@
         </is>
       </c>
       <c r="F55" s="15" t="n">
-        <v>330.1</v>
+        <v>1828.1</v>
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
@@ -3756,19 +3612,19 @@
         <v>25</v>
       </c>
       <c r="I55" s="17" t="n">
-        <v>1019.35</v>
+        <v>-21.8</v>
       </c>
       <c r="J55" s="18" t="n">
-        <v>0.1941</v>
+        <v>-0.0059</v>
       </c>
       <c r="K55" s="19" t="n">
-        <v>3.1</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
@@ -3777,7 +3633,7 @@
         </is>
       </c>
       <c r="C56" s="15" t="n">
-        <v>1462.5</v>
+        <v>1414</v>
       </c>
       <c r="D56" s="16" t="n">
         <v>3</v>
@@ -3788,7 +3644,7 @@
         </is>
       </c>
       <c r="F56" s="15" t="n">
-        <v>1564.7</v>
+        <v>1537.8</v>
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
@@ -3799,19 +3655,19 @@
         <v>25</v>
       </c>
       <c r="I56" s="17" t="n">
-        <v>306.6</v>
+        <v>371.4</v>
       </c>
       <c r="J56" s="18" t="n">
-        <v>0.0699</v>
+        <v>0.0876</v>
       </c>
       <c r="K56" s="19" t="n">
-        <v>1.78</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
@@ -3820,41 +3676,41 @@
         </is>
       </c>
       <c r="C57" s="15" t="n">
-        <v>798</v>
+        <v>1300</v>
       </c>
       <c r="D57" s="16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E57" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F57" s="15" t="n">
-        <v>750</v>
+        <v>1389.1</v>
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H57" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I57" s="17" t="n">
-        <v>-288</v>
+        <v>356.4</v>
       </c>
       <c r="J57" s="18" t="n">
-        <v>-0.0602</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="K57" s="19" t="n">
-        <v>-0.92</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>CROMPTON</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
@@ -3863,96 +3719,96 @@
         </is>
       </c>
       <c r="C58" s="15" t="n">
-        <v>260.45</v>
+        <v>276.45</v>
       </c>
       <c r="D58" s="16" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E58" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F58" s="15" t="n">
-        <v>257.85</v>
+        <v>330.1</v>
       </c>
       <c r="G58" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H58" s="14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I58" s="17" t="n">
-        <v>-52.07</v>
+        <v>1019.35</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>-0.01</v>
+        <v>0.1941</v>
       </c>
       <c r="K58" s="19" t="n">
-        <v>-0.13</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C59" s="15" t="n">
-        <v>6500</v>
+        <v>1462.5</v>
       </c>
       <c r="D59" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E59" s="14" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F59" s="15" t="n">
-        <v>6401.5</v>
+        <v>1564.7</v>
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>STOP_LOSS</t>
+          <t>TIME_STOP</t>
         </is>
       </c>
       <c r="H59" s="14" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I59" s="17" t="n">
-        <v>-98.5</v>
+        <v>306.6</v>
       </c>
       <c r="J59" s="18" t="n">
-        <v>-0.0152</v>
+        <v>0.0699</v>
       </c>
       <c r="K59" s="19" t="n">
-        <v>-0.31</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>ELGIEQUIP</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C60" s="15" t="n">
-        <v>571.5</v>
+        <v>798</v>
       </c>
       <c r="D60" s="16" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E60" s="14" t="inlineStr">
         <is>
@@ -3960,7 +3816,7 @@
         </is>
       </c>
       <c r="F60" s="15" t="n">
-        <v>571.1</v>
+        <v>750</v>
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
@@ -3968,34 +3824,34 @@
         </is>
       </c>
       <c r="H60" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I60" s="17" t="n">
-        <v>-6.4</v>
+        <v>-288</v>
       </c>
       <c r="J60" s="18" t="n">
-        <v>-0.0007</v>
+        <v>-0.0602</v>
       </c>
       <c r="K60" s="19" t="n">
-        <v>-0.01</v>
+        <v>-0.92</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>CROMPTON</t>
         </is>
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C61" s="15" t="n">
-        <v>965</v>
+        <v>260.45</v>
       </c>
       <c r="D61" s="16" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E61" s="14" t="inlineStr">
         <is>
@@ -4003,7 +3859,7 @@
         </is>
       </c>
       <c r="F61" s="15" t="n">
-        <v>933</v>
+        <v>257.85</v>
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
@@ -4011,42 +3867,42 @@
         </is>
       </c>
       <c r="H61" s="14" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I61" s="17" t="n">
-        <v>-288</v>
+        <v>-52.07</v>
       </c>
       <c r="J61" s="18" t="n">
-        <v>-0.0332</v>
+        <v>-0.01</v>
       </c>
       <c r="K61" s="19" t="n">
-        <v>-0.57</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C62" s="15" t="n">
-        <v>5479</v>
+        <v>6500</v>
       </c>
       <c r="D62" s="16" t="n">
         <v>1</v>
       </c>
       <c r="E62" s="14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F62" s="15" t="n">
-        <v>5424</v>
+        <v>6401.5</v>
       </c>
       <c r="G62" s="14" t="inlineStr">
         <is>
@@ -4054,42 +3910,42 @@
         </is>
       </c>
       <c r="H62" s="14" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="I62" s="17" t="n">
-        <v>-55</v>
+        <v>-98.5</v>
       </c>
       <c r="J62" s="18" t="n">
-        <v>-0.01</v>
+        <v>-0.0152</v>
       </c>
       <c r="K62" s="19" t="n">
-        <v>-0.18</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
         <is>
-          <t>CGPOWER</t>
+          <t>ELGIEQUIP</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C63" s="15" t="n">
-        <v>960.1</v>
+        <v>571.5</v>
       </c>
       <c r="D63" s="16" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E63" s="14" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F63" s="15" t="n">
-        <v>902.6799999999999</v>
+        <v>571.1</v>
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
@@ -4097,42 +3953,42 @@
         </is>
       </c>
       <c r="H63" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I63" s="17" t="n">
-        <v>-516.79</v>
+        <v>-6.4</v>
       </c>
       <c r="J63" s="18" t="n">
-        <v>-0.0598</v>
+        <v>-0.0007</v>
       </c>
       <c r="K63" s="19" t="n">
-        <v>-0.87</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C64" s="15" t="n">
-        <v>952.1</v>
+        <v>965</v>
       </c>
       <c r="D64" s="16" t="n">
         <v>9</v>
       </c>
       <c r="E64" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F64" s="15" t="n">
-        <v>948.8</v>
+        <v>933</v>
       </c>
       <c r="G64" s="14" t="inlineStr">
         <is>
@@ -4140,42 +3996,42 @@
         </is>
       </c>
       <c r="H64" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I64" s="17" t="n">
-        <v>-29.7</v>
+        <v>-288</v>
       </c>
       <c r="J64" s="18" t="n">
-        <v>-0.0035</v>
+        <v>-0.0332</v>
       </c>
       <c r="K64" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C65" s="15" t="n">
-        <v>1475</v>
+        <v>5479</v>
       </c>
       <c r="D65" s="16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E65" s="14" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F65" s="15" t="n">
-        <v>1394.19</v>
+        <v>5424</v>
       </c>
       <c r="G65" s="14" t="inlineStr">
         <is>
@@ -4183,42 +4039,42 @@
         </is>
       </c>
       <c r="H65" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I65" s="17" t="n">
-        <v>-484.86</v>
+        <v>-55</v>
       </c>
       <c r="J65" s="18" t="n">
-        <v>-0.0548</v>
+        <v>-0.01</v>
       </c>
       <c r="K65" s="19" t="n">
-        <v>-1</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>CGPOWER</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C66" s="15" t="n">
-        <v>248.05</v>
+        <v>960.1</v>
       </c>
       <c r="D66" s="16" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F66" s="15" t="n">
-        <v>242.8</v>
+        <v>902.6799999999999</v>
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
@@ -4226,16 +4082,16 @@
         </is>
       </c>
       <c r="H66" s="14" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I66" s="17" t="n">
-        <v>-110.25</v>
+        <v>-516.79</v>
       </c>
       <c r="J66" s="18" t="n">
-        <v>-0.0212</v>
+        <v>-0.0598</v>
       </c>
       <c r="K66" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="67">
@@ -4246,22 +4102,22 @@
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="C67" s="15" t="n">
-        <v>1039.2</v>
+        <v>952.1</v>
       </c>
       <c r="D67" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E67" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F67" s="15" t="n">
-        <v>970</v>
+        <v>948.8</v>
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
@@ -4269,42 +4125,42 @@
         </is>
       </c>
       <c r="H67" s="14" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I67" s="17" t="n">
-        <v>-346</v>
+        <v>-29.7</v>
       </c>
       <c r="J67" s="18" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0035</v>
       </c>
       <c r="K67" s="19" t="n">
-        <v>-0.82</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C68" s="15" t="n">
-        <v>199.96</v>
+        <v>1475</v>
       </c>
       <c r="D68" s="16" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E68" s="14" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F68" s="15" t="n">
-        <v>193.31</v>
+        <v>1394.19</v>
       </c>
       <c r="G68" s="14" t="inlineStr">
         <is>
@@ -4312,22 +4168,22 @@
         </is>
       </c>
       <c r="H68" s="14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="I68" s="17" t="n">
-        <v>-172.9</v>
+        <v>-484.86</v>
       </c>
       <c r="J68" s="18" t="n">
-        <v>-0.0333</v>
+        <v>-0.0548</v>
       </c>
       <c r="K68" s="19" t="n">
-        <v>-0.52</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B69" s="14" t="inlineStr">
@@ -4336,10 +4192,10 @@
         </is>
       </c>
       <c r="C69" s="15" t="n">
-        <v>986.4</v>
+        <v>248.05</v>
       </c>
       <c r="D69" s="16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E69" s="14" t="inlineStr">
         <is>
@@ -4347,7 +4203,7 @@
         </is>
       </c>
       <c r="F69" s="15" t="n">
-        <v>934.1900000000001</v>
+        <v>242.8</v>
       </c>
       <c r="G69" s="14" t="inlineStr">
         <is>
@@ -4358,17 +4214,146 @@
         <v>11</v>
       </c>
       <c r="I69" s="17" t="n">
+        <v>-110.25</v>
+      </c>
+      <c r="J69" s="18" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="K69" s="19" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="n">
+        <v>1039.2</v>
+      </c>
+      <c r="D70" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E70" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="n">
+        <v>970</v>
+      </c>
+      <c r="G70" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H70" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I70" s="17" t="n">
+        <v>-346</v>
+      </c>
+      <c r="J70" s="18" t="n">
+        <v>-0.06660000000000001</v>
+      </c>
+      <c r="K70" s="19" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="n">
+        <v>199.96</v>
+      </c>
+      <c r="D71" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="E71" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F71" s="15" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="G71" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H71" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I71" s="17" t="n">
+        <v>-172.9</v>
+      </c>
+      <c r="J71" s="18" t="n">
+        <v>-0.0333</v>
+      </c>
+      <c r="K71" s="19" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>SHYAMMETL</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="D72" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E72" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F72" s="15" t="n">
+        <v>934.1900000000001</v>
+      </c>
+      <c r="G72" s="14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="H72" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I72" s="17" t="n">
         <v>-261.05</v>
       </c>
-      <c r="J69" s="18" t="n">
+      <c r="J72" s="18" t="n">
         <v>-0.0529</v>
       </c>
-      <c r="K69" s="19" t="n">
+      <c r="K72" s="19" t="n">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I69">
+  <conditionalFormatting sqref="I2:I72">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -4386,7 +4371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5983,6 +5968,31 @@
       </c>
       <c r="G63" s="14" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B64" s="20" t="n">
+        <v>198669.34</v>
+      </c>
+      <c r="C64" s="20" t="n">
+        <v>118760.94</v>
+      </c>
+      <c r="D64" s="20" t="n">
+        <v>79908.39999999999</v>
+      </c>
+      <c r="E64" s="20" t="n">
+        <v>79886.10000000001</v>
+      </c>
+      <c r="F64" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G64" s="14" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -6065,7 +6075,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -6073,10 +6083,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>4360</v>
+        <v>4466</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>4168.96</v>
+        <v>4265.44</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6085,10 +6095,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.9</v>
+        <v>7.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8522804522752496</v>
+        <v>0.8762478037810106</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6103,7 +6113,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -6111,10 +6121,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>790</v>
+        <v>768</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>747.77</v>
+        <v>724.24</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6123,10 +6133,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8204737791342952</v>
+        <v>0.8680882352941177</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6141,18 +6151,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>872.6</v>
+        <v>9158</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>815.5</v>
+        <v>8706.860000000001</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6161,10 +6171,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8099125971143174</v>
+        <v>0.837395284278586</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6179,18 +6189,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>NEULANDLAB</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>22595</v>
+        <v>1219.9</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>21157.86</v>
+        <v>1132.11</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6199,10 +6209,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8055788706992231</v>
+        <v>0.8706869772998805</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6217,18 +6227,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>684</v>
+        <v>1895.7</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>632.9400000000001</v>
+        <v>1784.24</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6237,10 +6247,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7860831714761376</v>
+        <v>0.8402073230725982</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6255,18 +6265,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>11803</v>
+        <v>47555</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>11152.86</v>
+        <v>45128.57</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6275,10 +6285,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7834298695893452</v>
+        <v>0.8090990231217935</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6293,7 +6303,7 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -6301,10 +6311,10 @@
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>11424</v>
+        <v>11593</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>10945.86</v>
+        <v>11112.86</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6313,10 +6323,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7807072003329634</v>
+        <v>0.7979137676576007</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6331,18 +6341,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>EMCURE</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1993</v>
+        <v>1905.5</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1898.37</v>
+        <v>1794.34</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6351,10 +6361,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.8042712957824639</v>
+        <v>0.7863126361655773</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6369,18 +6379,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>NEULANDLAB</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>47070</v>
+        <v>22625</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>44728.57</v>
+        <v>21109.43</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6389,10 +6399,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7781284683684796</v>
+        <v>0.8031061564410711</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6407,18 +6417,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>9198</v>
+        <v>11510</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>8737.290000000001</v>
+        <v>10848.86</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6427,10 +6437,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7697957130965594</v>
+        <v>0.7861515215405159</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6445,18 +6455,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1906.4</v>
+        <v>835.6</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1810.24</v>
+        <v>776.54</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6465,10 +6475,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7734652469478357</v>
+        <v>0.7861487103802095</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6483,18 +6493,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2311.7</v>
+        <v>1706.9</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2160.41</v>
+        <v>1614.63</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -6503,10 +6513,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7675447419533852</v>
+        <v>0.7683008292922904</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6521,18 +6531,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>CORONA</t>
+          <t>BLSE</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>2217.9</v>
+        <v>313.55</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>2075.47</v>
+        <v>291.36</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -6541,10 +6551,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7727004716981132</v>
+        <v>0.7924555485276547</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6559,18 +6569,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>INNOVACAP</t>
+          <t>HAPPYFORGE</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1140.1</v>
+        <v>2155.9</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1038.86</v>
+        <v>1941.19</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -6579,10 +6589,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7650874028856826</v>
+        <v>0.7768478108089114</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -6597,7 +6607,7 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260915</v>
+        <v>20260916</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
@@ -6605,10 +6615,10 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>480.05</v>
+        <v>488.15</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>450.86</v>
+        <v>456.11</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -6617,10 +6627,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7797395255271921</v>
+        <v>0.7775560475086091</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-17
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 16 Sep 2026</t>
+          <t>As of Thu 17 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹198,669</t>
+          <t>₹199,561</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-987  (-0.49%)</t>
+          <t>₹+892  (+0.45%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-0.67%</t>
+          <t>-0.22%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-3.60%</t>
+          <t>-3.17%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹79,908</t>
+          <t>₹80,800</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8696.5</v>
+        <v>8768.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8696.5</v>
+        <v>8768.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-221</v>
+        <v>-149</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.02478273058592655</v>
+        <v>-0.01670871881132605</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.01832461335019842</v>
+        <v>0.02638535667445978</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1950.7</v>
+        <v>1970.3</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9753.5</v>
+        <v>9851.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>723.9999999999998</v>
+        <v>821.9999999999993</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.08018162688963948</v>
+        <v>0.09103494102663484</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1605.14</v>
@@ -910,13 +910,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.0673384645804804</v>
+        <v>0.07661632383755927</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>9158</v>
+        <v>9323</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9158</v>
+        <v>9323</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-81</v>
+        <v>84</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.008767182595518995</v>
+        <v>0.009091893062019699</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8902.93</v>
@@ -958,13 +958,13 @@
         <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.02785215112469968</v>
+        <v>0.0450573849619221</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>713.4</v>
+        <v>726.65</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9274.199999999999</v>
+        <v>9446.449999999999</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>148.1999999999997</v>
+        <v>320.4499999999997</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.01623931623931621</v>
+        <v>0.03511396011396008</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>683.88</v>
@@ -1006,13 +1006,13 @@
         <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.01661059714045419</v>
+        <v>0.03454207665313428</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>690.2</v>
+        <v>691</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>8972.6</v>
+        <v>8983</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>2.600000000000591</v>
+        <v>13</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.000289855072463834</v>
+        <v>0.001449275362318841</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>627</v>
@@ -1054,13 +1054,13 @@
         <v>627</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.09156766154737764</v>
+        <v>0.09261939218523878</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>835.6</v>
+        <v>870.4</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9191.6</v>
+        <v>9574.4</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-97.89999999999975</v>
+        <v>284.8999999999997</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.01053878034339843</v>
+        <v>0.03066903493191235</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>801.9400000000001</v>
@@ -1102,13 +1102,13 @@
         <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.0363810435615128</v>
+        <v>0.07490808823529417</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1404.6</v>
+        <v>1424</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8427.599999999999</v>
+        <v>8544</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-417</v>
+        <v>-300.5999999999995</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.0471474119801913</v>
+        <v>-0.03398683942744719</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1378.14</v>
@@ -1150,13 +1150,13 @@
         <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.01883810337462609</v>
+        <v>0.03220505617977521</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2297.2</v>
+        <v>2266</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9188.799999999999</v>
+        <v>9064</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-35.60000000000036</v>
+        <v>-160.3999999999996</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.003859329604093531</v>
+        <v>-0.01738866484540996</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>2152.33</v>
@@ -1198,13 +1198,13 @@
         <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.06306372975796617</v>
+        <v>0.05016328331862316</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -4371,7 +4371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5992,6 +5992,31 @@
         <v>-1275.21</v>
       </c>
       <c r="G64" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B65" s="20" t="n">
+        <v>199561.39</v>
+      </c>
+      <c r="C65" s="20" t="n">
+        <v>118760.94</v>
+      </c>
+      <c r="D65" s="20" t="n">
+        <v>80800.45</v>
+      </c>
+      <c r="E65" s="20" t="n">
+        <v>79886.10000000001</v>
+      </c>
+      <c r="F65" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G65" s="14" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6075,18 +6100,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>4466</v>
+        <v>777.9</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>4265.44</v>
+        <v>732.97</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6098,7 +6123,7 @@
         <v>7.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8762478037810106</v>
+        <v>0.8687545740238495</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6113,18 +6138,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>768</v>
+        <v>9323</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>724.24</v>
+        <v>8856.07</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6133,10 +6158,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8680882352941177</v>
+        <v>0.8136618020577726</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6151,18 +6176,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>9158</v>
+        <v>1924.7</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>8706.860000000001</v>
+        <v>1811.4</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6171,10 +6196,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.837395284278586</v>
+        <v>0.8306954668733049</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6189,18 +6214,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1219.9</v>
+        <v>4380</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1132.11</v>
+        <v>4177.51</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6209,10 +6234,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8706869772998805</v>
+        <v>0.8253551594989023</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6227,18 +6252,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>ENDURANCE</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1895.7</v>
+        <v>2690.8</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1784.24</v>
+        <v>2535.07</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6247,10 +6272,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8402073230725982</v>
+        <v>0.7796321408584098</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6265,18 +6290,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>47555</v>
+        <v>1948.1</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>45128.57</v>
+        <v>1834.36</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6285,10 +6310,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.8090990231217935</v>
+        <v>0.7471996211632012</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6303,18 +6328,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>11593</v>
+        <v>47735</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>11112.86</v>
+        <v>45291.43</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6323,10 +6348,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.8</v>
+        <v>6.4</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7979137676576007</v>
+        <v>0.7565682982478797</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6341,18 +6366,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>ACE</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1905.5</v>
+        <v>1205.6</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1794.34</v>
+        <v>1117.24</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6361,10 +6386,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.8</v>
+        <v>6.4</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7863126361655773</v>
+        <v>0.7537324034611907</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6379,18 +6404,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>NEULANDLAB</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>22625</v>
+        <v>1970.3</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>21109.43</v>
+        <v>1872.96</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6399,10 +6424,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.7</v>
+        <v>6.3</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.8031061564410711</v>
+        <v>0.7332827500107625</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6417,18 +6442,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>11510</v>
+        <v>323.75</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>10848.86</v>
+        <v>306.76</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6437,10 +6462,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.7</v>
+        <v>6.3</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7861515215405159</v>
+        <v>0.7311905376899565</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6455,18 +6480,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>APLLTD</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>835.6</v>
+        <v>826</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>776.54</v>
+        <v>773.3200000000001</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6475,10 +6500,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.7</v>
+        <v>6.2</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7861487103802095</v>
+        <v>0.7363790950966466</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6493,18 +6518,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1706.9</v>
+        <v>691</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1614.63</v>
+        <v>637.91</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -6513,10 +6538,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7683008292922904</v>
+        <v>0.7318879417968918</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6531,18 +6556,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>BLSE</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>313.55</v>
+        <v>435.2</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>291.36</v>
+        <v>402.45</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -6551,10 +6576,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7924555485276547</v>
+        <v>0.7405592147746352</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6569,18 +6594,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>HAPPYFORGE</t>
+          <t>SIS</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>2155.9</v>
+        <v>419.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1941.19</v>
+        <v>397.76</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -6589,10 +6614,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7768478108089114</v>
+        <v>0.7287743768565156</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -6607,18 +6632,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260916</v>
+        <v>20260917</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>HNDFDS</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>488.15</v>
+        <v>620.35</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>456.11</v>
+        <v>579.08</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -6627,10 +6652,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7775560475086091</v>
+        <v>0.7287237935339447</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-18
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 17 Sep 2026</t>
+          <t>As of Fri 18 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹199,561</t>
+          <t>₹201,423</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+892  (+0.45%)</t>
+          <t>₹+1,861  (+0.93%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-0.22%</t>
+          <t>+0.71%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-3.17%</t>
+          <t>-2.27%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹80,800</t>
+          <t>₹82,662</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8768.5</v>
+        <v>8944.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8768.5</v>
+        <v>8944.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-149</v>
+        <v>27</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.01670871881132605</v>
+        <v>0.003027754415475189</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.02638535667445978</v>
+        <v>0.04554307116104876</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1970.3</v>
+        <v>2009.6</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9851.5</v>
+        <v>10048</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>821.9999999999993</v>
+        <v>1018.499999999999</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.09103494102663484</v>
+        <v>0.112796943352345</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1605.14</v>
@@ -910,13 +910,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.07661632383755927</v>
+        <v>0.09467413557779807</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>9323</v>
+        <v>9375</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9323</v>
+        <v>9375</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>84</v>
+        <v>136</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.009091893062019699</v>
+        <v>0.01472020781469856</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8902.93</v>
@@ -958,13 +958,13 @@
         <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.0450573849619221</v>
+        <v>0.0503541333333333</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>726.65</v>
+        <v>732.75</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9446.449999999999</v>
+        <v>9525.75</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>320.4499999999997</v>
+        <v>399.75</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.03511396011396008</v>
+        <v>0.0438034188034188</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>683.88</v>
@@ -1006,13 +1006,13 @@
         <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.03454207665313428</v>
+        <v>0.0425793244626408</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>691</v>
+        <v>708.05</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>8983</v>
+        <v>9204.65</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>13</v>
+        <v>234.6499999999994</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.001449275362318841</v>
+        <v>0.02615942028985501</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>627</v>
@@ -1054,13 +1054,13 @@
         <v>627</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.09261939218523878</v>
+        <v>0.1144693171386201</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>870.4</v>
+        <v>875.5</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9574.4</v>
+        <v>9630.5</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>284.8999999999997</v>
+        <v>341</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.03066903493191235</v>
+        <v>0.03670811130846655</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>801.9400000000001</v>
@@ -1102,13 +1102,13 @@
         <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07490808823529417</v>
+        <v>0.08029697315819539</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1424</v>
+        <v>1499.4</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8544</v>
+        <v>8996.400000000001</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-300.5999999999995</v>
+        <v>151.8000000000011</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.03398683942744719</v>
+        <v>0.01716301472084674</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1378.14</v>
@@ -1150,13 +1150,13 @@
         <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.03220505617977521</v>
+        <v>0.08087234893957582</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2266</v>
+        <v>2422.8</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9064</v>
+        <v>9691.200000000001</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-160.3999999999996</v>
+        <v>466.8000000000011</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.01738866484540996</v>
+        <v>0.05060491739300129</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>2152.33</v>
@@ -1198,13 +1198,13 @@
         <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.05016328331862316</v>
+        <v>0.1116352980023115</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -4371,7 +4371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6017,6 +6017,31 @@
         <v>-1275.21</v>
       </c>
       <c r="G65" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B66" s="20" t="n">
+        <v>201422.54</v>
+      </c>
+      <c r="C66" s="20" t="n">
+        <v>118760.94</v>
+      </c>
+      <c r="D66" s="20" t="n">
+        <v>82661.60000000001</v>
+      </c>
+      <c r="E66" s="20" t="n">
+        <v>79886.10000000001</v>
+      </c>
+      <c r="F66" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G66" s="14" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6100,18 +6125,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>777.9</v>
+        <v>4535.4</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>732.97</v>
+        <v>4316.53</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6123,7 +6148,7 @@
         <v>7.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8687545740238495</v>
+        <v>0.8701640578179847</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6138,18 +6163,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>9323</v>
+        <v>808</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8856.07</v>
+        <v>761.28</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6158,10 +6183,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.9</v>
+        <v>7.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8136618020577726</v>
+        <v>0.8621311463713935</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6176,18 +6201,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>NEULANDLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1924.7</v>
+        <v>22840</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1811.4</v>
+        <v>21340.29</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6199,7 +6224,7 @@
         <v>6.8</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8306954668733049</v>
+        <v>0.8099597614223337</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6214,18 +6239,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>4380</v>
+        <v>9375</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>4177.51</v>
+        <v>8920.639999999999</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6234,10 +6259,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8253551594989023</v>
+        <v>0.7979563225935332</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6252,18 +6277,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>ENDURANCE</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>2690.8</v>
+        <v>1896.9</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>2535.07</v>
+        <v>1777.36</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6272,10 +6297,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7796321408584098</v>
+        <v>0.8134993650295368</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6290,18 +6315,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1948.1</v>
+        <v>2422.8</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1834.36</v>
+        <v>2249.03</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6310,10 +6335,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7471996211632012</v>
+        <v>0.783844104049542</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6328,7 +6353,7 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -6336,10 +6361,10 @@
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>47735</v>
+        <v>47000</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>45291.43</v>
+        <v>44450.71</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6348,10 +6373,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7565682982478797</v>
+        <v>0.7776752589823349</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6366,18 +6391,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>ACE</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1205.6</v>
+        <v>1372.4</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1117.24</v>
+        <v>1305.76</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6386,10 +6411,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7537324034611907</v>
+        <v>0.7632148768585372</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6404,18 +6429,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1970.3</v>
+        <v>162.57</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1872.96</v>
+        <v>153.62</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6424,10 +6449,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7332827500107625</v>
+        <v>0.7717884050112724</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6442,18 +6467,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>323.75</v>
+        <v>1954</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>306.76</v>
+        <v>1839.47</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6462,10 +6487,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7311905376899565</v>
+        <v>0.763551446876516</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6480,18 +6505,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>APLLTD</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>826</v>
+        <v>1228.2</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>773.3200000000001</v>
+        <v>1142.04</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6500,10 +6525,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7363790950966466</v>
+        <v>0.7895575896806598</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6518,18 +6543,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>691</v>
+        <v>11414</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>637.91</v>
+        <v>10957.57</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -6538,10 +6563,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7318879417968918</v>
+        <v>0.7563803829799378</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6556,18 +6581,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>435.2</v>
+        <v>1499.4</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>402.45</v>
+        <v>1397.24</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -6576,10 +6601,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7405592147746352</v>
+        <v>0.77688689677806</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6594,18 +6619,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SIS</t>
+          <t>SHINDL</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>419.8</v>
+        <v>161.64</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>397.76</v>
+        <v>151.36</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -6614,10 +6639,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7287743768565156</v>
+        <v>0.7751865671641791</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -6632,18 +6657,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260917</v>
+        <v>20260918</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>HNDFDS</t>
+          <t>SUPRAJIT</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>620.35</v>
+        <v>499.05</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>579.08</v>
+        <v>465.18</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -6652,10 +6677,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7287237935339447</v>
+        <v>0.7492201991952284</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-21
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 18 Sep 2026</t>
+          <t>As of Mon 21 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹201,423</t>
+          <t>₹201,447</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,861  (+0.93%)</t>
+          <t>₹+24  (+0.01%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.71%</t>
+          <t>+0.72%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-2.27%</t>
+          <t>-2.26%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹118,761</t>
+          <t>₹67,880</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹79,886</t>
+          <t>₹130,658</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹82,662</t>
+          <t>₹133,566</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8944.5</v>
+        <v>8912</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8944.5</v>
+        <v>8912</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>27</v>
+        <v>-5.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.003027754415475189</v>
+        <v>-0.0006167647883375386</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.04554307116104876</v>
+        <v>0.04206238779174154</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>2009.6</v>
+        <v>2008.2</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10048</v>
+        <v>10041</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>1018.499999999999</v>
+        <v>1011.5</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.112796943352345</v>
+        <v>0.112021706628274</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1605.14</v>
@@ -910,13 +910,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.09467413557779807</v>
+        <v>0.09404299514846286</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>9375</v>
+        <v>9410.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9375</v>
+        <v>9410.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>136</v>
+        <v>171.5</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01472020781469856</v>
+        <v>0.01856261500162355</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8902.93</v>
@@ -958,13 +958,13 @@
         <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.0503541333333333</v>
+        <v>0.05393656022528024</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>732.75</v>
+        <v>745</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9525.75</v>
+        <v>9685</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>399.75</v>
+        <v>559</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.0438034188034188</v>
+        <v>0.06125356125356125</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>683.88</v>
@@ -1006,13 +1006,13 @@
         <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.0425793244626408</v>
+        <v>0.05832214765100677</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>708.05</v>
+        <v>709.5</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9204.65</v>
+        <v>9223.5</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>234.6499999999994</v>
+        <v>253.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.02615942028985501</v>
+        <v>0.02826086956521739</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>627</v>
@@ -1054,13 +1054,13 @@
         <v>627</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1144693171386201</v>
+        <v>0.1162790697674419</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>875.5</v>
+        <v>875.15</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9630.5</v>
+        <v>9626.65</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>341</v>
+        <v>337.1499999999997</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.03670811130846655</v>
+        <v>0.0362936648904677</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>801.9400000000001</v>
@@ -1102,13 +1102,13 @@
         <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.08029697315819539</v>
+        <v>0.07992915500199971</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1499.4</v>
+        <v>1508.1</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8996.400000000001</v>
+        <v>9048.599999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>151.8000000000011</v>
+        <v>204</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.01716301472084674</v>
+        <v>0.02306492096872668</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1378.14</v>
@@ -1150,13 +1150,13 @@
         <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08087234893957582</v>
+        <v>0.08617465685299371</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2422.8</v>
+        <v>2329.6</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9691.200000000001</v>
+        <v>9318.4</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>466.8000000000011</v>
+        <v>94</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.05060491739300129</v>
+        <v>0.01019036468496596</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>2152.33</v>
@@ -1198,17 +1198,305 @@
         <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1116352980023115</v>
+        <v>0.07609460851648352</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>RADICO</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>4475</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>8950</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>4480</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>8960</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>0.00111731843575419</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>4316.53</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>4316.53</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.03648883928571434</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>111.57</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>810</v>
+      </c>
+      <c r="D12" s="8" t="n">
         <v>11</v>
       </c>
+      <c r="E12" s="9" t="n">
+        <v>8910</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>795.25</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>8747.75</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>-162.25</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>-0.01820987654320988</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>761.28</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>761.28</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0.0427161270040868</v>
+      </c>
+      <c r="M12" s="13" t="n">
+        <v>23.57</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>LALPATHLAB</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1896.9</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>7587.6</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1920.4</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>7681.6</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>94</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0.0123886340871949</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>1777.36</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>1777.36</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.0744844823995002</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>56.89</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>8160</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1385</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>8310</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>0.01838235294117647</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>1305.76</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>1305.76</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.0572129963898917</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>30.54</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>163.12</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>57</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>9297.84</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>162.91</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>9285.869999999999</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>-11.97000000000045</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>-0.001287395782246248</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>153.62</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>153.62</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.05702535142102997</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1966.6</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>7866.4</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>2017.5</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>8070</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>203.6000000000004</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0.02588223329604398</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>1839.47</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>1839.47</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.08824287484510532</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>55</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H10">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -4371,7 +4659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6043,6 +6331,31 @@
       </c>
       <c r="G66" s="14" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B67" s="20" t="n">
+        <v>201446.9</v>
+      </c>
+      <c r="C67" s="20" t="n">
+        <v>67880.42999999999</v>
+      </c>
+      <c r="D67" s="20" t="n">
+        <v>133566.47</v>
+      </c>
+      <c r="E67" s="20" t="n">
+        <v>130657.94</v>
+      </c>
+      <c r="F67" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G67" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -6125,7 +6438,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -6133,10 +6446,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>4535.4</v>
+        <v>4480</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>4316.53</v>
+        <v>4256.86</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6145,10 +6458,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8701640578179847</v>
+        <v>0.9000161436135864</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6163,7 +6476,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -6171,10 +6484,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>808</v>
+        <v>795.25</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>761.28</v>
+        <v>748.11</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6183,10 +6496,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8621311463713935</v>
+        <v>0.8411759008136381</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6201,7 +6514,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
@@ -6209,10 +6522,10 @@
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>22840</v>
+        <v>22610</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>21340.29</v>
+        <v>21105</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6221,10 +6534,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8099597614223337</v>
+        <v>0.8039659477377417</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6239,7 +6552,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
@@ -6247,10 +6560,10 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>9375</v>
+        <v>9410.5</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>8920.639999999999</v>
+        <v>8990.5</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6259,10 +6572,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7979563225935332</v>
+        <v>0.778293297171639</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6277,18 +6590,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1896.9</v>
+        <v>10911</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1777.36</v>
+        <v>10162.57</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6300,7 +6613,7 @@
         <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8134993650295368</v>
+        <v>0.7784407421757286</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6315,18 +6628,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>2422.8</v>
+        <v>2017.5</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>2249.03</v>
+        <v>1907.5</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6335,10 +6648,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.783844104049542</v>
+        <v>0.7657206509104998</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6353,18 +6666,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>AKUMS</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>47000</v>
+        <v>821.45</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>44450.71</v>
+        <v>762.79</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6373,10 +6686,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7776752589823349</v>
+        <v>0.7788023591200655</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6391,18 +6704,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1372.4</v>
+        <v>4826</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1305.76</v>
+        <v>4590.23</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6411,10 +6724,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7632148768585372</v>
+        <v>0.7466733393602825</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6429,18 +6742,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>UNITDSPR</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>162.57</v>
+        <v>1397</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>153.62</v>
+        <v>1335.01</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6449,10 +6762,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7717884050112724</v>
+        <v>0.7665482801670327</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6467,18 +6780,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SHINDL</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1954</v>
+        <v>163</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1839.47</v>
+        <v>152.56</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6487,10 +6800,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.763551446876516</v>
+        <v>0.7925093632958801</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6505,18 +6818,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1228.2</v>
+        <v>1920.4</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1142.04</v>
+        <v>1806.61</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6525,10 +6838,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7895575896806598</v>
+        <v>0.7555695466873305</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6543,18 +6856,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>11414</v>
+        <v>2329.6</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>10957.57</v>
+        <v>2150.99</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -6563,10 +6876,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7563803829799378</v>
+        <v>0.7467874208962935</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6581,18 +6894,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1499.4</v>
+        <v>47565</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1397.24</v>
+        <v>45081.43</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -6601,10 +6914,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.77688689677806</v>
+        <v>0.7490378406302466</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6619,18 +6932,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SHINDL</t>
+          <t>INNOVACAP</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>161.64</v>
+        <v>1198.3</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>151.36</v>
+        <v>1090.71</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -6642,7 +6955,7 @@
         <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7751865671641791</v>
+        <v>0.7611778380472685</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -6657,18 +6970,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260918</v>
+        <v>20260921</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>BLSE</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>499.05</v>
+        <v>317.25</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>465.18</v>
+        <v>297.99</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -6680,7 +6993,7 @@
         <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7492201991952284</v>
+        <v>0.7533567953850789</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-22
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 21 Sep 2026</t>
+          <t>As of Tue 22 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹201,447</t>
+          <t>₹200,739</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+24  (+0.01%)</t>
+          <t>₹-708  (-0.35%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.72%</t>
+          <t>+0.37%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-2.26%</t>
+          <t>-2.60%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹133,566</t>
+          <t>₹132,859</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8912</v>
+        <v>8835.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8912</v>
+        <v>8835.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-5.5</v>
+        <v>-82</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.0006167647883375386</v>
+        <v>-0.009195402298850575</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.04206238779174154</v>
+        <v>0.03376832097787342</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>2008.2</v>
+        <v>1992.4</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10041</v>
+        <v>9962</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>1011.5</v>
+        <v>932.5</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.112021706628274</v>
+        <v>0.1032726064566144</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1605.14</v>
@@ -910,13 +910,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.09404299514846286</v>
+        <v>0.08685863423867855</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>9410.5</v>
+        <v>9352</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9410.5</v>
+        <v>9352</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>171.5</v>
+        <v>113</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01856261500162355</v>
+        <v>0.01223076090485983</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8902.93</v>
@@ -958,13 +958,13 @@
         <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.05393656022528024</v>
+        <v>0.04801860564585112</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>745</v>
+        <v>736.25</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9685</v>
+        <v>9571.25</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>559</v>
+        <v>445.25</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.06125356125356125</v>
+        <v>0.04878917378917379</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>683.88</v>
@@ -1006,13 +1006,13 @@
         <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.05832214765100677</v>
+        <v>0.04713073005093385</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>709.5</v>
+        <v>719.35</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9223.5</v>
+        <v>9351.550000000001</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>253.5</v>
+        <v>381.5500000000003</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.02826086956521739</v>
+        <v>0.042536231884058</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>627</v>
@@ -1054,13 +1054,13 @@
         <v>627</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1162790697674419</v>
+        <v>0.1283797873079864</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>875.15</v>
+        <v>864.05</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9626.65</v>
+        <v>9504.549999999999</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>337.1499999999997</v>
+        <v>215.0499999999995</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.0362936648904677</v>
+        <v>0.02314979277679095</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>801.9400000000001</v>
@@ -1102,13 +1102,13 @@
         <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07992915500199971</v>
+        <v>0.06810948440483772</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1508.1</v>
+        <v>1487.8</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>9048.599999999999</v>
+        <v>8926.799999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>204</v>
+        <v>82.20000000000027</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.02306492096872668</v>
+        <v>0.009293806390339899</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1378.14</v>
@@ -1150,13 +1150,13 @@
         <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08617465685299371</v>
+        <v>0.07370614329883039</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2329.6</v>
+        <v>2310.8</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9318.4</v>
+        <v>9243.200000000001</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>94</v>
+        <v>18.80000000000109</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.01019036468496596</v>
+        <v>0.00203807293699331</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>2152.33</v>
@@ -1198,13 +1198,13 @@
         <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07609460851648352</v>
+        <v>0.06857798165137625</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8950</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4480</v>
+        <v>4448.8</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8960</v>
+        <v>8897.6</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>10</v>
+        <v>-52.39999999999964</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.00111731843575419</v>
+        <v>-0.005854748603351914</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>4316.53</v>
@@ -1246,13 +1246,13 @@
         <v>4316.53</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.03648883928571434</v>
+        <v>0.02973161301924124</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>111.57</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>8910</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>795.25</v>
+        <v>809</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8747.75</v>
+        <v>8899</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-162.25</v>
+        <v>-11</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.01820987654320988</v>
+        <v>-0.001234567901234568</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>761.28</v>
@@ -1294,13 +1294,13 @@
         <v>761.28</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.0427161270040868</v>
+        <v>0.0589864029666255</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>7587.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1920.4</v>
+        <v>1909.8</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>7681.6</v>
+        <v>7639.2</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>94</v>
+        <v>51.59999999999945</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.0123886340871949</v>
+        <v>0.00680056934999202</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1777.36</v>
@@ -1342,13 +1342,13 @@
         <v>1777.36</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.0744844823995002</v>
+        <v>0.06934757566237305</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>8160</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1385</v>
+        <v>1363.9</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8310</v>
+        <v>8183.400000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>150</v>
+        <v>23.40000000000055</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.01838235294117647</v>
+        <v>0.002867647058823596</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1305.76</v>
@@ -1390,13 +1390,13 @@
         <v>1305.76</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.0572129963898917</v>
+        <v>0.04262775863333096</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>30.54</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>9297.84</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>162.91</v>
+        <v>161.77</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>9285.869999999999</v>
+        <v>9220.890000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-11.97000000000045</v>
+        <v>-76.94999999999968</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.001287395782246248</v>
+        <v>-0.008276115743011245</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>153.62</v>
@@ -1438,13 +1438,13 @@
         <v>153.62</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05702535142102997</v>
+        <v>0.05038016937627499</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>4.22</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>7866.4</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2017.5</v>
+        <v>2006.5</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8070</v>
+        <v>8026</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>203.6000000000004</v>
+        <v>159.6000000000004</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.02588223329604398</v>
+        <v>0.02028882334994411</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1839.47</v>
@@ -1486,13 +1486,13 @@
         <v>1839.47</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.08824287484510532</v>
+        <v>0.08324445551956142</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4659,7 +4659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6355,6 +6355,31 @@
         <v>-1275.21</v>
       </c>
       <c r="G67" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B68" s="20" t="n">
+        <v>200738.97</v>
+      </c>
+      <c r="C68" s="20" t="n">
+        <v>67880.42999999999</v>
+      </c>
+      <c r="D68" s="20" t="n">
+        <v>132858.54</v>
+      </c>
+      <c r="E68" s="20" t="n">
+        <v>130657.94</v>
+      </c>
+      <c r="F68" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G68" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6438,18 +6463,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>BLSE</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>4480</v>
+        <v>328.1</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>4256.86</v>
+        <v>306.83</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6458,10 +6483,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.9000161436135864</v>
+        <v>0.8437000280053211</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6476,7 +6501,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -6484,10 +6509,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>795.25</v>
+        <v>809</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>748.11</v>
+        <v>763.01</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6496,10 +6521,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8411759008136381</v>
+        <v>0.8060120422880347</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6514,18 +6539,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>NEULANDLAB</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>22610</v>
+        <v>4448.8</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>21105</v>
+        <v>4235.7</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6534,10 +6559,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8039659477377417</v>
+        <v>0.8032319890779248</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6552,18 +6577,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>CUPID</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>9410.5</v>
+        <v>258.2</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>8990.5</v>
+        <v>234.3</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6572,10 +6597,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.778293297171639</v>
+        <v>0.7423148148148149</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6590,18 +6615,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>10911</v>
+        <v>1909.8</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>10162.57</v>
+        <v>1799.47</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6610,10 +6635,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7784407421757286</v>
+        <v>0.7799077574739202</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6628,18 +6653,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>DIXON</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>2017.5</v>
+        <v>13084</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1907.5</v>
+        <v>12280.57</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6648,10 +6673,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7657206509104998</v>
+        <v>0.7436655464538263</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6666,18 +6691,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>AKUMS</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>821.45</v>
+        <v>1190.9</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>762.79</v>
+        <v>1101.36</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6686,10 +6711,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7788023591200655</v>
+        <v>0.7896121263039977</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6704,18 +6729,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>4826</v>
+        <v>9352</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>4590.23</v>
+        <v>8967.93</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6724,10 +6749,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7466733393602825</v>
+        <v>0.7334863123993558</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6742,18 +6767,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>UNITDSPR</t>
+          <t>VARROC</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1397</v>
+        <v>864.5</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1335.01</v>
+        <v>786.12</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6762,10 +6787,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7665482801670327</v>
+        <v>0.7604949940488692</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6780,18 +6805,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SHINDL</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>163</v>
+        <v>48290</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>152.56</v>
+        <v>46011.43</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6800,10 +6825,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7925093632958801</v>
+        <v>0.7563053980256249</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6818,18 +6843,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1920.4</v>
+        <v>11363</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1806.61</v>
+        <v>10946.57</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6838,10 +6863,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7555695466873305</v>
+        <v>0.7392494573969054</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6856,18 +6881,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>SHINDL</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2329.6</v>
+        <v>162.53</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2150.99</v>
+        <v>151.82</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -6876,10 +6901,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7467874208962935</v>
+        <v>0.7733333333333332</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6894,18 +6919,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>STYLAMIND</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>47565</v>
+        <v>3309.4</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>45081.43</v>
+        <v>3061.3</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -6914,10 +6939,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7490378406302466</v>
+        <v>0.7386238885388223</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6932,18 +6957,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>INNOVACAP</t>
+          <t>TIIL</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1198.3</v>
+        <v>2983</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1090.71</v>
+        <v>2721.21</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -6952,10 +6977,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7611778380472685</v>
+        <v>0.7415024854722397</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -6970,18 +6995,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260921</v>
+        <v>20260922</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>BLSE</t>
+          <t>HAPPYFORGE</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>317.25</v>
+        <v>2108.5</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>297.99</v>
+        <v>1921.29</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -6993,7 +7018,7 @@
         <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7533567953850789</v>
+        <v>0.7390845760694532</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-23
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 22 Sep 2026</t>
+          <t>As of Wed 23 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹200,739</t>
+          <t>₹202,379</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-708  (-0.35%)</t>
+          <t>₹+1,640  (+0.82%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.37%</t>
+          <t>+1.19%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-2.60%</t>
+          <t>-1.80%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹132,859</t>
+          <t>₹134,498</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8835.5</v>
+        <v>9069</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8835.5</v>
+        <v>9069</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-82</v>
+        <v>151.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.009195402298850575</v>
+        <v>0.01698906644238856</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03376832097787342</v>
+        <v>0.05864593670746505</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1992.4</v>
+        <v>1962.6</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9962</v>
+        <v>9813</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>932.5</v>
+        <v>783.4999999999991</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1032726064566144</v>
+        <v>0.08677113904424376</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1605.14</v>
@@ -910,13 +910,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.08685863423867855</v>
+        <v>0.0729935508290752</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>9352</v>
+        <v>9624</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9352</v>
+        <v>9624</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>113</v>
+        <v>385</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01223076090485983</v>
+        <v>0.04167117653425696</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8902.93</v>
@@ -958,13 +958,13 @@
         <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.04801860564585112</v>
+        <v>0.07492414796342474</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>736.25</v>
+        <v>743.7</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9571.25</v>
+        <v>9668.1</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>445.25</v>
+        <v>542.1000000000006</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.04878917378917379</v>
+        <v>0.05940170940170947</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>683.88</v>
@@ -1006,13 +1006,13 @@
         <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.04713073005093385</v>
+        <v>0.05667607906413889</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>719.35</v>
+        <v>723.75</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9351.550000000001</v>
+        <v>9408.75</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>381.5500000000003</v>
+        <v>438.75</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.042536231884058</v>
+        <v>0.04891304347826087</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>627</v>
@@ -1054,13 +1054,13 @@
         <v>627</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1283797873079864</v>
+        <v>0.1336787564766839</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>864.05</v>
+        <v>860.25</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9504.549999999999</v>
+        <v>9462.75</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>215.0499999999995</v>
+        <v>173.25</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.02314979277679095</v>
+        <v>0.01865008880994671</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>801.9400000000001</v>
@@ -1102,13 +1102,13 @@
         <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06810948440483772</v>
+        <v>0.06399302528334794</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1487.8</v>
+        <v>1496.1</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8926.799999999999</v>
+        <v>8976.599999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>82.20000000000027</v>
+        <v>132</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.009293806390339899</v>
+        <v>0.01492436062682315</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1378.14</v>
@@ -1150,13 +1150,13 @@
         <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07370614329883039</v>
+        <v>0.07884499699217955</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2310.8</v>
+        <v>2334.1</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9243.200000000001</v>
+        <v>9336.4</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>18.80000000000109</v>
+        <v>112</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.00203807293699331</v>
+        <v>0.01214171111400199</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>2152.33</v>
@@ -1198,13 +1198,13 @@
         <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.06857798165137625</v>
+        <v>0.07787584079516729</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8950</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4448.8</v>
+        <v>4601.9</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8897.6</v>
+        <v>9203.799999999999</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-52.39999999999964</v>
+        <v>253.7999999999993</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.005854748603351914</v>
+        <v>0.02835754189944126</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>4316.53</v>
@@ -1246,13 +1246,13 @@
         <v>4316.53</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.02973161301924124</v>
+        <v>0.06201134314087658</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>111.57</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>8910</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>809</v>
+        <v>833</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8899</v>
+        <v>9163</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-11</v>
+        <v>253</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.001234567901234568</v>
+        <v>0.02839506172839506</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>761.28</v>
@@ -1294,13 +1294,13 @@
         <v>761.28</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.0589864029666255</v>
+        <v>0.08609843937575033</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>7587.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1909.8</v>
+        <v>1924.3</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>7639.2</v>
+        <v>7697.2</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>51.59999999999945</v>
+        <v>109.5999999999995</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.00680056934999202</v>
+        <v>0.01444462016975057</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1777.36</v>
@@ -1342,13 +1342,13 @@
         <v>1777.36</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.06934757566237305</v>
+        <v>0.0763602348906096</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>8160</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1363.9</v>
+        <v>1387.2</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8183.400000000001</v>
+        <v>8323.200000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>23.40000000000055</v>
+        <v>163.2000000000003</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.002867647058823596</v>
+        <v>0.02000000000000004</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1305.76</v>
@@ -1390,13 +1390,13 @@
         <v>1305.76</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.04262775863333096</v>
+        <v>0.05870818915801618</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>30.54</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>9297.84</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>161.77</v>
+        <v>164.4</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>9220.890000000001</v>
+        <v>9370.800000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-76.94999999999968</v>
+        <v>72.96000000000006</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.008276115743011245</v>
+        <v>0.007846983815595888</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>153.62</v>
@@ -1438,13 +1438,13 @@
         <v>153.62</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05038016937627499</v>
+        <v>0.06557177615571777</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>4.22</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>7866.4</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2006.5</v>
+        <v>2034</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8026</v>
+        <v>8136</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>159.6000000000004</v>
+        <v>269.6000000000004</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.02028882334994411</v>
+        <v>0.03427234821519378</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1839.47</v>
@@ -1486,13 +1486,13 @@
         <v>1839.47</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.08324445551956142</v>
+        <v>0.09563913470993116</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4659,7 +4659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6380,6 +6380,31 @@
         <v>-1275.21</v>
       </c>
       <c r="G68" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B69" s="20" t="n">
+        <v>202378.63</v>
+      </c>
+      <c r="C69" s="20" t="n">
+        <v>67880.42999999999</v>
+      </c>
+      <c r="D69" s="20" t="n">
+        <v>134498.2</v>
+      </c>
+      <c r="E69" s="20" t="n">
+        <v>130657.94</v>
+      </c>
+      <c r="F69" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G69" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6463,18 +6488,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>BLSE</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>328.1</v>
+        <v>4601.9</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>306.83</v>
+        <v>4377.5</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6483,10 +6508,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8437000280053211</v>
+        <v>0.8864057929656846</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6501,7 +6526,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -6509,10 +6534,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>809</v>
+        <v>833</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>763.01</v>
+        <v>788.13</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6521,10 +6546,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8060120422880347</v>
+        <v>0.8529581936220303</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6539,18 +6564,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>4448.8</v>
+        <v>9624</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>4235.7</v>
+        <v>9223.209999999999</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6559,10 +6584,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8032319890779248</v>
+        <v>0.781411321966184</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6577,18 +6602,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>CUPID</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>258.2</v>
+        <v>1185.4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>234.3</v>
+        <v>1097.04</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6600,7 +6625,7 @@
         <v>6.6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7423148148148149</v>
+        <v>0.8126448241421131</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6615,18 +6640,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>CUPID</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1909.8</v>
+        <v>273.85</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1799.47</v>
+        <v>248.11</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6635,10 +6660,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7799077574739202</v>
+        <v>0.7437383177570093</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6653,18 +6678,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>DIXON</t>
+          <t>INNOVACAP</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>13084</v>
+        <v>1297.6</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>12280.57</v>
+        <v>1185.87</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6676,7 +6701,7 @@
         <v>6.5</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7436655464538263</v>
+        <v>0.7760526503531426</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6691,18 +6716,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>GLAXO</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1190.9</v>
+        <v>2876.9</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1101.36</v>
+        <v>2714.26</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6711,10 +6736,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7896121263039977</v>
+        <v>0.781014839123921</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6729,18 +6754,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>BLSE</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>9352</v>
+        <v>322.45</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>8967.93</v>
+        <v>300.6</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6752,7 +6777,7 @@
         <v>6.4</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7334863123993558</v>
+        <v>0.8005612827281158</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6767,18 +6792,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>VARROC</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>864.5</v>
+        <v>11400</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>786.12</v>
+        <v>11027</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6790,7 +6815,7 @@
         <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7604949940488692</v>
+        <v>0.7395039951487479</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6805,18 +6830,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>AKUMS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>48290</v>
+        <v>823.3</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>46011.43</v>
+        <v>762.83</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6825,10 +6850,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7563053980256249</v>
+        <v>0.7523582078904187</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6843,18 +6868,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>11363</v>
+        <v>1924.3</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>10946.57</v>
+        <v>1814.04</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6863,10 +6888,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7392494573969054</v>
+        <v>0.7491337304701434</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6881,18 +6906,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SHINDL</t>
+          <t>UNITDSPR</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>162.53</v>
+        <v>1441</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>151.82</v>
+        <v>1379.53</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -6901,10 +6926,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7733333333333332</v>
+        <v>0.7423150460155525</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6919,18 +6944,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>STYLAMIND</t>
+          <t>TIIL</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>3309.4</v>
+        <v>3019.9</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>3061.3</v>
+        <v>2746.11</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -6942,7 +6967,7 @@
         <v>6.2</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7386238885388223</v>
+        <v>0.7530960619248055</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6957,18 +6982,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>TIIL</t>
+          <t>HONASA</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>2983</v>
+        <v>484.9</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>2721.21</v>
+        <v>454.73</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -6977,10 +7002,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7415024854722397</v>
+        <v>0.73862916458586</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -6995,18 +7020,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260922</v>
+        <v>20260923</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>HAPPYFORGE</t>
+          <t>AARTIDRUGS</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>2108.5</v>
+        <v>436.25</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1921.29</v>
+        <v>404.45</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -7018,7 +7043,7 @@
         <v>6.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7390845760694532</v>
+        <v>0.7448269957908255</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-24
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 23 Sep 2026</t>
+          <t>As of Thu 24 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹202,379</t>
+          <t>₹201,226</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,640  (+0.82%)</t>
+          <t>₹-1,153  (-0.57%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+1.19%</t>
+          <t>+0.61%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-1.80%</t>
+          <t>-2.36%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹134,498</t>
+          <t>₹133,345</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>9069</v>
+        <v>8888.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9069</v>
+        <v>8888.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>151.5</v>
+        <v>-29</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.01698906644238856</v>
+        <v>-0.003252032520325203</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.05864593670746505</v>
+        <v>0.03952972942566244</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1962.6</v>
+        <v>1997.1</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9813</v>
+        <v>9985.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>783.4999999999991</v>
+        <v>955.9999999999991</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.08677113904424376</v>
+        <v>0.1058751868874244</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1605.14</v>
@@ -910,13 +910,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.0729935508290752</v>
+        <v>0.08900763249569024</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>9624</v>
+        <v>9602</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9624</v>
+        <v>9602</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>385</v>
+        <v>363</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.04167117653425696</v>
+        <v>0.03928996644658513</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8902.93</v>
@@ -958,13 +958,13 @@
         <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07492414796342474</v>
+        <v>0.07280462403665899</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>743.7</v>
+        <v>728.8</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9668.1</v>
+        <v>9474.4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>542.1000000000006</v>
+        <v>348.3999999999994</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.05940170940170947</v>
+        <v>0.03817663817663811</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>683.88</v>
@@ -1006,13 +1006,13 @@
         <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.05667607906413889</v>
+        <v>0.03739023051591658</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>723.75</v>
+        <v>724.85</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9408.75</v>
+        <v>9423.050000000001</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>438.75</v>
+        <v>453.0500000000003</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.04891304347826087</v>
+        <v>0.05050724637681163</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>627</v>
@@ -1054,13 +1054,13 @@
         <v>627</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1336787564766839</v>
+        <v>0.1349934469200524</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>860.25</v>
+        <v>853</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9462.75</v>
+        <v>9383</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>173.25</v>
+        <v>93.5</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.01865008880994671</v>
+        <v>0.01006512729425696</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>801.9400000000001</v>
@@ -1102,13 +1102,13 @@
         <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06399302528334794</v>
+        <v>0.05603751465416186</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1496.1</v>
+        <v>1506.2</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8976.599999999999</v>
+        <v>9037.200000000001</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>132</v>
+        <v>192.6000000000008</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.01492436062682315</v>
+        <v>0.02177599891459205</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1378.14</v>
@@ -1150,13 +1150,13 @@
         <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07884499699217955</v>
+        <v>0.08502190944097726</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2334.1</v>
+        <v>2261.4</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9336.4</v>
+        <v>9045.6</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>112</v>
+        <v>-178.7999999999993</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.01214171111400199</v>
+        <v>-0.01938337452842454</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>2152.33</v>
@@ -1198,13 +1198,13 @@
         <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07787584079516729</v>
+        <v>0.04823118422216333</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8950</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4601.9</v>
+        <v>4481.3</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>9203.799999999999</v>
+        <v>8962.6</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>253.7999999999993</v>
+        <v>12.60000000000036</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02835754189944126</v>
+        <v>0.00140782122905032</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>4316.53</v>
@@ -1246,13 +1246,13 @@
         <v>4316.53</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.06201134314087658</v>
+        <v>0.03676834847031005</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>111.57</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>8910</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>833</v>
+        <v>816.3</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>9163</v>
+        <v>8979.299999999999</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>253</v>
+        <v>69.2999999999995</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.02839506172839506</v>
+        <v>0.007777777777777722</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>761.28</v>
@@ -1294,13 +1294,13 @@
         <v>761.28</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.08609843937575033</v>
+        <v>0.06740169055494302</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>7587.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1924.3</v>
+        <v>1961.3</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>7697.2</v>
+        <v>7845.2</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>109.5999999999995</v>
+        <v>257.5999999999995</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01444462016975057</v>
+        <v>0.03395012915809999</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1777.36</v>
@@ -1342,13 +1342,13 @@
         <v>1777.36</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.0763602348906096</v>
+        <v>0.09378473461479633</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>8160</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1387.2</v>
+        <v>1351</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8323.200000000001</v>
+        <v>8106</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>163.2000000000003</v>
+        <v>-54</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.02000000000000004</v>
+        <v>-0.006617647058823529</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1305.76</v>
@@ -1390,13 +1390,13 @@
         <v>1305.76</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05870818915801618</v>
+        <v>0.03348630643967433</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>30.54</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>9297.84</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>164.4</v>
+        <v>162.5</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>9370.800000000001</v>
+        <v>9262.5</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>72.96000000000006</v>
+        <v>-35.34000000000026</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.007846983815595888</v>
+        <v>-0.003800882785679282</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>153.62</v>
@@ -1438,13 +1438,13 @@
         <v>153.62</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.06557177615571777</v>
+        <v>0.05464615384615382</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>4.22</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>7866.4</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2034</v>
+        <v>2026.2</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8136</v>
+        <v>8104.8</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>269.6000000000004</v>
+        <v>238.4000000000005</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.03427234821519378</v>
+        <v>0.03030611207159572</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1839.47</v>
@@ -1486,13 +1486,13 @@
         <v>1839.47</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.09563913470993116</v>
+        <v>0.09215773368867831</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4659,7 +4659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6405,6 +6405,31 @@
         <v>-1275.21</v>
       </c>
       <c r="G69" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B70" s="20" t="n">
+        <v>201225.68</v>
+      </c>
+      <c r="C70" s="20" t="n">
+        <v>67880.42999999999</v>
+      </c>
+      <c r="D70" s="20" t="n">
+        <v>133345.25</v>
+      </c>
+      <c r="E70" s="20" t="n">
+        <v>130657.94</v>
+      </c>
+      <c r="F70" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G70" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6488,18 +6513,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>4601.9</v>
+        <v>816.3</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>4377.5</v>
+        <v>771.42</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6508,10 +6533,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8864057929656846</v>
+        <v>0.8433280698362229</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6526,18 +6551,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>833</v>
+        <v>9602</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>788.13</v>
+        <v>9186.639999999999</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6549,7 +6574,7 @@
         <v>7</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8529581936220303</v>
+        <v>0.8317872258147678</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6564,18 +6589,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>9624</v>
+        <v>4481.3</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>9223.209999999999</v>
+        <v>4255.41</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6584,10 +6609,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.781411321966184</v>
+        <v>0.8418396101431528</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6602,18 +6627,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>NEULANDLAB</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1185.4</v>
+        <v>21905</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1097.04</v>
+        <v>20305.71</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6622,10 +6647,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8126448241421131</v>
+        <v>0.8201461247054949</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6640,18 +6665,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>CUPID</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>273.85</v>
+        <v>1961.3</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>248.11</v>
+        <v>1846.49</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6660,10 +6685,10 @@
         <v>9333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7437383177570093</v>
+        <v>0.8285691523263226</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6678,18 +6703,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>INNOVACAP</t>
+          <t>SHINDL</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1297.6</v>
+        <v>162.78</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1185.87</v>
+        <v>152.35</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6698,10 +6723,10 @@
         <v>9333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7760526503531426</v>
+        <v>0.8370786516853932</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6716,18 +6741,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>GLAXO</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>2876.9</v>
+        <v>162.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>2714.26</v>
+        <v>155.15</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6736,10 +6761,10 @@
         <v>9333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.781014839123921</v>
+        <v>0.7593199704957713</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6754,18 +6779,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>BLSE</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>322.45</v>
+        <v>374.55</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>300.6</v>
+        <v>350.9</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6774,10 +6799,10 @@
         <v>9333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.8005612827281158</v>
+        <v>0.7763905300019335</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6792,18 +6817,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>11400</v>
+        <v>1097.9</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>11027</v>
+        <v>1030.67</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6815,7 +6840,7 @@
         <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7395039951487479</v>
+        <v>0.7474049527001382</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6830,18 +6855,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>AKUMS</t>
+          <t>BLSE</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>823.3</v>
+        <v>326.7</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>762.83</v>
+        <v>304.61</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6853,7 +6878,7 @@
         <v>6.3</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7523582078904187</v>
+        <v>0.7848563459155979</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6868,18 +6893,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>AARTIDRUGS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1924.3</v>
+        <v>437.25</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1814.04</v>
+        <v>406.48</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6891,7 +6916,7 @@
         <v>6.3</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7491337304701434</v>
+        <v>0.771104116985699</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6906,18 +6931,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>UNITDSPR</t>
+          <t>GOKULAGRO</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1441</v>
+        <v>224.98</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1379.53</v>
+        <v>210.31</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -6929,7 +6954,7 @@
         <v>6.3</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7423150460155525</v>
+        <v>0.7662642060712829</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6944,18 +6969,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>TIIL</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>3019.9</v>
+        <v>763.8</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>2746.11</v>
+        <v>717.49</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -6964,10 +6989,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7530960619248055</v>
+        <v>0.7664804749321474</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -6982,18 +7007,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>484.9</v>
+        <v>1221.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>454.73</v>
+        <v>1166.6</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -7002,10 +7027,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.73862916458586</v>
+        <v>0.749163927499803</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7020,18 +7045,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260923</v>
+        <v>20260924</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>AARTIDRUGS</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>436.25</v>
+        <v>1172.3</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>404.45</v>
+        <v>1082.14</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -7040,10 +7065,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7448269957908255</v>
+        <v>0.756412335918534</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-25
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 24 Sep 2026</t>
+          <t>As of Fri 25 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹201,226</t>
+          <t>₹202,159</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,153  (-0.57%)</t>
+          <t>₹+933  (+0.46%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.61%</t>
+          <t>+1.08%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-2.36%</t>
+          <t>-1.91%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹133,345</t>
+          <t>₹134,278</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8888.5</v>
+        <v>8889</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8888.5</v>
+        <v>8889</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-29</v>
+        <v>-28.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.003252032520325203</v>
+        <v>-0.0031959629941127</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03952972942566244</v>
+        <v>0.03958375520306003</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1997.1</v>
+        <v>1970.8</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9985.5</v>
+        <v>9854</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>955.9999999999991</v>
+        <v>824.4999999999993</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.1058751868874244</v>
+        <v>0.09131181128523166</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1605.14</v>
@@ -910,13 +910,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.08900763249569024</v>
+        <v>0.07685059004320227</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>9602</v>
+        <v>9619.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9602</v>
+        <v>9619.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>363</v>
+        <v>380.5</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.03928996644658513</v>
+        <v>0.0411841108345059</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8902.93</v>
@@ -958,13 +958,13 @@
         <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.07280462403665899</v>
+        <v>0.07449139768179217</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>728.8</v>
+        <v>726.8</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9474.4</v>
+        <v>9448.4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>348.3999999999994</v>
+        <v>322.3999999999994</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.03817663817663811</v>
+        <v>0.03532763532763526</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>683.88</v>
@@ -1006,13 +1006,13 @@
         <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.03739023051591658</v>
+        <v>0.03474133186571272</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>724.85</v>
+        <v>752.45</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9423.050000000001</v>
+        <v>9781.85</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>453.0500000000003</v>
+        <v>811.8500000000006</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.05050724637681163</v>
+        <v>0.09050724637681166</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>627</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>627</v>
+        <v>652.7642857142858</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1349934469200524</v>
+        <v>0.1324815127725619</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>853</v>
+        <v>868.65</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9383</v>
+        <v>9555.15</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>93.5</v>
+        <v>265.6499999999997</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.01006512729425696</v>
+        <v>0.02859680284191827</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>801.9400000000001</v>
@@ -1102,13 +1102,13 @@
         <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.05603751465416186</v>
+        <v>0.07304437920911765</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1506.2</v>
+        <v>1495.4</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>9037.200000000001</v>
+        <v>8972.400000000001</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>192.6000000000008</v>
+        <v>127.8000000000011</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.02177599891459205</v>
+        <v>0.0144494946068789</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1378.14</v>
@@ -1150,13 +1150,13 @@
         <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08502190944097726</v>
+        <v>0.07841380232713654</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2261.4</v>
+        <v>2317.6</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9045.6</v>
+        <v>9270.4</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-178.7999999999993</v>
+        <v>46</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.01938337452842454</v>
+        <v>0.004986774207536533</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>2152.33</v>
@@ -1198,13 +1198,13 @@
         <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.04823118422216333</v>
+        <v>0.07131083879875733</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8950</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4481.3</v>
+        <v>4557.1</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8962.6</v>
+        <v>9114.200000000001</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>12.60000000000036</v>
+        <v>164.2000000000007</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.00140782122905032</v>
+        <v>0.01834636871508388</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>4316.53</v>
@@ -1246,13 +1246,13 @@
         <v>4316.53</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.03676834847031005</v>
+        <v>0.05279015163152018</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>111.57</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>8910</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>816.3</v>
+        <v>824.5</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8979.299999999999</v>
+        <v>9069.5</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>69.2999999999995</v>
+        <v>159.5</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.007777777777777722</v>
+        <v>0.01790123456790123</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>761.28</v>
@@ -1294,13 +1294,13 @@
         <v>761.28</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06740169055494302</v>
+        <v>0.07667677380230446</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>7587.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1961.3</v>
+        <v>1952.3</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>7845.2</v>
+        <v>7809.2</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>257.5999999999995</v>
+        <v>221.5999999999995</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.03395012915809999</v>
+        <v>0.02920554589066364</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1777.36</v>
@@ -1342,13 +1342,13 @@
         <v>1777.36</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.09378473461479633</v>
+        <v>0.08960713005173389</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>8160</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1351</v>
+        <v>1362.6</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8106</v>
+        <v>8175.599999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-54</v>
+        <v>15.59999999999945</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.006617647058823529</v>
+        <v>0.001911764705882286</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1305.76</v>
@@ -1390,13 +1390,13 @@
         <v>1305.76</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.03348630643967433</v>
+        <v>0.04171436958755315</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>30.54</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>9297.84</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>162.5</v>
+        <v>165.71</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>9262.5</v>
+        <v>9445.470000000001</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-35.34000000000026</v>
+        <v>147.6300000000002</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.003800882785679282</v>
+        <v>0.01587788131436981</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>153.62</v>
@@ -1438,13 +1438,13 @@
         <v>153.62</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05464615384615382</v>
+        <v>0.07295878341681251</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>4.22</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>7866.4</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2026.2</v>
+        <v>2007</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8104.8</v>
+        <v>8028</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>238.4000000000005</v>
+        <v>161.6000000000004</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.03030611207159572</v>
+        <v>0.02054306925658502</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1839.47</v>
@@ -1486,13 +1486,13 @@
         <v>1839.47</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.09215773368867831</v>
+        <v>0.08347284504235175</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4659,7 +4659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6430,6 +6430,31 @@
         <v>-1275.21</v>
       </c>
       <c r="G70" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B71" s="20" t="n">
+        <v>202158.7</v>
+      </c>
+      <c r="C71" s="20" t="n">
+        <v>67880.42999999999</v>
+      </c>
+      <c r="D71" s="20" t="n">
+        <v>134278.27</v>
+      </c>
+      <c r="E71" s="20" t="n">
+        <v>130657.94</v>
+      </c>
+      <c r="F71" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G71" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6513,7 +6538,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -6521,22 +6546,22 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>816.3</v>
+        <v>824.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>771.42</v>
+        <v>779.95</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G2" s="14" t="n">
         <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8433280698362229</v>
+        <v>0.8377653236838621</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6551,30 +6576,30 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>9602</v>
+        <v>4557.1</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>9186.639999999999</v>
+        <v>4330.8</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8317872258147678</v>
+        <v>0.8473565082447083</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6589,30 +6614,30 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>4481.3</v>
+        <v>1952.3</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>4255.41</v>
+        <v>1835.4</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G4" s="14" t="n">
         <v>6.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8418396101431528</v>
+        <v>0.8419490902137299</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6627,30 +6652,30 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>NEULANDLAB</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>21905</v>
+        <v>9619.5</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>20305.71</v>
+        <v>9208.5</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8201461247054949</v>
+        <v>0.8183637821220011</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6665,30 +6690,30 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1961.3</v>
+        <v>48250</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1846.49</v>
+        <v>46116.43</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.8285691523263226</v>
+        <v>0.8122054410661489</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6703,30 +6728,30 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SHINDL</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>162.78</v>
+        <v>376.45</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>152.35</v>
+        <v>352.42</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G7" s="14" t="n">
         <v>6.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.8370786516853932</v>
+        <v>0.7927696997778856</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6741,30 +6766,30 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>NEULANDLAB</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>162.5</v>
+        <v>21890</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>155.15</v>
+        <v>20245.71</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G8" s="14" t="n">
         <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7593199704957713</v>
+        <v>0.7921772722592413</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6779,30 +6804,30 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>HYUNDAI</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>374.55</v>
+        <v>2115</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>350.9</v>
+        <v>2002.71</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7763905300019335</v>
+        <v>0.7593048997543503</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6817,30 +6842,30 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>SHINDL</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1097.9</v>
+        <v>161.16</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1030.67</v>
+        <v>151.13</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>6.4</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7474049527001382</v>
+        <v>0.8037950664136622</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6855,30 +6880,30 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>BLSE</t>
+          <t>QUESS</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>326.7</v>
+        <v>340.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>304.61</v>
+        <v>306.15</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0467</v>
+        <v>0.0458</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>9333</v>
+        <v>9168</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7848563459155979</v>
+        <v>0.7720696718297221</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6893,30 +6918,30 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>AARTIDRUGS</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>437.25</v>
+        <v>752.45</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>406.48</v>
+        <v>702.61</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.771104116985699</v>
+        <v>0.755762470029272</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6931,30 +6956,30 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>GOKULAGRO</t>
+          <t>INDGN</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>224.98</v>
+        <v>608.95</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>210.31</v>
+        <v>574.6900000000001</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7662642060712829</v>
+        <v>0.7535766294514805</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -6969,30 +6994,30 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>RAINBOW</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>763.8</v>
+        <v>1374.2</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>717.49</v>
+        <v>1291.31</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>6.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7664804749321474</v>
+        <v>0.7525430990100466</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7007,30 +7032,30 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>KAJARIACER</t>
+          <t>BLSE</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1221.8</v>
+        <v>324.55</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1166.6</v>
+        <v>302.26</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.749163927499803</v>
+        <v>0.7603290528514481</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7045,30 +7070,30 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260924</v>
+        <v>20260925</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>ENDURANCE</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1172.3</v>
+        <v>2645.9</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1082.14</v>
+        <v>2496.19</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>9333</v>
+        <v>9345</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.756412335918534</v>
+        <v>0.7508035097009547</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-28
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
@@ -868,7 +868,7 @@
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
@@ -964,7 +964,7 @@
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -1012,7 +1012,7 @@
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -1060,7 +1060,7 @@
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1108,7 +1108,7 @@
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1156,7 +1156,7 @@
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -1204,7 +1204,7 @@
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
@@ -1252,7 +1252,7 @@
         <v>111.57</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1300,7 +1300,7 @@
         <v>23.57</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1348,7 +1348,7 @@
         <v>56.89</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1396,7 +1396,7 @@
         <v>30.54</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1444,7 +1444,7 @@
         <v>4.22</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -1492,7 +1492,7 @@
         <v>55</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V5 daily refresh 2026-09-29
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 28 Sep 2026</t>
+          <t>As of Tue 29 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹200,160</t>
+          <t>₹199,910</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,998  (-0.99%)</t>
+          <t>₹-250  (-0.13%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>+0.08%</t>
+          <t>-0.05%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-2.88%</t>
+          <t>-3.00%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹132,280</t>
+          <t>₹132,029</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>8917.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>8860</v>
+        <v>8659</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>8860</v>
+        <v>8659</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-57.5</v>
+        <v>-258.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.006447995514437903</v>
+        <v>-0.02898794505186431</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8537.139999999999</v>
@@ -862,13 +862,13 @@
         <v>8537.139999999999</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03644018058690752</v>
+        <v>0.01407321861646848</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>194.79</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9029.5</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1919.3</v>
+        <v>1938.1</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9596.5</v>
+        <v>9690.5</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>566.9999999999993</v>
+        <v>660.9999999999991</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.06279417464975905</v>
+        <v>0.07320449637299951</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1605.14</v>
@@ -910,13 +910,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.0520799994045449</v>
+        <v>0.06127503372227593</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9239</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>9550</v>
+        <v>9431</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9550</v>
+        <v>9431</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>311</v>
+        <v>192</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.03366165169390627</v>
+        <v>0.02078146985604503</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>8902.93</v>
@@ -958,13 +958,13 @@
         <v>8902.93</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06775602094240835</v>
+        <v>0.05599300180256597</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>9126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>711</v>
+        <v>714.35</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>9243</v>
+        <v>9286.550000000001</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>117</v>
+        <v>160.5500000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.01282051282051282</v>
+        <v>0.01759259259259262</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>683.88</v>
@@ -1006,13 +1006,13 @@
         <v>701.55</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.01329113924050639</v>
+        <v>0.01791838734513903</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
@@ -1036,31 +1036,31 @@
         <v>8970</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>752.8</v>
+        <v>763.3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9786.4</v>
+        <v>9922.9</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>816.3999999999994</v>
+        <v>952.8999999999994</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.09101449275362312</v>
+        <v>0.1062318840579709</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>627</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>655.1</v>
+        <v>665.8857142857142</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1297821466524973</v>
+        <v>0.1276225412213883</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>9289.5</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>851.4</v>
+        <v>866.75</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>9365.4</v>
+        <v>9534.25</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>75.89999999999975</v>
+        <v>244.75</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.008170515097690914</v>
+        <v>0.02634695085849615</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>801.9400000000001</v>
@@ -1102,13 +1102,13 @@
         <v>805.1999999999999</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.05426356589147292</v>
+        <v>0.07101240265359109</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>24.01</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>8844.6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1433.4</v>
+        <v>1415.1</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8600.400000000001</v>
+        <v>8490.599999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-244.1999999999989</v>
+        <v>-354</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.0276100671596227</v>
+        <v>-0.04002442168102571</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1378.14</v>
@@ -1150,13 +1150,13 @@
         <v>1378.14</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.03855169526998743</v>
+        <v>0.02611829552681776</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>47.59</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>9224.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2261.7</v>
+        <v>2309.8</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>9046.799999999999</v>
+        <v>9239.200000000001</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>-177.6000000000004</v>
+        <v>14.80000000000109</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>-0.01925328476648892</v>
+        <v>0.001604440397207525</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>2152.33</v>
@@ -1198,13 +1198,13 @@
         <v>2152.33</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.04835743025158062</v>
+        <v>0.06817473374318134</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>8950</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4478.3</v>
+        <v>4364</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8956.6</v>
+        <v>8728</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>6.600000000000364</v>
+        <v>-222</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.000737430167597806</v>
+        <v>-0.02480446927374302</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>4316.53</v>
@@ -1246,13 +1246,13 @@
         <v>4316.53</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.03612308241966827</v>
+        <v>0.01087763519706697</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>111.57</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>8910</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>807.9</v>
+        <v>815.65</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>8886.9</v>
+        <v>8972.15</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-23.10000000000025</v>
+        <v>62.14999999999975</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.002592592592592621</v>
+        <v>0.006975308641975281</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>761.28</v>
@@ -1294,13 +1294,13 @@
         <v>761.28</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.05770516152989232</v>
+        <v>0.06665849322626127</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>7587.6</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1942.1</v>
+        <v>1950.4</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>7768.4</v>
+        <v>7801.6</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>180.7999999999993</v>
+        <v>214</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.02382835152090243</v>
+        <v>0.02820391164531604</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1777.36</v>
@@ -1342,13 +1342,13 @@
         <v>1777.36</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.08482570413469956</v>
+        <v>0.0887202625102544</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>8160</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1346</v>
+        <v>1345.7</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>8076</v>
+        <v>8074.200000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-84</v>
+        <v>-85.79999999999973</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.01029411764705882</v>
+        <v>-0.01051470588235291</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1305.76</v>
@@ -1390,13 +1390,13 @@
         <v>1305.76</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.0298959881129272</v>
+        <v>0.02967972059151375</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>30.54</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>9297.84</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>162.37</v>
+        <v>158.56</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>9255.09</v>
+        <v>9037.92</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-42.75</v>
+        <v>-259.9200000000001</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.004597842079450711</v>
+        <v>-0.02795487984306034</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>153.62</v>
@@ -1438,13 +1438,13 @@
         <v>153.62</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05388926525836053</v>
+        <v>0.03115539858728555</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>4.22</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>7866.4</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2010.7</v>
+        <v>1979</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>8042.8</v>
+        <v>7916</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>176.4000000000005</v>
+        <v>49.60000000000036</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.02242448896572772</v>
+        <v>0.006305298484694443</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1839.47</v>
@@ -1486,13 +1486,13 @@
         <v>1839.47</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.08515939722484707</v>
+        <v>0.0705053057099545</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -4659,7 +4659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6480,6 +6480,31 @@
         <v>-1275.21</v>
       </c>
       <c r="G72" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B73" s="20" t="n">
+        <v>199909.9</v>
+      </c>
+      <c r="C73" s="20" t="n">
+        <v>67880.42999999999</v>
+      </c>
+      <c r="D73" s="20" t="n">
+        <v>132029.47</v>
+      </c>
+      <c r="E73" s="20" t="n">
+        <v>130657.94</v>
+      </c>
+      <c r="F73" s="20" t="n">
+        <v>-1275.21</v>
+      </c>
+      <c r="G73" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -6563,7 +6588,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -6571,10 +6596,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>807.9</v>
+        <v>815.65</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>761.9299999999999</v>
+        <v>769.34</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0467</v>
@@ -6583,10 +6608,10 @@
         <v>9333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8587331084710077</v>
+        <v>0.8300320767045554</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6601,18 +6626,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>GLAXO</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2896.4</v>
+        <v>1979</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>2728.09</v>
+        <v>1881.37</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0467</v>
@@ -6621,10 +6646,10 @@
         <v>9333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8126470735672188</v>
+        <v>0.8231186383823278</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -6639,18 +6664,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>11024</v>
+        <v>9431</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>10645.86</v>
+        <v>9046.93</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0467</v>
@@ -6659,10 +6684,10 @@
         <v>9333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8074678998288469</v>
+        <v>0.8179152587975079</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -6677,18 +6702,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>9550</v>
+        <v>10811</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>9143.709999999999</v>
+        <v>10425.43</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0467</v>
@@ -6697,10 +6722,10 @@
         <v>9333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7970886057819694</v>
+        <v>0.8108195982375284</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -6715,18 +6740,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>DIXON</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>13640</v>
+        <v>1143.2</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>12868.86</v>
+        <v>1059.93</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0467</v>
@@ -6738,7 +6763,7 @@
         <v>6.8</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7853304187165659</v>
+        <v>0.8402536435712065</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -6753,18 +6778,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>UNITDSPR</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>4738</v>
+        <v>1363</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>4514.49</v>
+        <v>1302.29</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0467</v>
@@ -6776,7 +6801,7 @@
         <v>6.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7751494904791573</v>
+        <v>0.7690611798496798</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -6791,18 +6816,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>379.65</v>
+        <v>1950.4</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>355.61</v>
+        <v>1831.07</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0467</v>
@@ -6814,7 +6839,7 @@
         <v>6.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.784650281794029</v>
+        <v>0.7904984118886471</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -6829,18 +6854,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>ZYDUSLIFE</t>
+          <t>LODHA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1215</v>
+        <v>1106.6</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1160.11</v>
+        <v>1023.79</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0467</v>
@@ -6852,7 +6877,7 @@
         <v>6.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7681075042430232</v>
+        <v>0.7417648826474812</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -6867,18 +6892,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SIS</t>
+          <t>NEULANDLAB</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>394.2</v>
+        <v>21375</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>366.54</v>
+        <v>19802.14</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0467</v>
@@ -6887,10 +6912,10 @@
         <v>9333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7710391289091313</v>
+        <v>0.7712997354894842</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -6905,18 +6930,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>47020</v>
+        <v>388.4</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>44982.86</v>
+        <v>362.31</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0467</v>
@@ -6925,10 +6950,10 @@
         <v>9333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7662484513860541</v>
+        <v>0.7817718360943293</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -6943,18 +6968,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>HONASA</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>466.05</v>
+        <v>4364</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>434.41</v>
+        <v>4125.94</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0467</v>
@@ -6963,10 +6988,10 @@
         <v>9333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7508335660730014</v>
+        <v>0.7732872332619353</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -6981,18 +7006,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>4478.3</v>
+        <v>1190.5</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>4246.06</v>
+        <v>1133.77</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0467</v>
@@ -7001,10 +7026,10 @@
         <v>9333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7450773769881338</v>
+        <v>0.7455557341477136</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7019,18 +7044,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>AARTIDRUGS</t>
+          <t>INDGN</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>429.65</v>
+        <v>605.15</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>398.93</v>
+        <v>569.29</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0467</v>
@@ -7039,10 +7064,10 @@
         <v>9333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7551865139894444</v>
+        <v>0.7634559679093187</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7057,7 +7082,7 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
@@ -7065,10 +7090,10 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1996.7</v>
+        <v>2074.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1837.06</v>
+        <v>1908.44</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0467</v>
@@ -7077,10 +7102,10 @@
         <v>9333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7526910076553448</v>
+        <v>0.7760465985764653</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7095,18 +7120,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20260928</v>
+        <v>20260929</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>INDIGOPNTS</t>
+          <t>AARTIDRUGS</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1110</v>
+        <v>428.6</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1032.81</v>
+        <v>395.99</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0467</v>
@@ -7115,10 +7140,10 @@
         <v>9333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7472262802472053</v>
+        <v>0.7446295979230509</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-02
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3">
@@ -868,7 +868,7 @@
         <v>73.94</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>170.46</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -964,7 +964,7 @@
         <v>13.22</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -1012,7 +1012,7 @@
         <v>25.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
@@ -1060,7 +1060,7 @@
         <v>24.01</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -1108,7 +1108,7 @@
         <v>23.57</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -1156,7 +1156,7 @@
         <v>56.89</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -1204,7 +1204,7 @@
         <v>4.22</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -1252,7 +1252,7 @@
         <v>55</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-07
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 06 Oct 2026</t>
+          <t>As of Wed 07 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹198,583</t>
+          <t>₹198,319</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,164  (+0.59%)</t>
+          <t>₹-264  (-0.13%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-0.71%</t>
+          <t>-0.84%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-3.65%</t>
+          <t>-3.77%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹98,458</t>
+          <t>₹98,194</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9029.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1945.5</v>
+        <v>1938.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9727.5</v>
+        <v>9692.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>697.9999999999995</v>
+        <v>662.9999999999995</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.07730217620023251</v>
+        <v>0.07342599257987702</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1605.14</v>
@@ -862,13 +862,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.06484561442155902</v>
+        <v>0.06146873503076764</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9239</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9550</v>
+        <v>9588</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9550</v>
+        <v>9588</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>311</v>
+        <v>349</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.03366165169390627</v>
+        <v>0.03777465093624851</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8902.93</v>
@@ -910,13 +910,13 @@
         <v>8902.93</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.06775602094240835</v>
+        <v>0.0714507717980809</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9126</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>736</v>
+        <v>731.3</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9568</v>
+        <v>9506.9</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>442</v>
+        <v>380.8999999999994</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.04843304843304843</v>
+        <v>0.04173789173789167</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>683.88</v>
@@ -958,13 +958,13 @@
         <v>701.55</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.04680706521739136</v>
+        <v>0.04068097907835362</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>8970</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>796.5</v>
+        <v>802.1</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10354.5</v>
+        <v>10427.3</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1384.5</v>
+        <v>1457.3</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1543478260869565</v>
+        <v>0.1624637681159421</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>627</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>713.7571428571429</v>
+        <v>727.1</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.1038830598152632</v>
+        <v>0.09350455055479366</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8910</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>820</v>
+        <v>810.5</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>9020</v>
+        <v>8915.5</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>110</v>
+        <v>5.5</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.01234567901234568</v>
+        <v>0.0006172839506172839</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>761.28</v>
@@ -1054,13 +1054,13 @@
         <v>761.28</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.07160975609756101</v>
+        <v>0.06072794571252317</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>7587.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1964.2</v>
+        <v>1945.1</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>7856.8</v>
+        <v>7780.4</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>269.1999999999998</v>
+        <v>192.7999999999993</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.03547893932205174</v>
+        <v>0.02540987927671454</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1777.36</v>
@@ -1102,13 +1102,13 @@
         <v>1777.36</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.09512269626310974</v>
+        <v>0.08623721145442395</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>9297.84</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>160</v>
+        <v>159.2</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>9120</v>
+        <v>9074.4</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-177.8400000000003</v>
+        <v>-223.4400000000009</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.01912702305051498</v>
+        <v>-0.02403138793526248</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>153.62</v>
@@ -1150,13 +1150,13 @@
         <v>153.62</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.03987499999999997</v>
+        <v>0.03505025125628131</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>4.22</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>7866.4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2050</v>
+        <v>2052.8</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>8200</v>
+        <v>8211.200000000001</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>333.6000000000004</v>
+        <v>344.8000000000011</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.04240821722770268</v>
+        <v>0.04383199430489183</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1839.47</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1840.657142857142</v>
+        <v>1856.971428571428</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1021184668989549</v>
+        <v>0.09539583565304553</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>4242</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4460.1</v>
+        <v>4495</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4460.1</v>
+        <v>4495</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>218.1000000000004</v>
+        <v>253</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.0514144271570015</v>
+        <v>0.05964167845355964</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>3979.77</v>
@@ -1246,13 +1246,13 @@
         <v>3979.77</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.107694894733302</v>
+        <v>0.114622914349277</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>126.65</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>5025</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>338.2</v>
+        <v>341.25</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>5073</v>
+        <v>5118.75</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>47.99999999999983</v>
+        <v>93.75</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.009552238805970115</v>
+        <v>0.01865671641791045</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>306.13</v>
@@ -1294,13 +1294,13 @@
         <v>306.13</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.09482554701360141</v>
+        <v>0.1029157509157509</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4249.2</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>2152</v>
+        <v>2135</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4304</v>
+        <v>4270</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>54.80000000000018</v>
+        <v>20.80000000000018</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01289654523204372</v>
+        <v>0.004895039066177206</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1983.64</v>
@@ -1342,13 +1342,13 @@
         <v>1983.64</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.07823420074349438</v>
+        <v>0.07089461358313813</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4006</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1989.4</v>
+        <v>1934.3</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>3978.8</v>
+        <v>3868.6</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-27.19999999999982</v>
+        <v>-137.4000000000001</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.006789815277084328</v>
+        <v>-0.03429855217174241</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1842.51</v>
@@ -1390,13 +1390,13 @@
         <v>1842.51</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.07383633256258174</v>
+        <v>0.04745385927725791</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>79.15000000000001</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4907,7 +4907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6853,6 +6853,31 @@
         <v>-4952.3</v>
       </c>
       <c r="G77" s="14" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B78" s="20" t="n">
+        <v>198318.97</v>
+      </c>
+      <c r="C78" s="20" t="n">
+        <v>100124.82</v>
+      </c>
+      <c r="D78" s="20" t="n">
+        <v>98194.14999999999</v>
+      </c>
+      <c r="E78" s="20" t="n">
+        <v>94794.14</v>
+      </c>
+      <c r="F78" s="20" t="n">
+        <v>-4952.3</v>
+      </c>
+      <c r="G78" s="14" t="n">
         <v>13</v>
       </c>
     </row>
@@ -6936,7 +6961,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -6944,10 +6969,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>4460.1</v>
+        <v>4495</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>4194.27</v>
+        <v>4234.67</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -6956,10 +6981,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8509634228384229</v>
+        <v>0.8150977224011481</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -6974,18 +6999,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2050</v>
+        <v>9588</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1945.33</v>
+        <v>9190.209999999999</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -6994,10 +7019,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8325706388206389</v>
+        <v>0.8139444643250884</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7012,18 +7037,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>9550</v>
+        <v>9884</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>9136.639999999999</v>
+        <v>9403.860000000001</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -7032,10 +7057,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8227810196560197</v>
+        <v>0.7976923994491255</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7050,18 +7075,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>677.65</v>
+        <v>2052.8</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>621.24</v>
+        <v>1954.89</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -7070,10 +7095,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7704026266526267</v>
+        <v>0.795347025674948</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7088,18 +7113,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>NEULANDLAB</t>
+          <t>GLAND</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>21905</v>
+        <v>3150.6</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>20498.57</v>
+        <v>2972.21</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -7108,10 +7133,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7682074119574119</v>
+        <v>0.7810163346599146</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7126,18 +7151,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>HAPPYFORGE</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1989.4</v>
+        <v>1561.8</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1836.29</v>
+        <v>1463.14</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -7146,10 +7171,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7908425470925471</v>
+        <v>0.7948619379651619</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7164,18 +7189,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>4816</v>
+        <v>802.1</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>4602.14</v>
+        <v>764.6</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -7184,10 +7209,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7304851117351117</v>
+        <v>0.7860896942356976</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7202,18 +7227,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1964.2</v>
+        <v>1294.1</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1818.29</v>
+        <v>1193.04</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -7222,10 +7247,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7540416227916228</v>
+        <v>0.7683039280537574</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7240,18 +7265,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>GLAXO</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>796.5</v>
+        <v>2634</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>755.13</v>
+        <v>2466.86</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -7263,7 +7288,7 @@
         <v>5.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.747025272025272</v>
+        <v>0.7677617286762022</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7278,18 +7303,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>RRKABEL</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>2789.7</v>
+        <v>1945.1</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>2607.57</v>
+        <v>1817.66</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -7301,7 +7326,7 @@
         <v>5.6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7289655727155727</v>
+        <v>0.7611694879107612</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7316,18 +7341,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>HAPPYFORGE</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>45000</v>
+        <v>1934.3</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>42512.14</v>
+        <v>1785.73</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -7336,10 +7361,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.745130967005967</v>
+        <v>0.752481465817944</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7354,18 +7379,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>INDGN</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>820</v>
+        <v>607.1</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>766.88</v>
+        <v>566.91</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -7377,7 +7402,7 @@
         <v>5.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7266851673101673</v>
+        <v>0.7474897976150457</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7392,18 +7417,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>KPIL</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1451.5</v>
+        <v>1067.3</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1360.36</v>
+        <v>997.64</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -7415,7 +7440,7 @@
         <v>5.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7239627208377208</v>
+        <v>0.7439168844500833</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7430,18 +7455,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>VARROC</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>814.45</v>
+        <v>661.25</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>745.29</v>
+        <v>605.15</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -7450,10 +7475,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7332426582426583</v>
+        <v>0.7398746073572841</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7468,18 +7493,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261006</v>
+        <v>20261007</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SOMANYCERA</t>
+          <t>ADOR</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>625</v>
+        <v>1552.1</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>582.76</v>
+        <v>1440.13</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -7491,7 +7516,7 @@
         <v>5.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7309596934596935</v>
+        <v>0.7388964796801747</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-09
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 08 Oct 2026</t>
+          <t>As of Fri 09 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹196,502</t>
+          <t>₹197,155</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,817  (-0.92%)</t>
+          <t>₹+654  (+0.33%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-1.75%</t>
+          <t>-1.42%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-4.66%</t>
+          <t>-4.34%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹87,631</t>
+          <t>₹88,285</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9029.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1938.4</v>
+        <v>1915.4</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9692</v>
+        <v>9577</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>662.5</v>
+        <v>547.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.0733706185281577</v>
+        <v>0.06063458663270391</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1605.14</v>
@@ -862,13 +862,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.06142031719827856</v>
+        <v>0.05014991273736199</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9239</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9361</v>
+        <v>9340</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9361</v>
+        <v>9340</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.01320489230436194</v>
+        <v>0.01093191903885702</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8902.93</v>
@@ -910,13 +910,13 @@
         <v>8902.93</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.04893387458604847</v>
+        <v>0.04679550321199141</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9126</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>711.65</v>
+        <v>715.65</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9251.449999999999</v>
+        <v>9303.449999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>125.4499999999997</v>
+        <v>177.4499999999997</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01374643874643871</v>
+        <v>0.01944444444444441</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>683.88</v>
@@ -958,13 +958,13 @@
         <v>701.55</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.01419236984472707</v>
+        <v>0.01970236847621047</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>8970</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>800.75</v>
+        <v>811.8</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10409.75</v>
+        <v>10553.4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1439.75</v>
+        <v>1583.399999999999</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1605072463768116</v>
+        <v>0.1765217391304347</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>627</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>727.1</v>
+        <v>742.7571428571428</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.09197627224477049</v>
+        <v>0.08504909724421927</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8910</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>793</v>
+        <v>783.3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>8723</v>
+        <v>8616.299999999999</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-187</v>
+        <v>-293.7000000000005</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.02098765432098765</v>
+        <v>-0.03296296296296302</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>761.28</v>
@@ -1054,13 +1054,13 @@
         <v>761.28</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04000000000000004</v>
+        <v>0.02811183454615088</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>7587.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1898.9</v>
+        <v>1933.6</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>7595.6</v>
+        <v>7734.4</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>8</v>
+        <v>146.7999999999993</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.001054351837208076</v>
+        <v>0.0193473562127681</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1777.36</v>
@@ -1102,13 +1102,13 @@
         <v>1777.36</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.06400547685502142</v>
+        <v>0.08080264791063302</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>7866.4</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1997.9</v>
+        <v>2036.6</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>7991.6</v>
+        <v>8146.4</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>125.2000000000007</v>
+        <v>280</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.01591579375572063</v>
+        <v>0.03559442692972643</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1839.47</v>
@@ -1150,13 +1150,13 @@
         <v>1860.571428571429</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.06873645899623164</v>
+        <v>0.08643256968897722</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4242</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4415</v>
+        <v>4550</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4415</v>
+        <v>4550</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>173</v>
+        <v>308</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.04078264969354078</v>
+        <v>0.07260726072607261</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3979.77</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>3979.77</v>
+        <v>4016.857142857143</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.09857984144960363</v>
+        <v>0.1171742543171114</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>126.65</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5025</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>332.3</v>
+        <v>343</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4984.5</v>
+        <v>5145</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-40.49999999999983</v>
+        <v>120</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.008059701492537279</v>
+        <v>0.02388059701492537</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>306.13</v>
@@ -1246,13 +1246,13 @@
         <v>306.13</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.07875413782726456</v>
+        <v>0.1074927113702624</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4249.2</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2040</v>
+        <v>2114.1</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4080</v>
+        <v>4228.2</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-169.1999999999998</v>
+        <v>-21</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.03981926009601804</v>
+        <v>-0.00494210674950579</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1983.64</v>
@@ -1294,13 +1294,13 @@
         <v>1983.64</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.02762745098039211</v>
+        <v>0.06170947448086647</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4006</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1940.9</v>
+        <v>1922.6</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>3881.8</v>
+        <v>3845.2</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-124.1999999999998</v>
+        <v>-160.8000000000002</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.03100349475786316</v>
+        <v>-0.04013979031452825</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1842.51</v>
@@ -1342,13 +1342,13 @@
         <v>1842.51</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.05069297748467211</v>
+        <v>0.04165713096848014</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>79.15000000000001</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4902,7 +4902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6898,6 +6898,31 @@
         <v>-5524.56</v>
       </c>
       <c r="G79" s="14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B80" s="20" t="n">
+        <v>197155.25</v>
+      </c>
+      <c r="C80" s="20" t="n">
+        <v>108870.3</v>
+      </c>
+      <c r="D80" s="20" t="n">
+        <v>88284.95</v>
+      </c>
+      <c r="E80" s="20" t="n">
+        <v>85496.3</v>
+      </c>
+      <c r="F80" s="20" t="n">
+        <v>-5524.56</v>
+      </c>
+      <c r="G80" s="14" t="n">
         <v>12</v>
       </c>
     </row>
@@ -6981,30 +7006,30 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>376</v>
+        <v>9340</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>350.45</v>
+        <v>8923.209999999999</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G2" s="14" t="n">
         <v>6.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8221680642907058</v>
+        <v>0.8151164151164152</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7019,30 +7044,30 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>9361</v>
+        <v>4550</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8953.57</v>
+        <v>4283.43</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8133298392732355</v>
+        <v>0.8089303995553996</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7057,7 +7082,7 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
@@ -7065,22 +7090,22 @@
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1997.9</v>
+        <v>2036.6</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1901.79</v>
+        <v>1936.89</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7609032145352901</v>
+        <v>0.7946519977769977</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7095,30 +7120,30 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>7666</v>
+        <v>43545</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>7222.14</v>
+        <v>41153.57</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7260464709993012</v>
+        <v>0.7921313765063764</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7133,30 +7158,30 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>800.75</v>
+        <v>8027.5</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>762.75</v>
+        <v>7557.14</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7539430468204052</v>
+        <v>0.7535637504387505</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7171,30 +7196,30 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1938.4</v>
+        <v>811.8</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1826.86</v>
+        <v>777.28</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7466649196366177</v>
+        <v>0.7629584942084942</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7209,7 +7234,7 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
@@ -7217,22 +7242,22 @@
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1505.6</v>
+        <v>1487.9</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1403.37</v>
+        <v>1388.51</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7490216631726067</v>
+        <v>0.7674896893646893</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7247,30 +7272,30 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>153.08</v>
+        <v>783.3</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>143.98</v>
+        <v>734.34</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7332512229210343</v>
+        <v>0.7591695185445186</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7285,30 +7310,30 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1898.9</v>
+        <v>9778</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1768.61</v>
+        <v>9255.57</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7359853249475891</v>
+        <v>0.7391540891540892</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7323,30 +7348,30 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>PRICOLLTD</t>
+          <t>COFORGE</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>650.1</v>
+        <v>1867.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>594.24</v>
+        <v>1752.11</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7416422082459818</v>
+        <v>0.7287802006552007</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7361,30 +7386,30 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>ADOR</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1486.1</v>
+        <v>377.65</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1368.53</v>
+        <v>353.13</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7596715583508036</v>
+        <v>0.7580697174447174</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7399,30 +7424,30 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1066.1</v>
+        <v>1693</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>982.76</v>
+        <v>1621.9</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.735798392732355</v>
+        <v>0.7258899321399321</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7437,30 +7462,30 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>UNIPARTS</t>
+          <t>SUDEEPPHRM</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>776.6</v>
+        <v>1050.3</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>714.47</v>
+        <v>924.9400000000001</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0226</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>5333</v>
+        <v>4517</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7293588399720474</v>
+        <v>0.7230329355329356</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7475,30 +7500,30 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>INDIGOPNTS</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1035.7</v>
+        <v>1023.6</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>964.89</v>
+        <v>934.23</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7312596086652691</v>
+        <v>0.7304065022815023</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7513,30 +7538,30 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261008</v>
+        <v>20261009</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>HNDFDS</t>
+          <t>UNIPARTS</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>572.6</v>
+        <v>757.95</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>536.6900000000001</v>
+        <v>698.22</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.027</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>5333</v>
+        <v>5392</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7325768693221523</v>
+        <v>0.7296807359307359</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-12
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 09 Oct 2026</t>
+          <t>As of Mon 12 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹197,155</t>
+          <t>₹198,043</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+654  (+0.33%)</t>
+          <t>₹+888  (+0.45%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-1.42%</t>
+          <t>-0.98%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-4.34%</t>
+          <t>-3.91%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹108,870</t>
+          <t>₹95,308</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹85,496</t>
+          <t>₹99,029</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹88,285</t>
+          <t>₹102,735</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -697,7 +697,7 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9029.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1915.4</v>
+        <v>1899.9</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9577</v>
+        <v>9499.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>547.5</v>
+        <v>470</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.06063458663270391</v>
+        <v>0.05205160861620244</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1605.14</v>
@@ -862,13 +862,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.05014991273736199</v>
+        <v>0.04240072785785734</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9239</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9340</v>
+        <v>9426</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9340</v>
+        <v>9426</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>101</v>
+        <v>187</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.01093191903885702</v>
+        <v>0.02024028574521052</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8902.93</v>
@@ -910,13 +910,13 @@
         <v>8902.93</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.04679550321199141</v>
+        <v>0.05549225546361126</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9126</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>715.65</v>
+        <v>711.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9303.449999999999</v>
+        <v>9249.5</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>177.4499999999997</v>
+        <v>123.5</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01944444444444441</v>
+        <v>0.01353276353276353</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>683.88</v>
@@ -958,13 +958,13 @@
         <v>701.55</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.01970236847621047</v>
+        <v>0.01398453970484898</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>8970</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>811.8</v>
+        <v>823.5</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10553.4</v>
+        <v>10705.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1583.399999999999</v>
+        <v>1735.5</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1765217391304347</v>
+        <v>0.1934782608695652</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>627</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>742.7571428571428</v>
+        <v>753.6428571428571</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08504909724421927</v>
+        <v>0.08482956023939635</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8910</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>783.3</v>
+        <v>798</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>8616.299999999999</v>
+        <v>8778</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-293.7000000000005</v>
+        <v>-132</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.03296296296296302</v>
+        <v>-0.01481481481481482</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>761.28</v>
@@ -1054,13 +1054,13 @@
         <v>761.28</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.02811183454615088</v>
+        <v>0.04601503759398499</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>7587.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1933.6</v>
+        <v>1969.7</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>7734.4</v>
+        <v>7878.8</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>146.7999999999993</v>
+        <v>291.1999999999998</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.0193473562127681</v>
+        <v>0.03837840687437395</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1777.36</v>
@@ -1102,13 +1102,13 @@
         <v>1777.36</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.08080264791063302</v>
+        <v>0.09764938823171049</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1132,31 +1132,31 @@
         <v>7866.4</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2036.6</v>
+        <v>2069.2</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8146.4</v>
+        <v>8276.799999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>280</v>
+        <v>410.3999999999996</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.03559442692972643</v>
+        <v>0.05217126004271327</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1839.47</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1860.571428571429</v>
+        <v>1880.171428571428</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08643256968897722</v>
+        <v>0.09135345613211458</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4242</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4550</v>
+        <v>4555</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4550</v>
+        <v>4555</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.07260726072607261</v>
+        <v>0.07378595002357378</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3979.77</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>4016.857142857143</v>
+        <v>4039.885714285715</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1171742543171114</v>
+        <v>0.113087658773718</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>126.65</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5025</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5145</v>
+        <v>5100</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>120</v>
+        <v>75</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02388059701492537</v>
+        <v>0.01492537313432836</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>306.13</v>
@@ -1246,13 +1246,13 @@
         <v>306.13</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.1074927113702624</v>
+        <v>0.09961764705882355</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4249.2</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2114.1</v>
+        <v>2157.4</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4228.2</v>
+        <v>4314.8</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-21</v>
+        <v>65.60000000000036</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.00494210674950579</v>
+        <v>0.0154382001317896</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1983.64</v>
@@ -1294,13 +1294,13 @@
         <v>1983.64</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.06170947448086647</v>
+        <v>0.08054139241679799</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4006</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1922.6</v>
+        <v>1966.3</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>3845.2</v>
+        <v>3932.6</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-160.8000000000002</v>
+        <v>-73.40000000000009</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.04013979031452825</v>
+        <v>-0.01832251622566153</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1842.51</v>
@@ -1342,17 +1342,161 @@
         <v>1842.51</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.04165713096848014</v>
+        <v>0.06295580531963585</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>79.15000000000001</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>SAILIFE</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1489</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>4467</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1471.3</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>4413.9</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>-53.10000000000014</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>-0.0118871725990598</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>1388.51</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>1388.51</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.05626996533677698</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>50.46</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>COFORGE</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1880</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>3760</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1846.6</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>3693.2</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>-66.80000000000018</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>-0.01776595744680856</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1752.11</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>1752.11</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.05116971731831475</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>57.73</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>NAZARA</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>379</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>5306</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>404.7</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>5665.8</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>359.7999999999998</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0.06781002638522425</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>353.13</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>353.13</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.1274277242401779</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>14.18</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H13">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -4902,7 +5046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6924,6 +7068,31 @@
       </c>
       <c r="G80" s="14" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B81" s="20" t="n">
+        <v>198043.33</v>
+      </c>
+      <c r="C81" s="20" t="n">
+        <v>95308.33</v>
+      </c>
+      <c r="D81" s="20" t="n">
+        <v>102735</v>
+      </c>
+      <c r="E81" s="20" t="n">
+        <v>99029.3</v>
+      </c>
+      <c r="F81" s="20" t="n">
+        <v>-5524.56</v>
+      </c>
+      <c r="G81" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -7006,7 +7175,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -7014,22 +7183,22 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9340</v>
+        <v>9426</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8923.209999999999</v>
+        <v>9002.360000000001</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
         <v>6.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8151164151164152</v>
+        <v>0.8205243105950653</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7044,30 +7213,30 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>4550</v>
+        <v>2069.2</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>4283.43</v>
+        <v>1974.69</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8089303995553996</v>
+        <v>0.8157293178519593</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7082,30 +7251,30 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>2036.6</v>
+        <v>404.7</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1936.89</v>
+        <v>376.34</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
         <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7946519977769977</v>
+        <v>0.8117271407837445</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7120,30 +7289,30 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>43545</v>
+        <v>1706.9</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>41153.57</v>
+        <v>1635.59</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7921313765063764</v>
+        <v>0.7949673439767779</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7158,7 +7327,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
@@ -7166,22 +7335,22 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>8027.5</v>
+        <v>7775</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>7557.14</v>
+        <v>7277.07</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7535637504387505</v>
+        <v>0.7640747460087083</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7196,30 +7365,30 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>811.8</v>
+        <v>44585</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>777.28</v>
+        <v>42211.43</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7629584942084942</v>
+        <v>0.786416908563135</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7234,30 +7403,30 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1487.9</v>
+        <v>1169.7</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1388.51</v>
+        <v>1094.96</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7674896893646893</v>
+        <v>0.8226578374455733</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7272,30 +7441,30 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>783.3</v>
+        <v>10034</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>734.34</v>
+        <v>9477.139999999999</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7591695185445186</v>
+        <v>0.7632982583454282</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7310,30 +7479,30 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>9778</v>
+        <v>1471.3</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>9255.57</v>
+        <v>1370.39</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>5.7</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7391540891540892</v>
+        <v>0.7778392597968069</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7348,30 +7517,30 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>COFORGE</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1867.9</v>
+        <v>4555</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1752.11</v>
+        <v>4297.44</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7287802006552007</v>
+        <v>0.7707311320754717</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7386,30 +7555,30 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>377.65</v>
+        <v>798</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>353.13</v>
+        <v>750.14</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7580697174447174</v>
+        <v>0.7575380986937591</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7424,30 +7593,30 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1693</v>
+        <v>4760</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1621.9</v>
+        <v>4537.34</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7258899321399321</v>
+        <v>0.7420682148040639</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7462,30 +7631,30 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SUDEEPPHRM</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1050.3</v>
+        <v>7119</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>924.9400000000001</v>
+        <v>6813.57</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0226</v>
+        <v>0.0267</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>4517</v>
+        <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7230329355329356</v>
+        <v>0.7299945573294631</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7500,30 +7669,30 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1023.6</v>
+        <v>1969.7</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>934.23</v>
+        <v>1836.56</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7304065022815023</v>
+        <v>0.7387590711175618</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7538,30 +7707,30 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261009</v>
+        <v>20261012</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>UNIPARTS</t>
+          <t>ADOR</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>757.95</v>
+        <v>1540.2</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>698.22</v>
+        <v>1416.21</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.027</v>
+        <v>0.0267</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>5392</v>
+        <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7296807359307359</v>
+        <v>0.7400380986937591</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-13
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 12 Oct 2026</t>
+          <t>As of Tue 13 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹198,043</t>
+          <t>₹197,988</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+888  (+0.45%)</t>
+          <t>₹-55  (-0.03%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-0.98%</t>
+          <t>-1.01%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-3.91%</t>
+          <t>-3.93%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹102,735</t>
+          <t>₹102,680</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9029.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1899.9</v>
+        <v>1919.2</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9499.5</v>
+        <v>9596</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>470</v>
+        <v>566.4999999999998</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.05205160861620244</v>
+        <v>0.06273880059803973</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1605.14</v>
@@ -862,13 +862,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.04240072785785734</v>
+        <v>0.05203060799142514</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9239</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9426</v>
+        <v>9285</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9426</v>
+        <v>9285</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>187</v>
+        <v>46</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.02024028574521052</v>
+        <v>0.004978893819677454</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8902.93</v>
@@ -910,13 +910,13 @@
         <v>8902.93</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.05549225546361126</v>
+        <v>0.04114916532040923</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9126</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>711.5</v>
+        <v>724.15</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9249.5</v>
+        <v>9413.949999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>123.5</v>
+        <v>287.9499999999997</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.01353276353276353</v>
+        <v>0.03155270655270652</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>683.88</v>
@@ -958,13 +958,13 @@
         <v>701.55</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.01398453970484898</v>
+        <v>0.03120900365946285</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>8970</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>823.5</v>
+        <v>824.8</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10705.5</v>
+        <v>10722.4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1735.5</v>
+        <v>1752.399999999999</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1934782608695652</v>
+        <v>0.1953623188405796</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>627</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>753.6428571428571</v>
+        <v>759.1285714285714</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.08482956023939635</v>
+        <v>0.07962103367050022</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8910</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>798</v>
+        <v>802.95</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>8778</v>
+        <v>8832.450000000001</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-132</v>
+        <v>-77.5499999999995</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.01481481481481482</v>
+        <v>-0.008703703703703648</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>761.28</v>
@@ -1054,13 +1054,13 @@
         <v>761.28</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04601503759398499</v>
+        <v>0.05189613300952745</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>7587.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1969.7</v>
+        <v>1910.6</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>7878.8</v>
+        <v>7642.4</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>291.1999999999998</v>
+        <v>54.79999999999927</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.03837840687437395</v>
+        <v>0.007222310084875227</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1777.36</v>
@@ -1102,13 +1102,13 @@
         <v>1777.36</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.09764938823171049</v>
+        <v>0.0697372553124673</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>7866.4</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2069.2</v>
+        <v>2059.4</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8276.799999999999</v>
+        <v>8237.6</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>410.3999999999996</v>
+        <v>371.2000000000007</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.05217126004271327</v>
+        <v>0.0471880402725517</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1839.47</v>
@@ -1150,13 +1150,13 @@
         <v>1880.171428571428</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.09135345613211458</v>
+        <v>0.08702950928841979</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4242</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4555</v>
+        <v>4540</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4555</v>
+        <v>4540</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.07378595002357378</v>
+        <v>0.07024988213107025</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3979.77</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>4039.885714285715</v>
+        <v>4044.571428571429</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.113087658773718</v>
+        <v>0.1091252359974826</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>126.65</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5025</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5100</v>
+        <v>5070</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.01492537313432836</v>
+        <v>0.008955223880597015</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>306.13</v>
@@ -1246,13 +1246,13 @@
         <v>306.13</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09961764705882355</v>
+        <v>0.09428994082840238</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4249.2</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2157.4</v>
+        <v>2185</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4314.8</v>
+        <v>4370</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>65.60000000000036</v>
+        <v>120.8000000000002</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.0154382001317896</v>
+        <v>0.02842888073049049</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1983.64</v>
@@ -1294,13 +1294,13 @@
         <v>1983.64</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.08054139241679799</v>
+        <v>0.09215560640732261</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4006</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1966.3</v>
+        <v>1936.6</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>3932.6</v>
+        <v>3873.2</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-73.40000000000009</v>
+        <v>-132.8000000000002</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.01832251622566153</v>
+        <v>-0.03315027458811787</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1842.51</v>
@@ -1342,13 +1342,13 @@
         <v>1842.51</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.06295580531963585</v>
+        <v>0.04858514923061031</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>79.15000000000001</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4467</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1471.3</v>
+        <v>1462.3</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4413.9</v>
+        <v>4386.9</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-53.10000000000014</v>
+        <v>-80.10000000000014</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.0118871725990598</v>
+        <v>-0.01793149764942918</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1388.51</v>
@@ -1390,13 +1390,13 @@
         <v>1388.51</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05626996533677698</v>
+        <v>0.05046160158654173</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>50.46</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>3760</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1846.6</v>
+        <v>1929</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>3693.2</v>
+        <v>3858</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>-66.80000000000018</v>
+        <v>98</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>-0.01776595744680856</v>
+        <v>0.02606382978723404</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1752.11</v>
@@ -1438,13 +1438,13 @@
         <v>1752.11</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.05116971731831475</v>
+        <v>0.0917003628823225</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>5306</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>404.7</v>
+        <v>400.45</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>5665.8</v>
+        <v>5606.3</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>359.7999999999998</v>
+        <v>300.2999999999998</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.06781002638522425</v>
+        <v>0.05659630606860155</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>353.13</v>
@@ -1486,13 +1486,13 @@
         <v>353.13</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1274277242401779</v>
+        <v>0.1181670620551879</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5046,7 +5046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7092,6 +7092,31 @@
         <v>-5524.56</v>
       </c>
       <c r="G81" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B82" s="20" t="n">
+        <v>197988.13</v>
+      </c>
+      <c r="C82" s="20" t="n">
+        <v>95308.33</v>
+      </c>
+      <c r="D82" s="20" t="n">
+        <v>102679.8</v>
+      </c>
+      <c r="E82" s="20" t="n">
+        <v>99029.3</v>
+      </c>
+      <c r="F82" s="20" t="n">
+        <v>-5524.56</v>
+      </c>
+      <c r="G82" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7175,7 +7200,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -7183,10 +7208,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9426</v>
+        <v>9285</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>9002.360000000001</v>
+        <v>8842.360000000001</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -7198,7 +7223,7 @@
         <v>6.1</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8205243105950653</v>
+        <v>0.817126191819883</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7213,18 +7238,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2069.2</v>
+        <v>1462.3</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1974.69</v>
+        <v>1357.01</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -7233,10 +7258,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8157293178519593</v>
+        <v>0.822923040365937</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7251,18 +7276,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>NEULANDLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>404.7</v>
+        <v>20360</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>376.34</v>
+        <v>18898.57</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -7271,10 +7296,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8117271407837445</v>
+        <v>0.7877435619449312</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7289,18 +7314,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1706.9</v>
+        <v>2059.4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1635.59</v>
+        <v>1960.49</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -7312,7 +7337,7 @@
         <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7949673439767779</v>
+        <v>0.7758294472331957</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7327,18 +7352,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>7775</v>
+        <v>10318</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>7277.07</v>
+        <v>9737.860000000001</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -7347,10 +7372,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7640747460087083</v>
+        <v>0.7577969525054209</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7365,18 +7390,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>HYUNDAI</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>44585</v>
+        <v>1964.9</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>42211.43</v>
+        <v>1844.23</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -7385,10 +7410,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.786416908563135</v>
+        <v>0.7570748061900378</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7403,18 +7428,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1169.7</v>
+        <v>1919.2</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1094.96</v>
+        <v>1806.23</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -7423,10 +7448,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.8226578374455733</v>
+        <v>0.7644885941723349</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7441,18 +7466,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>10034</v>
+        <v>4869</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>9477.139999999999</v>
+        <v>4638.96</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -7461,10 +7486,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7632982583454282</v>
+        <v>0.7357972940861972</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7479,18 +7504,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>NYKAA</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1471.3</v>
+        <v>338</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1370.39</v>
+        <v>317.08</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -7502,7 +7527,7 @@
         <v>5.7</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7778392597968069</v>
+        <v>0.7376318056256869</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7517,18 +7542,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>4555</v>
+        <v>1684.6</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>4297.44</v>
+        <v>1611.61</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -7540,7 +7565,7 @@
         <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7707311320754717</v>
+        <v>0.7516199097038643</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7555,18 +7580,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>HAPPYFORGE</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>798</v>
+        <v>1936.6</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>750.14</v>
+        <v>1770.54</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -7575,10 +7600,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7575380986937591</v>
+        <v>0.7627873733923427</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7593,18 +7618,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>4760</v>
+        <v>44900</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>4537.34</v>
+        <v>42496.43</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -7613,10 +7638,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7420682148040639</v>
+        <v>0.7443204770249799</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7631,18 +7656,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>7119</v>
+        <v>400.45</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>6813.57</v>
+        <v>371.16</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -7654,7 +7679,7 @@
         <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7299945573294631</v>
+        <v>0.7474258918228531</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7669,18 +7694,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1969.7</v>
+        <v>802.95</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1836.56</v>
+        <v>754.65</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -7689,10 +7714,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7387590711175618</v>
+        <v>0.7360972911159296</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7707,7 +7732,7 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261012</v>
+        <v>20261013</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
@@ -7715,10 +7740,10 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1540.2</v>
+        <v>1529</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1416.21</v>
+        <v>1405.44</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -7727,10 +7752,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7400380986937591</v>
+        <v>0.7605741527311611</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-14
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 13 Oct 2026</t>
+          <t>As of Wed 14 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹197,988</t>
+          <t>₹197,668</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-55  (-0.03%)</t>
+          <t>₹-320  (-0.16%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-1.01%</t>
+          <t>-1.17%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-3.93%</t>
+          <t>-4.09%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹102,680</t>
+          <t>₹102,359</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9029.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1919.2</v>
+        <v>1911.6</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9596</v>
+        <v>9558</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>566.4999999999998</v>
+        <v>528.4999999999991</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.06273880059803973</v>
+        <v>0.05853037266736797</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1605.14</v>
@@ -862,13 +862,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.05203060799142514</v>
+        <v>0.0482617403521359</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9239</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9285</v>
+        <v>9023</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9285</v>
+        <v>9023</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>46</v>
+        <v>-216</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.004978893819677454</v>
+        <v>-0.02337915358805066</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8902.93</v>
@@ -910,13 +910,13 @@
         <v>8902.93</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.04114916532040923</v>
+        <v>0.01330710406738332</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9126</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>724.15</v>
+        <v>725.4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9413.949999999999</v>
+        <v>9430.199999999999</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>287.9499999999997</v>
+        <v>304.1999999999997</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.03155270655270652</v>
+        <v>0.0333333333333333</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>683.88</v>
@@ -958,13 +958,13 @@
         <v>701.55</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03120900365946285</v>
+        <v>0.03287841191067001</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>8970</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>824.8</v>
+        <v>826.45</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10722.4</v>
+        <v>10743.85</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1752.399999999999</v>
+        <v>1773.850000000001</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1953623188405796</v>
+        <v>0.1977536231884059</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>627</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>759.1285714285714</v>
+        <v>760.3928571428571</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.07962103367050022</v>
+        <v>0.07992878317761865</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8910</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>802.95</v>
+        <v>807</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>8832.450000000001</v>
+        <v>8877</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-77.5499999999995</v>
+        <v>-33</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.008703703703703648</v>
+        <v>-0.003703703703703704</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>761.28</v>
@@ -1054,13 +1054,13 @@
         <v>761.28</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.05189613300952745</v>
+        <v>0.05665427509293684</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>7587.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1910.6</v>
+        <v>1938</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>7642.4</v>
+        <v>7752</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>54.79999999999927</v>
+        <v>164.3999999999996</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.007222310084875227</v>
+        <v>0.02166693025462592</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1777.36</v>
@@ -1102,13 +1102,13 @@
         <v>1777.36</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.0697372553124673</v>
+        <v>0.08288957688338498</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>7866.4</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2059.4</v>
+        <v>2036.9</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8237.6</v>
+        <v>8147.6</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>371.2000000000007</v>
+        <v>281.2000000000007</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.0471880402725517</v>
+        <v>0.03574697447371106</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1839.47</v>
@@ -1150,13 +1150,13 @@
         <v>1880.171428571428</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.08702950928841979</v>
+        <v>0.07694465679639242</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4242</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4540</v>
+        <v>4554.1</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4540</v>
+        <v>4554.1</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>298</v>
+        <v>312.1000000000004</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.07024988213107025</v>
+        <v>0.07357378595002366</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3979.77</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>4044.571428571429</v>
+        <v>4069.314285714286</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1091252359974826</v>
+        <v>0.1064503885039227</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>126.65</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5025</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>338</v>
+        <v>336.5</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5070</v>
+        <v>5047.5</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>45</v>
+        <v>22.5</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.008955223880597015</v>
+        <v>0.004477611940298508</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>306.13</v>
@@ -1246,13 +1246,13 @@
         <v>306.13</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09428994082840238</v>
+        <v>0.09025260029717683</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4249.2</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2185</v>
+        <v>2160</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4370</v>
+        <v>4320</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>120.8000000000002</v>
+        <v>70.80000000000018</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.02842888073049049</v>
+        <v>0.01666195989833385</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1983.64</v>
@@ -1294,13 +1294,13 @@
         <v>1983.64</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.09215560640732261</v>
+        <v>0.08164814814814811</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4006</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1936.6</v>
+        <v>1917.7</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>3873.2</v>
+        <v>3835.4</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-132.8000000000002</v>
+        <v>-170.5999999999999</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.03315027458811787</v>
+        <v>-0.04258612081877182</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1842.51</v>
@@ -1342,13 +1342,13 @@
         <v>1842.51</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.04858514923061031</v>
+        <v>0.03920842676122441</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>79.15000000000001</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4467</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1462.3</v>
+        <v>1432.1</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4386.9</v>
+        <v>4296.299999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-80.10000000000014</v>
+        <v>-170.7000000000003</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.01793149764942918</v>
+        <v>-0.03821356615177978</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1388.51</v>
@@ -1390,13 +1390,13 @@
         <v>1388.51</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.05046160158654173</v>
+        <v>0.03043781858808737</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>50.46</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>3760</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1929</v>
+        <v>1928</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>3858</v>
+        <v>3856</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.02606382978723404</v>
+        <v>0.02553191489361702</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1752.11</v>
@@ -1438,13 +1438,13 @@
         <v>1752.11</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.0917003628823225</v>
+        <v>0.09122925311203324</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>5306</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>400.45</v>
+        <v>405.2</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>5606.3</v>
+        <v>5672.8</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>300.2999999999998</v>
+        <v>366.7999999999998</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.05659630606860155</v>
+        <v>0.06912928759894456</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>353.13</v>
@@ -1486,13 +1486,13 @@
         <v>353.13</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1181670620551879</v>
+        <v>0.1285044422507404</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5046,7 +5046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7117,6 +7117,31 @@
         <v>-5524.56</v>
       </c>
       <c r="G82" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B83" s="20" t="n">
+        <v>197667.68</v>
+      </c>
+      <c r="C83" s="20" t="n">
+        <v>95308.33</v>
+      </c>
+      <c r="D83" s="20" t="n">
+        <v>102359.35</v>
+      </c>
+      <c r="E83" s="20" t="n">
+        <v>99029.3</v>
+      </c>
+      <c r="F83" s="20" t="n">
+        <v>-5524.56</v>
+      </c>
+      <c r="G83" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7200,7 +7225,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -7208,10 +7233,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9285</v>
+        <v>9023</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8842.360000000001</v>
+        <v>8570.93</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -7220,10 +7245,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.817126191819883</v>
+        <v>0.8539886981317016</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7238,18 +7263,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1462.3</v>
+        <v>2036.9</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1357.01</v>
+        <v>1937.6</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -7261,7 +7286,7 @@
         <v>6</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.822923040365937</v>
+        <v>0.7921833694715894</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7276,18 +7301,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>NEULANDLAB</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>20360</v>
+        <v>45000</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>18898.57</v>
+        <v>42620.71</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -7299,7 +7324,7 @@
         <v>5.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7877435619449312</v>
+        <v>0.7935664003326699</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7314,18 +7339,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>2059.4</v>
+        <v>807</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1960.49</v>
+        <v>758.64</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -7337,7 +7362,7 @@
         <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7758294472331957</v>
+        <v>0.7733017494876289</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7352,18 +7377,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>10318</v>
+        <v>4933</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>9737.860000000001</v>
+        <v>4698.57</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -7372,10 +7397,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7577969525054209</v>
+        <v>0.738606795972317</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7390,18 +7415,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>HYUNDAI</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1964.9</v>
+        <v>1432.1</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1844.23</v>
+        <v>1325.7</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -7410,10 +7435,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7570748061900378</v>
+        <v>0.759678245759943</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7428,18 +7453,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>HNDFDS</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1919.2</v>
+        <v>582.1</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1806.23</v>
+        <v>544.74</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -7448,10 +7473,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7644885941723349</v>
+        <v>0.785719324561143</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7466,18 +7491,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>4869</v>
+        <v>1662.9</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>4638.96</v>
+        <v>1589.7</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -7486,10 +7511,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7357972940861972</v>
+        <v>0.7406161820179997</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7504,18 +7529,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>NYKAA</t>
+          <t>SIRCA</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>338</v>
+        <v>430.2</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>317.08</v>
+        <v>408.93</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -7524,10 +7549,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.7</v>
+        <v>5.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7376318056256869</v>
+        <v>0.7561462262749874</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7542,18 +7567,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>MINDACORP</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1684.6</v>
+        <v>657.15</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1611.61</v>
+        <v>619.26</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -7562,10 +7587,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.7</v>
+        <v>5.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7516199097038643</v>
+        <v>0.7543570113167196</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7580,18 +7605,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>HAPPYFORGE</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1936.6</v>
+        <v>405.2</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1770.54</v>
+        <v>375.25</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -7600,10 +7625,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7627873733923427</v>
+        <v>0.7405370986425878</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7618,18 +7643,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>44900</v>
+        <v>4554.1</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>42496.43</v>
+        <v>4311.26</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -7638,10 +7663,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7443204770249799</v>
+        <v>0.7264520895832716</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7656,18 +7681,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>400.45</v>
+        <v>1938</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>371.16</v>
+        <v>1794.9</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -7676,10 +7701,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7474258918228531</v>
+        <v>0.7347335669943862</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7694,18 +7719,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>802.95</v>
+        <v>847.75</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>754.65</v>
+        <v>792.26</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -7714,10 +7739,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7360972911159296</v>
+        <v>0.7304355897466361</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7732,18 +7757,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261013</v>
+        <v>20261014</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>ADOR</t>
+          <t>GPPL</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1529</v>
+        <v>175.53</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>1405.44</v>
+        <v>164.19</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -7755,7 +7780,7 @@
         <v>5.4</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7605741527311611</v>
+        <v>0.7282427896753497</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-15
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 14 Oct 2026</t>
+          <t>As of Thu 15 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹197,668</t>
+          <t>₹197,367</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-320  (-0.16%)</t>
+          <t>₹-301  (-0.15%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>-1.32%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-4.09%</t>
+          <t>-4.24%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹102,359</t>
+          <t>₹102,058</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9029.5</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1911.6</v>
+        <v>1913.1</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9558</v>
+        <v>9565.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>528.4999999999991</v>
+        <v>535.9999999999991</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.05853037266736797</v>
+        <v>0.05936098344315843</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>1605.14</v>
@@ -862,13 +862,13 @@
         <v>1819.342857142857</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.0482617403521359</v>
+        <v>0.04900796762173592</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>73.94</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9239</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>9023</v>
+        <v>9030</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9023</v>
+        <v>9030</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-216</v>
+        <v>-209</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02337915358805066</v>
+        <v>-0.02262149583288235</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8902.93</v>
@@ -910,13 +910,13 @@
         <v>8902.93</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.01330710406738332</v>
+        <v>0.01407198228128457</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>9126</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>725.4</v>
+        <v>741.45</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>9430.199999999999</v>
+        <v>9638.85</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>304.1999999999997</v>
+        <v>512.8500000000006</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.0333333333333333</v>
+        <v>0.05619658119658126</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>683.88</v>
@@ -958,13 +958,13 @@
         <v>701.55</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03287841191067001</v>
+        <v>0.05381347359902905</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>8970</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>826.45</v>
+        <v>835.15</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>10743.85</v>
+        <v>10856.95</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>1773.850000000001</v>
+        <v>1886.95</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.1977536231884059</v>
+        <v>0.2103623188405797</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>627</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>760.3928571428571</v>
+        <v>770.3071428571427</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.07992878317761865</v>
+        <v>0.07764216864378527</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>8910</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>807</v>
+        <v>801</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>8877</v>
+        <v>8811</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-33</v>
+        <v>-99</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.003703703703703704</v>
+        <v>-0.01111111111111111</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>761.28</v>
@@ -1054,13 +1054,13 @@
         <v>761.28</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.05665427509293684</v>
+        <v>0.04958801498127344</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>7587.6</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1938</v>
+        <v>1885.1</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>7752</v>
+        <v>7540.4</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>164.3999999999996</v>
+        <v>-47.20000000000073</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.02166693025462592</v>
+        <v>-0.006220675839527746</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1777.36</v>
@@ -1102,13 +1102,13 @@
         <v>1777.36</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.08288957688338498</v>
+        <v>0.05715346665959366</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>7866.4</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2036.9</v>
+        <v>2018.5</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>8147.6</v>
+        <v>8074</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>281.2000000000007</v>
+        <v>207.6000000000004</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.03574697447371106</v>
+        <v>0.02639072510932579</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1839.47</v>
@@ -1150,13 +1150,13 @@
         <v>1880.171428571428</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.07694465679639242</v>
+        <v>0.06853037970204194</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>4242</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4554.1</v>
+        <v>4449</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4554.1</v>
+        <v>4449</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>312.1000000000004</v>
+        <v>207</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.07357378595002366</v>
+        <v>0.0487977369165488</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>3979.77</v>
@@ -1198,13 +1198,13 @@
         <v>4069.314285714286</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1064503885039227</v>
+        <v>0.08534181035866799</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>126.65</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>5025</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>336.5</v>
+        <v>338.4</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5047.5</v>
+        <v>5076</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>22.5</v>
+        <v>50.99999999999966</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.004477611940298508</v>
+        <v>0.01014925373134322</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>306.13</v>
@@ -1246,13 +1246,13 @@
         <v>306.13</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09025260029717683</v>
+        <v>0.0953605200945626</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4249.2</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>2160</v>
+        <v>2139</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4320</v>
+        <v>4278</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>70.80000000000018</v>
+        <v>28.80000000000018</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.01666195989833385</v>
+        <v>0.006777746399322268</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1983.64</v>
@@ -1294,13 +1294,13 @@
         <v>1983.64</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.08164814814814811</v>
+        <v>0.07263207106124353</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4006</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1917.7</v>
+        <v>1873.2</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>3835.4</v>
+        <v>3746.4</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-170.5999999999999</v>
+        <v>-259.5999999999999</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.04258612081877182</v>
+        <v>-0.06480279580629054</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1842.51</v>
@@ -1342,13 +1342,13 @@
         <v>1842.51</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.03920842676122441</v>
+        <v>0.0163837283792441</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>79.15000000000001</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4467</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1432.1</v>
+        <v>1394.7</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4296.299999999999</v>
+        <v>4184.1</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>-170.7000000000003</v>
+        <v>-282.8999999999999</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>-0.03821356615177978</v>
+        <v>-0.06333109469442576</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1388.51</v>
@@ -1390,13 +1390,13 @@
         <v>1388.51</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.03043781858808737</v>
+        <v>0.004438230443823084</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>50.46</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>3760</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1928</v>
+        <v>1934.3</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>3856</v>
+        <v>3868.6</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>96</v>
+        <v>108.5999999999999</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.02553191489361702</v>
+        <v>0.02888297872340423</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1752.11</v>
@@ -1438,13 +1438,13 @@
         <v>1752.11</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.09122925311203324</v>
+        <v>0.09418911234038156</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>5306</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>405.2</v>
+        <v>406.7</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>5672.8</v>
+        <v>5693.8</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>366.7999999999998</v>
+        <v>387.7999999999998</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.06912928759894456</v>
+        <v>0.07308707124010551</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>353.13</v>
@@ -1486,13 +1486,13 @@
         <v>353.13</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1285044422507404</v>
+        <v>0.1317187115810179</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5046,7 +5046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7142,6 +7142,31 @@
         <v>-5524.56</v>
       </c>
       <c r="G83" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B84" s="20" t="n">
+        <v>197366.53</v>
+      </c>
+      <c r="C84" s="20" t="n">
+        <v>95308.33</v>
+      </c>
+      <c r="D84" s="20" t="n">
+        <v>102058.2</v>
+      </c>
+      <c r="E84" s="20" t="n">
+        <v>99029.3</v>
+      </c>
+      <c r="F84" s="20" t="n">
+        <v>-5524.56</v>
+      </c>
+      <c r="G84" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7225,7 +7250,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -7233,10 +7258,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9023</v>
+        <v>9030</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8570.93</v>
+        <v>8581.57</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -7248,7 +7273,7 @@
         <v>6.4</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8539886981317016</v>
+        <v>0.8473468771185192</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7263,18 +7288,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2036.9</v>
+        <v>1394.7</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1937.6</v>
+        <v>1289.17</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -7283,10 +7308,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7921833694715894</v>
+        <v>0.80449789253397</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7301,18 +7326,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>45000</v>
+        <v>4449</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>42620.71</v>
+        <v>4183.06</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -7324,7 +7349,7 @@
         <v>5.9</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7935664003326699</v>
+        <v>0.7864702154626109</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7339,18 +7364,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>807</v>
+        <v>842.1</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>758.64</v>
+        <v>785.52</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -7359,10 +7384,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7733017494876289</v>
+        <v>0.7973402452324108</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7377,18 +7402,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>4933</v>
+        <v>1885.1</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>4698.57</v>
+        <v>1739.61</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -7400,7 +7425,7 @@
         <v>5.7</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.738606795972317</v>
+        <v>0.7798928581955376</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7415,18 +7440,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1432.1</v>
+        <v>741.45</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1325.7</v>
+        <v>707.16</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -7435,10 +7460,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.759678245759943</v>
+        <v>0.7309399593244319</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7453,18 +7478,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>HNDFDS</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>582.1</v>
+        <v>1116.1</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>544.74</v>
+        <v>1039.27</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -7476,7 +7501,7 @@
         <v>5.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.785719324561143</v>
+        <v>0.7849312494473428</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7491,18 +7516,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>HAPPYFORGE</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1662.9</v>
+        <v>1873.2</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1589.7</v>
+        <v>1706.09</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -7514,7 +7539,7 @@
         <v>5.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7406161820179997</v>
+        <v>0.7616087481946532</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7529,18 +7554,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SIRCA</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>430.2</v>
+        <v>45035</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>408.93</v>
+        <v>42685</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -7549,10 +7574,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7561462262749874</v>
+        <v>0.753727119992926</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7567,18 +7592,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>MINDACORP</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>657.15</v>
+        <v>1677.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>619.26</v>
+        <v>1603.67</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -7587,10 +7612,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7543570113167196</v>
+        <v>0.7386281575146639</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7605,18 +7630,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>405.2</v>
+        <v>2018.5</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>375.25</v>
+        <v>1918.77</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -7625,10 +7650,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7405370986425878</v>
+        <v>0.7435818079995284</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7643,18 +7668,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>NEULANDLAB</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>4554.1</v>
+        <v>19955</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>4311.26</v>
+        <v>18565.71</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -7666,7 +7691,7 @@
         <v>5.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7264520895832716</v>
+        <v>0.7324413446517523</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7681,18 +7706,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>PRICOLLTD</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1938</v>
+        <v>666.9</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1794.9</v>
+        <v>612.73</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -7701,10 +7726,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7347335669943862</v>
+        <v>0.7456841158958941</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7719,18 +7744,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>ANTHEM</t>
+          <t>UNIPARTS</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>847.75</v>
+        <v>718.2</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>792.26</v>
+        <v>654.85</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -7742,7 +7767,7 @@
         <v>5.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7304355897466361</v>
+        <v>0.7453694697438619</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7757,18 +7782,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261014</v>
+        <v>20261015</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>GPPL</t>
+          <t>DODLA</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>175.53</v>
+        <v>997.6</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>164.19</v>
+        <v>935.14</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -7777,10 +7802,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7282427896753497</v>
+        <v>0.7367284905827217</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-19
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 16 Oct 2026</t>
+          <t>As of Mon 19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹197,806</t>
+          <t>₹196,735</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+439  (+0.22%)</t>
+          <t>₹-1,071  (-0.54%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-1.10%</t>
+          <t>-1.63%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-4.02%</t>
+          <t>-4.54%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹108,535</t>
+          <t>₹99,392</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹85,533</t>
+          <t>₹94,656</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹89,271</t>
+          <t>₹97,343</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -693,7 +693,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9239</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>9144.5</v>
+        <v>9087</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9144.5</v>
+        <v>9087</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-94.5</v>
+        <v>-152</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.01022837969477216</v>
+        <v>-0.01645199696936898</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8902.93</v>
@@ -862,13 +862,13 @@
         <v>8902.93</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.02641697195035264</v>
+        <v>0.02025641025641023</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9126</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>772.1</v>
+        <v>760</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>10037.3</v>
+        <v>9880</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>911.3000000000003</v>
+        <v>754</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.0998575498575499</v>
+        <v>0.08262108262108261</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>683.88</v>
@@ -910,13 +910,13 @@
         <v>701.55</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.09137417432975012</v>
+        <v>0.07690789473684216</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>8970</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>840</v>
+        <v>814</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>10920</v>
+        <v>10582</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>1950</v>
+        <v>1612</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.2173913043478261</v>
+        <v>0.1797101449275362</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>627</v>
@@ -958,13 +958,13 @@
         <v>781.3285714285713</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.06984693877551035</v>
+        <v>0.04013689013689029</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>25.79</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>8910</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>800</v>
+        <v>794</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>8800</v>
+        <v>8734</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>-110</v>
+        <v>-176</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-0.01234567901234568</v>
+        <v>-0.01975308641975309</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>761.28</v>
@@ -1006,13 +1006,13 @@
         <v>761.28</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.04840000000000003</v>
+        <v>0.0412090680100756</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>23.57</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>7587.6</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1859.9</v>
+        <v>1843.7</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>7439.6</v>
+        <v>7374.8</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-148</v>
+        <v>-212.8000000000002</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.01950550898834941</v>
+        <v>-0.02804575886973485</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1777.36</v>
@@ -1054,13 +1054,13 @@
         <v>1777.36</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04437873003924953</v>
+        <v>0.03598199273200637</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>7866.4</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>2060.1</v>
+        <v>2069</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>8240.4</v>
+        <v>8276</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>374</v>
+        <v>409.6000000000004</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.04754398454184888</v>
+        <v>0.052069561680057</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1839.47</v>
@@ -1102,13 +1102,13 @@
         <v>1880.171428571428</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.08733972692032987</v>
+        <v>0.09126562176344691</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>4242</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>4473.4</v>
+        <v>4435.5</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4473.4</v>
+        <v>4435.5</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>231.3999999999996</v>
+        <v>193.5</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.05454974068835446</v>
+        <v>0.04561527581329562</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>3979.77</v>
@@ -1150,13 +1150,13 @@
         <v>4069.314285714286</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.09033078067816729</v>
+        <v>0.08255793355556619</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>126.65</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>5025</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>345</v>
+        <v>336.65</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5175</v>
+        <v>5049.75</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>150</v>
+        <v>24.74999999999966</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.02985074626865672</v>
+        <v>0.00492537313432829</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>306.13</v>
@@ -1198,13 +1198,13 @@
         <v>306.13</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1126666666666667</v>
+        <v>0.09065795336402788</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>4249.2</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>2152.7</v>
+        <v>2144.6</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4305.4</v>
+        <v>4289.2</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>56.19999999999982</v>
+        <v>40</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.01322601901534402</v>
+        <v>0.009413536665725314</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>1983.64</v>
@@ -1246,13 +1246,13 @@
         <v>1983.64</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.07853393412923293</v>
+        <v>0.07505362305324993</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4006</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1866</v>
+        <v>1866.8</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>3732</v>
+        <v>3733.6</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>-274</v>
+        <v>-272.4000000000001</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>-0.06839740389415876</v>
+        <v>-0.06799800299550676</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1842.51</v>
@@ -1294,13 +1294,13 @@
         <v>1842.51</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.01258842443729904</v>
+        <v>0.01301157060209983</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>79.15000000000001</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>3760</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1951.9</v>
+        <v>1925</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>3903.8</v>
+        <v>3850</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>143.8000000000002</v>
+        <v>90</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.03824468085106388</v>
+        <v>0.02393617021276596</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>1752.11</v>
@@ -1342,13 +1342,13 @@
         <v>1752.11</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.1023566781085097</v>
+        <v>0.08981298701298707</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>5306</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>418.15</v>
+        <v>404.2</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>5854.099999999999</v>
+        <v>5658.8</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>548.0999999999997</v>
+        <v>352.7999999999998</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.1032981530343007</v>
+        <v>0.06649076517150393</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>353.13</v>
@@ -1390,17 +1390,113 @@
         <v>357.65</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.1446849216788233</v>
+        <v>0.1151657595249875</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>SAILIFE</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1381</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>4143</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1395.9</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>4187.700000000001</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>44.70000000000027</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.01078928312816806</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1285.37</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>1285.37</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.07918188982018783</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>51.67</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>4980</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>4980</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>4959</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>4959</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>-21</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>-0.004216867469879518</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>4749.53</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>4749.53</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.04224037104254895</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>120.43</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H14">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -5036,7 +5132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7183,6 +7279,31 @@
       </c>
       <c r="G85" s="14" t="n">
         <v>13</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B86" s="20" t="n">
+        <v>196735.22</v>
+      </c>
+      <c r="C86" s="20" t="n">
+        <v>99392.27</v>
+      </c>
+      <c r="D86" s="20" t="n">
+        <v>97342.95</v>
+      </c>
+      <c r="E86" s="20" t="n">
+        <v>94655.8</v>
+      </c>
+      <c r="F86" s="20" t="n">
+        <v>-5804.15</v>
+      </c>
+      <c r="G86" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -7265,7 +7386,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -7273,10 +7394,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9144.5</v>
+        <v>9087</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8678.360000000001</v>
+        <v>8607.07</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -7285,10 +7406,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.860433821976895</v>
+        <v>0.8289897195168319</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7303,7 +7424,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -7311,10 +7432,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2060.1</v>
+        <v>2069</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1959.41</v>
+        <v>1966.99</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -7323,10 +7444,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8343445540373421</v>
+        <v>0.8110193471966307</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7341,18 +7462,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1389.4</v>
+        <v>1843.7</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1285.37</v>
+        <v>1703.66</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -7361,10 +7482,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8108779748439057</v>
+        <v>0.7867446842736394</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7379,18 +7500,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>SHYAMMETL</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1859.9</v>
+        <v>1226.6</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1718.43</v>
+        <v>1146.8</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -7399,10 +7520,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8014606521280125</v>
+        <v>0.7641082448597584</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7417,18 +7538,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>VIJAYA</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>4989</v>
+        <v>1368.2</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>4749.53</v>
+        <v>1274.5</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -7437,10 +7558,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.747941739812385</v>
+        <v>0.7672366265976427</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7455,18 +7576,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>772.1</v>
+        <v>1621.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>734.1799999999999</v>
+        <v>1541.79</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -7475,10 +7596,10 @@
         <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7462982233885319</v>
+        <v>0.7441750021935597</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7493,18 +7614,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>45560</v>
+        <v>814</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>43172.86</v>
+        <v>781.1</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -7513,10 +7634,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7737878170904593</v>
+        <v>0.751684653856278</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7531,18 +7652,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1198.5</v>
+        <v>158.15</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1124.64</v>
+        <v>148.56</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -7551,10 +7672,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7577655114167647</v>
+        <v>0.7334711620016964</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7569,18 +7690,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>CORONA</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2003.9</v>
+        <v>1324.1</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1873.53</v>
+        <v>1272.11</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -7592,7 +7713,7 @@
         <v>5.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7759271408319006</v>
+        <v>0.7410393085899798</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7607,18 +7728,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1666.9</v>
+        <v>1395.9</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1592.91</v>
+        <v>1292.56</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -7627,10 +7748,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7435993726057974</v>
+        <v>0.7434365037582989</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7645,18 +7766,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>VIJAYA</t>
+          <t>AKUMS</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1381.7</v>
+        <v>709.55</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1287.07</v>
+        <v>649.11</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -7665,10 +7786,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7565276898018279</v>
+        <v>0.7517658155654997</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7683,18 +7804,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>RAINBOW</t>
+          <t>ANTHEM</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1248.9</v>
+        <v>808.5</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1155.07</v>
+        <v>751.71</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -7703,10 +7824,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7430809429010949</v>
+        <v>0.7365871135678981</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7721,18 +7842,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>MEDANTA</t>
+          <t>EMCURE</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1240</v>
+        <v>1766.6</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1143.61</v>
+        <v>1648.66</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -7741,10 +7862,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7539630651826381</v>
+        <v>0.7492176303705653</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7759,18 +7880,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>QUESS</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>380.5</v>
+        <v>321.85</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>347.75</v>
+        <v>294.86</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -7782,7 +7903,7 @@
         <v>5.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7581553705547008</v>
+        <v>0.7340246702348572</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7797,18 +7918,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261016</v>
+        <v>20261019</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>HNDFDS</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>465.45</v>
+        <v>565.15</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>436.47</v>
+        <v>526.54</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -7817,10 +7938,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.738342306880222</v>
+        <v>0.7633872949021672</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-20
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
@@ -868,7 +868,7 @@
         <v>170.46</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         <v>13.22</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -964,7 +964,7 @@
         <v>25.79</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -1012,7 +1012,7 @@
         <v>23.57</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
@@ -1060,7 +1060,7 @@
         <v>56.89</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -1108,7 +1108,7 @@
         <v>55</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -1156,7 +1156,7 @@
         <v>126.65</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1204,7 +1204,7 @@
         <v>10.42</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -1252,7 +1252,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -1300,7 +1300,7 @@
         <v>79.15000000000001</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -1348,7 +1348,7 @@
         <v>57.73</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1396,7 +1396,7 @@
         <v>14.18</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1444,7 +1444,7 @@
         <v>51.67</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1492,7 +1492,7 @@
         <v>120.43</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-22
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 21 Oct 2026</t>
+          <t>As of Thu 22 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹195,157</t>
+          <t>₹194,990</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-1,578  (-0.80%)</t>
+          <t>₹-168  (-0.09%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-2.42%</t>
+          <t>-2.51%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-5.31%</t>
+          <t>-5.39%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹73,576</t>
+          <t>₹73,408</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9239</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>9190</v>
+        <v>9162</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9190</v>
+        <v>9162</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>-49</v>
+        <v>-77</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>-0.005303604286178158</v>
+        <v>-0.00833423530685139</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>8902.93</v>
@@ -862,13 +862,13 @@
         <v>8902.93</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.03123721436343849</v>
+        <v>0.02827657716655749</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>170.46</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>9126</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>753</v>
+        <v>782.3</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>9789</v>
+        <v>10169.9</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>663</v>
+        <v>1043.899999999999</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.07264957264957266</v>
+        <v>0.1143874643874643</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>683.88</v>
@@ -910,13 +910,13 @@
         <v>701.55</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.0683266932270917</v>
+        <v>0.1032212706122971</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>7587.6</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1836.1</v>
+        <v>1843.7</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>7344.4</v>
+        <v>7374.8</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>-243.2000000000007</v>
+        <v>-212.8000000000002</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>-0.03205229585112562</v>
+        <v>-0.02804575886973485</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1777.36</v>
@@ -958,13 +958,13 @@
         <v>1777.36</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.03199172158379174</v>
+        <v>0.03598199273200637</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>7866.4</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>2012.5</v>
+        <v>2002.5</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>8050</v>
+        <v>8010</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>183.6000000000004</v>
+        <v>143.6000000000004</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.02333977422963495</v>
+        <v>0.01825485609681689</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>1839.47</v>
@@ -1006,13 +1006,13 @@
         <v>1880.171428571428</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.06575332741792381</v>
+        <v>0.06108792580702704</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>4242</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>4356.1</v>
+        <v>4201.3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4356.1</v>
+        <v>4201.3</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>114.1000000000004</v>
+        <v>-40.69999999999982</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.02689768976897698</v>
+        <v>-0.009594530881659551</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>3979.77</v>
@@ -1054,13 +1054,13 @@
         <v>4069.314285714286</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.06583542946344532</v>
+        <v>0.03141544623942923</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>126.65</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>5025</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>329.7</v>
+        <v>321.9</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>4945.5</v>
+        <v>4828.5</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>-79.50000000000017</v>
+        <v>-196.5000000000003</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>-0.01582089552238809</v>
+        <v>-0.03910447761194037</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>306.13</v>
@@ -1102,13 +1102,13 @@
         <v>306.13</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07148923263572943</v>
+        <v>0.0489903696800248</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>4249.2</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2066.8</v>
+        <v>2052.4</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>4133.6</v>
+        <v>4104.8</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>-115.5999999999995</v>
+        <v>-144.3999999999996</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>-0.02720512096394603</v>
+        <v>-0.0339828673632683</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>1983.64</v>
@@ -1150,13 +1150,13 @@
         <v>1983.64</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.04023611379910977</v>
+        <v>0.03350224127850321</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>3760</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1951</v>
+        <v>1908.8</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>3902</v>
+        <v>3817.6</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>142</v>
+        <v>57.59999999999991</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.03776595744680851</v>
+        <v>0.01531914893617019</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1752.11</v>
@@ -1198,13 +1198,13 @@
         <v>1752.11</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1019425935417735</v>
+        <v>0.08208822296730933</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1228,31 +1228,31 @@
         <v>5306</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>398.9</v>
+        <v>387.95</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5584.599999999999</v>
+        <v>5431.3</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>278.5999999999997</v>
+        <v>125.2999999999998</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.05250659630606854</v>
+        <v>0.02361477572559364</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>353.13</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>357.7928571428572</v>
+        <v>358.0214285714286</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.1030512480750634</v>
+        <v>0.07714543479461629</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4143</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>1393.6</v>
+        <v>1395.9</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4180.799999999999</v>
+        <v>4187.700000000001</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>37.79999999999973</v>
+        <v>44.70000000000027</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.009123823316437298</v>
+        <v>0.01078928312816806</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1285.37</v>
@@ -1294,13 +1294,13 @@
         <v>1285.37</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.07766216991963262</v>
+        <v>0.07918188982018783</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>51.67</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4980</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>4854.4</v>
+        <v>4875</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>4854.4</v>
+        <v>4875</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>-125.6000000000004</v>
+        <v>-105</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>-0.02522088353413662</v>
+        <v>-0.02108433734939759</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>4749.53</v>
@@ -1342,13 +1342,13 @@
         <v>4749.53</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.02160308174027684</v>
+        <v>0.02573743589743595</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>120.43</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5117,7 +5117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7313,6 +7313,31 @@
         <v>-5548.18</v>
       </c>
       <c r="G87" s="14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B88" s="20" t="n">
+        <v>194989.58</v>
+      </c>
+      <c r="C88" s="20" t="n">
+        <v>121581.08</v>
+      </c>
+      <c r="D88" s="20" t="n">
+        <v>73408.5</v>
+      </c>
+      <c r="E88" s="20" t="n">
+        <v>72769.8</v>
+      </c>
+      <c r="F88" s="20" t="n">
+        <v>-5548.18</v>
+      </c>
+      <c r="G88" s="14" t="n">
         <v>12</v>
       </c>
     </row>
@@ -7396,7 +7421,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -7404,22 +7429,22 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9190</v>
+        <v>9162</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8706.860000000001</v>
+        <v>8685.5</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8446132278785596</v>
+        <v>0.8638766961440694</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7434,7 +7459,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -7442,22 +7467,22 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2012.5</v>
+        <v>2002.5</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1904.7</v>
+        <v>1892.31</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.780389387567217</v>
+        <v>0.8215473846264008</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7472,30 +7497,30 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>779.35</v>
+        <v>782.3</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>736.5599999999999</v>
+        <v>740.4</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.7806896407423682</v>
+        <v>0.7895948945615983</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7510,30 +7535,30 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>IPCALAB</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1918.9</v>
+        <v>1843.7</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1788.73</v>
+        <v>1715.53</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7862244470947629</v>
+        <v>0.8227315527550034</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7548,30 +7573,30 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>MEDANTA</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>1836.1</v>
+        <v>1198.2</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1694.29</v>
+        <v>1116.41</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>5.8</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7887070282258908</v>
+        <v>0.7878393183201461</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7586,30 +7611,30 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SHYAMMETL</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1195.6</v>
+        <v>1610.9</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1110.7</v>
+        <v>1523.4</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G7" s="14" t="n">
         <v>5.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7789749544912435</v>
+        <v>0.7635813254090438</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7624,30 +7649,30 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>COFORGE</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>1578.8</v>
+        <v>1908.8</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1492.06</v>
+        <v>1785.07</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G8" s="14" t="n">
         <v>5.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7634627455903584</v>
+        <v>0.7360545630303248</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7662,30 +7687,30 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>PETRONET</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>295</v>
+        <v>4201.3</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>283.24</v>
+        <v>3925.69</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G9" s="14" t="n">
         <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7715863201724101</v>
+        <v>0.7518338047330922</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7700,30 +7725,30 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>HNDFDS</t>
+          <t>HYUNDAI</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>554.15</v>
+        <v>1895.5</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>515.77</v>
+        <v>1791.27</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7936052350762663</v>
+        <v>0.751942644373635</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7738,7 +7763,7 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
@@ -7746,22 +7771,22 @@
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>3023.3</v>
+        <v>2987</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>2825.71</v>
+        <v>2778.33</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>5.6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7624678300169481</v>
+        <v>0.7506852601052594</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7776,30 +7801,30 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1393.6</v>
+        <v>1903.5</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1291.11</v>
+        <v>1773.43</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>5.6</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7596588412529032</v>
+        <v>0.7590254555869822</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7814,30 +7839,30 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>NEULANDLAB</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>18975</v>
+        <v>788.85</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>17567.86</v>
+        <v>742.46</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G13" s="14" t="n">
         <v>5.6</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7497578097210889</v>
+        <v>0.7371349038702517</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7852,30 +7877,30 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>EMCURE</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>143.19</v>
+        <v>1782.6</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>132.58</v>
+        <v>1662.5</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7606835729081665</v>
+        <v>0.7596213884214671</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7890,30 +7915,30 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>GUFICBIO</t>
+          <t>VADILALIND</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>389.5</v>
+        <v>7207.5</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>353.24</v>
+        <v>6819.79</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>5333</v>
+        <v>5337</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7496490071767832</v>
+        <v>0.7388548566109341</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7928,30 +7953,30 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261021</v>
+        <v>20261022</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>SUPRAJIT</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>463.15</v>
+        <v>349.05</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>435.79</v>
+        <v>313.81</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0264</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>5333</v>
+        <v>5287</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7562122068085284</v>
+        <v>0.7360921556693281</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-26
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Fri 23 Oct 2026</t>
+          <t>As of Mon 26 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹194,376</t>
+          <t>₹195,810</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-613  (-0.31%)</t>
+          <t>₹+1,434  (+0.74%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-2.81%</t>
+          <t>-2.09%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-5.69%</t>
+          <t>-4.99%</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>₹139,261</t>
+          <t>₹111,139</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>₹54,309</t>
+          <t>₹82,370</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹55,115</t>
+          <t>₹84,671</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>9126</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>781.75</v>
+        <v>795.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>10162.75</v>
+        <v>10341.5</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>1036.75</v>
+        <v>1215.5</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1136039886039886</v>
+        <v>0.1331908831908832</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>683.88</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>701.55</v>
+        <v>704.1285714285714</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.1025903421810042</v>
+        <v>0.1148603753254917</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>7587.6</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1838.2</v>
+        <v>1855.6</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>7352.8</v>
+        <v>7422.4</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-234.8000000000002</v>
+        <v>-165.2000000000007</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.03094522642205706</v>
+        <v>-0.02177236543834687</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1777.36</v>
@@ -910,13 +910,13 @@
         <v>1777.36</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.03309759547383317</v>
+        <v>0.04216425953869369</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -940,16 +940,16 @@
         <v>7866.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1970</v>
+        <v>2058.9</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>7880</v>
+        <v>8235.6</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>13.60000000000036</v>
+        <v>369.2000000000007</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.001728872165158187</v>
+        <v>0.0469337943659108</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1839.47</v>
@@ -958,13 +958,13 @@
         <v>1880.171428571428</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.045598259608412</v>
+        <v>0.08680779611859329</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>5025</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>319.3</v>
+        <v>329.85</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4789.5</v>
+        <v>4947.75</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>-235.4999999999998</v>
+        <v>-77.24999999999966</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-0.04686567164179101</v>
+        <v>-0.01537313432835814</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>306.13</v>
@@ -1006,13 +1006,13 @@
         <v>306.13</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.04124647666771067</v>
+        <v>0.07191147491283925</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>4249.2</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>2033.7</v>
+        <v>2077.9</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4067.4</v>
+        <v>4155.8</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-181.7999999999997</v>
+        <v>-93.39999999999964</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.04278452414572149</v>
+        <v>-0.02198060811446852</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1983.64</v>
@@ -1054,13 +1054,13 @@
         <v>1983.64</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.02461523331858187</v>
+        <v>0.04536310698301169</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>3760</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1900.5</v>
+        <v>1993</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3801</v>
+        <v>3986</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>41</v>
+        <v>226</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.01090425531914894</v>
+        <v>0.0601063829787234</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1752.11</v>
@@ -1102,13 +1102,13 @@
         <v>1752.11</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.07807945277558542</v>
+        <v>0.1208680381334672</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5306</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>402.15</v>
+        <v>400.25</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5630.099999999999</v>
+        <v>5603.5</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>324.0999999999997</v>
+        <v>297.5</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.0610817941952506</v>
+        <v>0.05606860158311346</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>353.13</v>
@@ -1150,13 +1150,13 @@
         <v>358.0214285714286</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.1097316211079731</v>
+        <v>0.1055054876416525</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>4143</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1395.3</v>
+        <v>1445.3</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4185.9</v>
+        <v>4335.9</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>42.89999999999986</v>
+        <v>192.8999999999999</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.01035481535119475</v>
+        <v>0.0465604634322954</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1285.37</v>
@@ -1198,17 +1198,305 @@
         <v>1285.37</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.07878592417401281</v>
+        <v>0.1106552272884523</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>51.67</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>RADICO</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>4150</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>4150</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>4200</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>0.01204819277108434</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>3879.27</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>3879.27</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.07636428571428572</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>144.81</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>VARROC</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>764.25</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>4585.5</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>778.55</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>4671.299999999999</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>85.79999999999973</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>0.01871115472685634</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>710.29</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>710.29</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0.0876758075910346</v>
+      </c>
+      <c r="M12" s="13" t="n">
+        <v>27.71</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>INDIGOPNTS</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>996.9</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>4984.5</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>5109</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>124.4999999999999</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0.0249774300331026</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>949</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>949</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.07124681933842235</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>32.99</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>LGBBROSLTD</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1640</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>4920</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1664.4</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>4993.200000000001</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>73.20000000000027</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>0.01487804878048786</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>1536.33</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>1536.33</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.0769466474405192</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>54.19</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>EMCURE</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1773.2</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>5319.6</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1780.2</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>5340.6</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>0.003947665237987818</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1647.97</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>1647.97</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.07427817099202337</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>60.79</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>CORONA</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>2051</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>4102</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>2041.4</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>4082.8</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>-19.19999999999982</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>-0.004680643588493374</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>1942.67</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>1942.67</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.04836386793377095</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>53.81</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:H10">
+  <conditionalFormatting sqref="H2:H16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -5102,7 +5390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7349,6 +7637,31 @@
       </c>
       <c r="G89" s="14" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B90" s="20" t="n">
+        <v>195810.39</v>
+      </c>
+      <c r="C90" s="20" t="n">
+        <v>111139.44</v>
+      </c>
+      <c r="D90" s="20" t="n">
+        <v>84670.95</v>
+      </c>
+      <c r="E90" s="20" t="n">
+        <v>82370.39999999999</v>
+      </c>
+      <c r="F90" s="20" t="n">
+        <v>-6348.9</v>
+      </c>
+      <c r="G90" s="14" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -7431,7 +7744,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -7439,10 +7752,10 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1970</v>
+        <v>2058.9</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1856.77</v>
+        <v>1937.04</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -7451,10 +7764,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.808113296042803</v>
+        <v>0.8312095528754229</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7469,7 +7782,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -7477,10 +7790,10 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>8950</v>
+        <v>9050</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8453.709999999999</v>
+        <v>8546.860000000001</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -7489,10 +7802,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.7814082965639441</v>
+        <v>0.8302333063685836</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7507,18 +7820,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1395.3</v>
+        <v>1855.6</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1298.87</v>
+        <v>1732.4</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -7527,10 +7840,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8007990827919258</v>
+        <v>0.8331795116928959</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7545,7 +7858,7 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
@@ -7553,10 +7866,10 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>4157.3</v>
+        <v>4200</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>3879.27</v>
+        <v>3910.37</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -7565,10 +7878,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7851665913907515</v>
+        <v>0.7965858949845566</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7583,18 +7896,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>781.75</v>
+        <v>781.9</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>738.58</v>
+        <v>732.63</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -7606,7 +7919,7 @@
         <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.760060626063996</v>
+        <v>0.7762667304015296</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7621,18 +7934,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>COFORGE</t>
+          <t>ZYDUSLIFE</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1900.5</v>
+        <v>1160.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1773.84</v>
+        <v>1094.91</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -7644,7 +7957,7 @@
         <v>5.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7366779001493937</v>
+        <v>0.7599279305780262</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7659,18 +7972,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>402.15</v>
+        <v>811.5</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>371.24</v>
+        <v>760.01</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -7682,7 +7995,7 @@
         <v>5.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7620070875169371</v>
+        <v>0.7534904030004412</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -7697,18 +8010,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>VARROC</t>
+          <t>HAPPYFORGE</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>764.25</v>
+        <v>1758.4</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>710.29</v>
+        <v>1608.14</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -7717,10 +8030,10 @@
         <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7586370426988153</v>
+        <v>0.7753116267098102</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -7735,18 +8048,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>INDIGOPNTS</t>
+          <t>SOMANYCERA</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1013.9</v>
+        <v>554.15</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>949</v>
+        <v>503.24</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -7755,10 +8068,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7628973699753328</v>
+        <v>0.781791439917635</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -7773,18 +8086,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>LGBBROSLTD</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1644.2</v>
+        <v>1048.8</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1536.33</v>
+        <v>967.87</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -7793,10 +8106,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7562345829135253</v>
+        <v>0.7718910869245478</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7811,18 +8124,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>VADILALIND</t>
+          <t>EMCURE</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>6958</v>
+        <v>1780.2</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>6555.36</v>
+        <v>1658.63</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -7831,10 +8144,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7550229302018553</v>
+        <v>0.7516620091189881</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7849,18 +8162,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>EMCURE</t>
+          <t>CONCORDBIO</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1770.4</v>
+        <v>1311.2</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1647.97</v>
+        <v>1215.29</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -7869,10 +8182,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7336544140638571</v>
+        <v>0.7502031548757171</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -7887,18 +8200,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>CORONA</t>
+          <t>INDGN</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>2051.1</v>
+        <v>601.75</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>1942.67</v>
+        <v>561.33</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -7907,10 +8220,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7353958934093041</v>
+        <v>0.747824128548316</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -7925,18 +8238,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>UTIAMC</t>
+          <t>GUFICBIO</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>817.05</v>
+        <v>407.35</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>776.65</v>
+        <v>372.55</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -7948,7 +8261,7 @@
         <v>5.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7268769759927735</v>
+        <v>0.7515553757905574</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -7963,18 +8276,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261023</v>
+        <v>20261026</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>DHARMAJ</t>
+          <t>VADILALIND</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>239.2</v>
+        <v>6879</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>222.47</v>
+        <v>6470.43</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -7983,10 +8296,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.1</v>
+        <v>5.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7273694541917104</v>
+        <v>0.7491303868215915</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-27
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Mon 26 Oct 2026</t>
+          <t>As of Tue 27 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹195,810</t>
+          <t>₹198,149</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+1,434  (+0.74%)</t>
+          <t>₹+2,338  (+1.19%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-2.09%</t>
+          <t>-0.93%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-4.99%</t>
+          <t>-3.86%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹84,671</t>
+          <t>₹87,009</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>9126</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>795.5</v>
+        <v>812.85</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>10341.5</v>
+        <v>10567.05</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>1215.5</v>
+        <v>1441.05</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1331908831908832</v>
+        <v>0.1579059829059829</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>683.88</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>704.1285714285714</v>
+        <v>719.4642857142858</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.1148603753254917</v>
+        <v>0.114886774048981</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>7587.6</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1855.6</v>
+        <v>1901.8</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>7422.4</v>
+        <v>7607.2</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>-165.2000000000007</v>
+        <v>19.59999999999945</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>-0.02177236543834687</v>
+        <v>0.002583162001159715</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1777.36</v>
@@ -910,13 +910,13 @@
         <v>1777.36</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.04216425953869369</v>
+        <v>0.06543274792302033</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>7866.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2058.9</v>
+        <v>2142</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8235.6</v>
+        <v>8568</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>369.2000000000007</v>
+        <v>701.6000000000004</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.0469337943659108</v>
+        <v>0.08918946404962885</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1839.47</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1880.171428571428</v>
+        <v>1901.914285714286</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.08680779611859329</v>
+        <v>0.1120848339335734</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>5025</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>329.85</v>
+        <v>339.4</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>4947.75</v>
+        <v>5091</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>-77.24999999999966</v>
+        <v>65.99999999999966</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-0.01537313432835814</v>
+        <v>0.01313432835820889</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>306.13</v>
@@ -1006,13 +1006,13 @@
         <v>306.13</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.07191147491283925</v>
+        <v>0.09802592810842659</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>4249.2</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>2077.9</v>
+        <v>2213.9</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4155.8</v>
+        <v>4427.8</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>-93.39999999999964</v>
+        <v>178.6000000000004</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-0.02198060811446852</v>
+        <v>0.04203144121246361</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1983.64</v>
@@ -1054,13 +1054,13 @@
         <v>1983.64</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.04536310698301169</v>
+        <v>0.1040065043588238</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>3760</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1993</v>
+        <v>1997</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3986</v>
+        <v>3994</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.0601063829787234</v>
+        <v>0.06223404255319149</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1752.11</v>
@@ -1102,13 +1102,13 @@
         <v>1752.11</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.1208680381334672</v>
+        <v>0.1226289434151227</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5306</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>400.25</v>
+        <v>401.3</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5603.5</v>
+        <v>5618.2</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>297.5</v>
+        <v>312.2000000000002</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.05606860158311346</v>
+        <v>0.05883905013192615</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>353.13</v>
@@ -1150,13 +1150,13 @@
         <v>358.0214285714286</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.1055054876416525</v>
+        <v>0.1078459293011996</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4143</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1445.3</v>
+        <v>1486.2</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4335.9</v>
+        <v>4458.6</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>192.8999999999999</v>
+        <v>315.6000000000001</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.0465604634322954</v>
+        <v>0.07617668356263581</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1285.37</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1285.37</v>
+        <v>1293.628571428572</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1106552272884523</v>
+        <v>0.1295730242036257</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>51.67</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>4150</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4200</v>
+        <v>4290</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4200</v>
+        <v>4290</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.01204819277108434</v>
+        <v>0.03373493975903614</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>3879.27</v>
@@ -1246,13 +1246,13 @@
         <v>3879.27</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.07636428571428572</v>
+        <v>0.09574125874125874</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>144.81</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4585.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>778.55</v>
+        <v>805.45</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4671.299999999999</v>
+        <v>4832.700000000001</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>85.79999999999973</v>
+        <v>247.2000000000003</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.01871115472685634</v>
+        <v>0.05390906117108282</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>710.29</v>
@@ -1294,13 +1294,13 @@
         <v>710.29</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.0876758075910346</v>
+        <v>0.1181451362592341</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>27.71</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4984.5</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1021.8</v>
+        <v>1027.3</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5109</v>
+        <v>5136.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>124.4999999999999</v>
+        <v>151.9999999999999</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.0249774300331026</v>
+        <v>0.03049453305246261</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>949</v>
@@ -1342,13 +1342,13 @@
         <v>949</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.07124681933842235</v>
+        <v>0.07621921541905963</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>32.99</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4920</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1664.4</v>
+        <v>1747.7</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4993.200000000001</v>
+        <v>5243.1</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>73.20000000000027</v>
+        <v>323.1000000000001</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.01487804878048786</v>
+        <v>0.0656707317073171</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1536.33</v>
@@ -1390,13 +1390,13 @@
         <v>1536.33</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.0769466474405192</v>
+        <v>0.1209418092349946</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>54.19</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>5319.6</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1780.2</v>
+        <v>1875.2</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>5340.6</v>
+        <v>5625.6</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>21</v>
+        <v>306</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.003947665237987818</v>
+        <v>0.05752312203925107</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1647.97</v>
@@ -1438,13 +1438,13 @@
         <v>1647.97</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.07427817099202337</v>
+        <v>0.1211764078498294</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>60.79</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>4102</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2041.4</v>
+        <v>2152</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>4082.8</v>
+        <v>4304</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>-19.19999999999982</v>
+        <v>202</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>-0.004680643588493374</v>
+        <v>0.0492442710872745</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1942.67</v>
@@ -1486,13 +1486,13 @@
         <v>1942.67</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.04836386793377095</v>
+        <v>0.09727230483271372</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>53.81</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5390,7 +5390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7661,6 +7661,31 @@
         <v>-6348.9</v>
       </c>
       <c r="G90" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B91" s="20" t="n">
+        <v>198148.79</v>
+      </c>
+      <c r="C91" s="20" t="n">
+        <v>111139.44</v>
+      </c>
+      <c r="D91" s="20" t="n">
+        <v>87009.35000000001</v>
+      </c>
+      <c r="E91" s="20" t="n">
+        <v>82370.39999999999</v>
+      </c>
+      <c r="F91" s="20" t="n">
+        <v>-6348.9</v>
+      </c>
+      <c r="G91" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7744,30 +7769,30 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2058.9</v>
+        <v>9505.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1937.04</v>
+        <v>8993.360000000001</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8312095528754229</v>
+        <v>0.8434516523867809</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7782,30 +7807,30 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>9050</v>
+        <v>2142</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>8546.860000000001</v>
+        <v>2021.96</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8302333063685836</v>
+        <v>0.8422055623555011</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7820,30 +7845,30 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1855.6</v>
+        <v>4290</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1732.4</v>
+        <v>4007.34</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8331795116928959</v>
+        <v>0.8104583163334693</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7858,30 +7883,30 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>4200</v>
+        <v>45600</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>3910.37</v>
+        <v>43593.57</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7965858949845566</v>
+        <v>0.8192166462668298</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7896,7 +7921,7 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
@@ -7904,22 +7929,22 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>781.9</v>
+        <v>851.85</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>732.63</v>
+        <v>794.34</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7762667304015296</v>
+        <v>0.7666995330704022</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7934,30 +7959,30 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>ZYDUSLIFE</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1160.4</v>
+        <v>1350</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1094.91</v>
+        <v>1292.73</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7599279305780262</v>
+        <v>0.7588217960922979</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7972,30 +7997,30 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>811.5</v>
+        <v>401.3</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>760.01</v>
+        <v>369.19</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7534904030004412</v>
+        <v>0.7952304048234282</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -8010,30 +8035,30 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>HAPPYFORGE</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1758.4</v>
+        <v>1901.8</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1608.14</v>
+        <v>1775.77</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7753116267098102</v>
+        <v>0.7909555056892879</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -8048,30 +8073,30 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SOMANYCERA</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>554.15</v>
+        <v>1059.9</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>503.24</v>
+        <v>981.67</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.781791439917635</v>
+        <v>0.817645292170996</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -8086,30 +8111,30 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1048.8</v>
+        <v>1627.5</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>967.87</v>
+        <v>1533.83</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7718910869245478</v>
+        <v>0.7772683485198785</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -8124,30 +8149,30 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>EMCURE</t>
+          <t>INDGN</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1780.2</v>
+        <v>599.95</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1658.63</v>
+        <v>558.58</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7516620091189881</v>
+        <v>0.7760800580262024</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -8162,30 +8187,30 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>CONCORDBIO</t>
+          <t>APLAPOLLO</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1311.2</v>
+        <v>2213.9</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1215.29</v>
+        <v>2081.76</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7502031548757171</v>
+        <v>0.7371900358130468</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -8200,30 +8225,30 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>INDGN</t>
+          <t>VARROC</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>601.75</v>
+        <v>805.45</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>561.33</v>
+        <v>748.54</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>5.5</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.747824128548316</v>
+        <v>0.7556122217688925</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -8238,30 +8263,30 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>GUFICBIO</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>407.35</v>
+        <v>364.1</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>372.55</v>
+        <v>322.85</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0237</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>5333</v>
+        <v>4745</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7515553757905574</v>
+        <v>0.7390033546398296</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -8276,30 +8301,30 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261026</v>
+        <v>20261027</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>VADILALIND</t>
+          <t>AARTIDRUGS</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>6879</v>
+        <v>402.25</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>6470.43</v>
+        <v>374.22</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0267</v>
+        <v>0.0269</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>5333</v>
+        <v>5375</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>5.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7491303868215915</v>
+        <v>0.737078403372773</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-28
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Tue 27 Oct 2026</t>
+          <t>As of Wed 28 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹198,149</t>
+          <t>₹197,797</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+2,338  (+1.19%)</t>
+          <t>₹-352  (-0.18%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-0.93%</t>
+          <t>-1.10%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-3.86%</t>
+          <t>-4.03%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹87,009</t>
+          <t>₹86,657</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>9126</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>812.85</v>
+        <v>805.2</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>10567.05</v>
+        <v>10467.6</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>1441.05</v>
+        <v>1341.600000000001</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1579059829059829</v>
+        <v>0.1470085470085471</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>683.88</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>719.4642857142858</v>
+        <v>719.6642857142857</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.114886774048981</v>
+        <v>0.106229153360301</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>7587.6</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1901.8</v>
+        <v>1922.3</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>7607.2</v>
+        <v>7689.2</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>19.59999999999945</v>
+        <v>101.5999999999995</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.002583162001159715</v>
+        <v>0.0133902683325425</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1777.36</v>
@@ -910,13 +910,13 @@
         <v>1777.36</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.06543274792302033</v>
+        <v>0.07539926130156586</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>7866.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2142</v>
+        <v>2181.9</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8568</v>
+        <v>8727.6</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>701.6000000000004</v>
+        <v>861.2000000000007</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.08918946404962885</v>
+        <v>0.109478287399573</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1839.47</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1901.914285714286</v>
+        <v>1931.1</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.1120848339335734</v>
+        <v>0.1149456895366423</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -988,16 +988,16 @@
         <v>5025</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>339.4</v>
+        <v>342.5</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5091</v>
+        <v>5137.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>65.99999999999966</v>
+        <v>112.5</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.01313432835820889</v>
+        <v>0.02238805970149254</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>306.13</v>
@@ -1006,13 +1006,13 @@
         <v>306.13</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.09802592810842659</v>
+        <v>0.1061897810218978</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>4249.2</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>2213.9</v>
+        <v>2165.3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4427.8</v>
+        <v>4330.6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>178.6000000000004</v>
+        <v>81.40000000000055</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.04203144121246361</v>
+        <v>0.01915654711475114</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1983.64</v>
@@ -1054,13 +1054,13 @@
         <v>1983.64</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.1040065043588238</v>
+        <v>0.08389599593589805</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>3760</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1997</v>
+        <v>1961.9</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3994</v>
+        <v>3923.8</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>234</v>
+        <v>163.8000000000002</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.06223404255319149</v>
+        <v>0.04356382978723409</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1752.11</v>
@@ -1102,13 +1102,13 @@
         <v>1752.11</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.1226289434151227</v>
+        <v>0.1069320556603294</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5306</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>401.3</v>
+        <v>400</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5618.2</v>
+        <v>5600</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>312.2000000000002</v>
+        <v>294</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.05883905013192615</v>
+        <v>0.0554089709762533</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>353.13</v>
@@ -1150,13 +1150,13 @@
         <v>358.0214285714286</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.1078459293011996</v>
+        <v>0.1049464285714285</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1180,16 +1180,16 @@
         <v>4143</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1486.2</v>
+        <v>1487.2</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4458.6</v>
+        <v>4461.6</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>315.6000000000001</v>
+        <v>318.6000000000001</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.07617668356263581</v>
+        <v>0.07690079652425781</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1285.37</v>
@@ -1198,13 +1198,13 @@
         <v>1293.628571428572</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1295730242036257</v>
+        <v>0.1301583032352262</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>51.67</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>4150</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4290</v>
+        <v>4135.1</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4290</v>
+        <v>4135.1</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>140</v>
+        <v>-14.89999999999964</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.03373493975903614</v>
+        <v>-0.003590361445783045</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>3879.27</v>
@@ -1246,13 +1246,13 @@
         <v>3879.27</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.09574125874125874</v>
+        <v>0.06186791129597842</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>144.81</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4585.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>805.45</v>
+        <v>807.5</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4832.700000000001</v>
+        <v>4845</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>247.2000000000003</v>
+        <v>259.5</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.05390906117108282</v>
+        <v>0.05659142950605169</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>710.29</v>
@@ -1294,13 +1294,13 @@
         <v>710.29</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.1181451362592341</v>
+        <v>0.1203839009287926</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>27.71</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4984.5</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1027.3</v>
+        <v>1012.9</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5136.5</v>
+        <v>5064.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>151.9999999999999</v>
+        <v>80</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.03049453305246261</v>
+        <v>0.01604975423813823</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>949</v>
@@ -1342,13 +1342,13 @@
         <v>949</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.07621921541905963</v>
+        <v>0.06308618817257378</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>32.99</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4920</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1747.7</v>
+        <v>1667.6</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>5243.1</v>
+        <v>5002.799999999999</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>323.1000000000001</v>
+        <v>82.79999999999973</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.0656707317073171</v>
+        <v>0.01682926829268287</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1536.33</v>
@@ -1390,13 +1390,13 @@
         <v>1536.33</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.1209418092349946</v>
+        <v>0.07871791796593906</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>54.19</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>5319.6</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1875.2</v>
+        <v>1875</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>5625.6</v>
+        <v>5625</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>306</v>
+        <v>305.3999999999999</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.05752312203925107</v>
+        <v>0.05741033160387996</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1647.97</v>
@@ -1438,13 +1438,13 @@
         <v>1647.97</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.1211764078498294</v>
+        <v>0.1210826666666667</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>60.79</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>4102</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2152</v>
+        <v>2200.6</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>4304</v>
+        <v>4401.2</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>202</v>
+        <v>299.1999999999998</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.0492442710872745</v>
+        <v>0.07294002925402239</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1942.67</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>1942.67</v>
+        <v>1953.428571428571</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.09727230483271372</v>
+        <v>0.1123200166188442</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>53.81</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5390,7 +5390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7686,6 +7686,31 @@
         <v>-6348.9</v>
       </c>
       <c r="G91" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B92" s="20" t="n">
+        <v>197796.54</v>
+      </c>
+      <c r="C92" s="20" t="n">
+        <v>111139.44</v>
+      </c>
+      <c r="D92" s="20" t="n">
+        <v>86657.10000000001</v>
+      </c>
+      <c r="E92" s="20" t="n">
+        <v>82370.39999999999</v>
+      </c>
+      <c r="F92" s="20" t="n">
+        <v>-6348.9</v>
+      </c>
+      <c r="G92" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7769,7 +7794,7 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -7777,22 +7802,22 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9505.5</v>
+        <v>9558.5</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>8993.360000000001</v>
+        <v>9023</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8434516523867809</v>
+        <v>0.836168918096629</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7807,7 +7832,7 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
@@ -7815,22 +7840,22 @@
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2142</v>
+        <v>2181.9</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>2021.96</v>
+        <v>2056.5</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8422055623555011</v>
+        <v>0.8092734574662285</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7845,30 +7870,30 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>4290</v>
+        <v>47625</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>4007.34</v>
+        <v>45412.14</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8104583163334693</v>
+        <v>0.8209748083242059</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7883,30 +7908,30 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>45600</v>
+        <v>11014</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>43593.57</v>
+        <v>10124.14</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.8192166462668298</v>
+        <v>0.7822775952294024</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7921,30 +7946,30 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>851.85</v>
+        <v>4135.1</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>794.34</v>
+        <v>3841.43</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7666995330704022</v>
+        <v>0.7718540829986613</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7959,30 +7984,30 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>1350</v>
+        <v>840.3</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1292.73</v>
+        <v>786.79</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7588217960922979</v>
+        <v>0.7676250456370939</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -7997,30 +8022,30 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>SONACOMS</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>401.3</v>
+        <v>879.45</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>369.19</v>
+        <v>819.54</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7952304048234282</v>
+        <v>0.752354874041621</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -8035,30 +8060,30 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1901.8</v>
+        <v>1487.2</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1775.77</v>
+        <v>1389.76</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7909555056892879</v>
+        <v>0.7730497748570038</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -8073,30 +8098,30 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>HYUNDAI</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1059.9</v>
+        <v>1866.9</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>981.67</v>
+        <v>1756.89</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.817645292170996</v>
+        <v>0.7296914932457101</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -8111,30 +8136,30 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>SIRCA</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1627.5</v>
+        <v>413.5</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1533.83</v>
+        <v>389.69</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7772683485198785</v>
+        <v>0.7393270049896555</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -8149,7 +8174,7 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
@@ -8157,22 +8182,22 @@
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>599.95</v>
+        <v>598.95</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>558.58</v>
+        <v>559.5</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.7</v>
+        <v>5.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7760800580262024</v>
+        <v>0.7552847754654984</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -8187,30 +8212,30 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>APLAPOLLO</t>
+          <t>VARROC</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2213.9</v>
+        <v>807.5</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2081.76</v>
+        <v>749.1</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.7</v>
+        <v>5.4</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7371900358130468</v>
+        <v>0.7466745770962638</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -8225,30 +8250,30 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>VARROC</t>
+          <t>SOMANYCERA</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>805.45</v>
+        <v>543.8</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>748.54</v>
+        <v>494.03</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7556122217688925</v>
+        <v>0.7637337227698674</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -8263,30 +8288,30 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>364.1</v>
+        <v>1080.2</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>322.85</v>
+        <v>1004.9</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0.0237</v>
+        <v>0.0267</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>4745</v>
+        <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7390033546398296</v>
+        <v>0.7378270658391139</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -8301,30 +8326,30 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261027</v>
+        <v>20261028</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>AARTIDRUGS</t>
+          <t>VADILALIND</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>402.25</v>
+        <v>7342</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>374.22</v>
+        <v>6894.07</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.0269</v>
+        <v>0.0267</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>5375</v>
+        <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.737078403372773</v>
+        <v>0.7232688329073871</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-29
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Wed 28 Oct 2026</t>
+          <t>As of Thu 29 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹197,797</t>
+          <t>₹198,496</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹-352  (-0.18%)</t>
+          <t>₹+700  (+0.35%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-1.10%</t>
+          <t>-0.75%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-4.03%</t>
+          <t>-3.69%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹86,657</t>
+          <t>₹87,357</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3">
@@ -844,31 +844,31 @@
         <v>9126</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>805.2</v>
+        <v>810</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>10467.6</v>
+        <v>10530</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>1341.600000000001</v>
+        <v>1404</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1470085470085471</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>683.88</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>719.6642857142857</v>
+        <v>722.4071428571428</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.106229153360301</v>
+        <v>0.1081393298059965</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>7587.6</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1922.3</v>
+        <v>1911.7</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>7689.2</v>
+        <v>7646.8</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>101.5999999999995</v>
+        <v>59.19999999999982</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.0133902683325425</v>
+        <v>0.007802203595339741</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1777.36</v>
@@ -910,13 +910,13 @@
         <v>1777.36</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.07539926130156586</v>
+        <v>0.07027253230109334</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>7866.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2181.9</v>
+        <v>2244</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8727.6</v>
+        <v>8976</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>861.2000000000007</v>
+        <v>1109.6</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.109478287399573</v>
+        <v>0.1410556290043731</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1839.47</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1931.1</v>
+        <v>1987.228571428571</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.1149456895366423</v>
+        <v>0.1144257703081233</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>5025</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>342.5</v>
+        <v>352.9</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5137.5</v>
+        <v>5293.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>112.5</v>
+        <v>268.4999999999997</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.02238805970149254</v>
+        <v>0.05343283582089545</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>306.13</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>306.13</v>
+        <v>308.6428571428572</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.1061897810218978</v>
+        <v>0.1254098692466501</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>4249.2</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>2165.3</v>
+        <v>2195</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4330.6</v>
+        <v>4390</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>81.40000000000055</v>
+        <v>140.8000000000002</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.01915654711475114</v>
+        <v>0.03313564906335315</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1983.64</v>
@@ -1054,13 +1054,13 @@
         <v>1983.64</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.08389599593589805</v>
+        <v>0.09629157175398628</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>3760</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1961.9</v>
+        <v>1962</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3923.8</v>
+        <v>3924</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>163.8000000000002</v>
+        <v>164</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.04356382978723409</v>
+        <v>0.04361702127659575</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1752.11</v>
@@ -1102,13 +1102,13 @@
         <v>1752.11</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.1069320556603294</v>
+        <v>0.1069775739041795</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5306</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>400</v>
+        <v>405.4</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5600</v>
+        <v>5675.599999999999</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>294</v>
+        <v>369.5999999999997</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.0554089709762533</v>
+        <v>0.06965699208443266</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>353.13</v>
@@ -1150,13 +1150,13 @@
         <v>358.0214285714286</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.1049464285714285</v>
+        <v>0.1168687011064908</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4143</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1487.2</v>
+        <v>1495.7</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4461.6</v>
+        <v>4487.1</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>318.6000000000001</v>
+        <v>344.1000000000001</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.07690079652425781</v>
+        <v>0.08305575669804492</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1285.37</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1293.628571428572</v>
+        <v>1310.214285714286</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1301583032352262</v>
+        <v>0.1240126457750313</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>51.67</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>4150</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4135.1</v>
+        <v>4235</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4135.1</v>
+        <v>4235</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>-14.89999999999964</v>
+        <v>85</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>-0.003590361445783045</v>
+        <v>0.02048192771084337</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>3879.27</v>
@@ -1246,13 +1246,13 @@
         <v>3879.27</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.06186791129597842</v>
+        <v>0.08399763872491145</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>144.81</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4585.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>807.5</v>
+        <v>804.4</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4845</v>
+        <v>4826.4</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>259.5</v>
+        <v>240.8999999999999</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.05659142950605169</v>
+        <v>0.05253516519463523</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>710.29</v>
@@ -1294,13 +1294,13 @@
         <v>710.29</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.1203839009287926</v>
+        <v>0.1169940328194928</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>27.71</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4984.5</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1012.9</v>
+        <v>1011.8</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5064.5</v>
+        <v>5059</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>80</v>
+        <v>74.49999999999989</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.01604975423813823</v>
+        <v>0.0149463336342662</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>949</v>
@@ -1342,13 +1342,13 @@
         <v>949</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.06308618817257378</v>
+        <v>0.06206760229294322</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>32.99</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4920</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1667.6</v>
+        <v>1679.4</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>5002.799999999999</v>
+        <v>5038.200000000001</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>82.79999999999973</v>
+        <v>118.2000000000003</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.01682926829268287</v>
+        <v>0.0240243902439025</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1536.33</v>
@@ -1390,13 +1390,13 @@
         <v>1536.33</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.07871791796593906</v>
+        <v>0.0851911396927475</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>54.19</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>5319.6</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1875</v>
+        <v>1865</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>5625</v>
+        <v>5595</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>305.3999999999999</v>
+        <v>275.3999999999999</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.05741033160387996</v>
+        <v>0.05177080983532593</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1647.97</v>
@@ -1438,13 +1438,13 @@
         <v>1647.97</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.1210826666666667</v>
+        <v>0.1163699731903485</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>60.79</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1468,31 +1468,31 @@
         <v>4102</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2200.6</v>
+        <v>2217.4</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>4401.2</v>
+        <v>4434.8</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>299.1999999999998</v>
+        <v>332.8000000000002</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.07294002925402239</v>
+        <v>0.08113115553388596</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1942.67</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>1953.428571428571</v>
+        <v>1963.742857142857</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1123200166188442</v>
+        <v>0.1143939491553815</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>53.81</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5390,7 +5390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7711,6 +7711,31 @@
         <v>-6348.9</v>
       </c>
       <c r="G92" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B93" s="20" t="n">
+        <v>198496.44</v>
+      </c>
+      <c r="C93" s="20" t="n">
+        <v>111139.44</v>
+      </c>
+      <c r="D93" s="20" t="n">
+        <v>87357</v>
+      </c>
+      <c r="E93" s="20" t="n">
+        <v>82370.39999999999</v>
+      </c>
+      <c r="F93" s="20" t="n">
+        <v>-6348.9</v>
+      </c>
+      <c r="G93" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7794,18 +7819,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>9558.5</v>
+        <v>2244</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>9023</v>
+        <v>2115.61</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -7814,10 +7839,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.836168918096629</v>
+        <v>0.8227190248905368</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7832,18 +7857,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>2181.9</v>
+        <v>47565</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>2056.5</v>
+        <v>45456.43</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -7855,7 +7880,7 @@
         <v>6.1</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8092734574662285</v>
+        <v>0.8227645852234626</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7870,18 +7895,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>SUNDRMFAST</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>47625</v>
+        <v>1071.6</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>45412.14</v>
+        <v>992.47</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -7893,7 +7918,7 @@
         <v>6</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8209748083242059</v>
+        <v>0.8377979172419234</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7908,18 +7933,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>RADICO</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>11014</v>
+        <v>4235</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>10124.14</v>
+        <v>3941.09</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -7928,10 +7953,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7822775952294024</v>
+        <v>0.7617774446767386</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7946,18 +7971,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>4135.1</v>
+        <v>9664</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>3841.43</v>
+        <v>9150.139999999999</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -7966,10 +7991,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7718540829986613</v>
+        <v>0.7634917754723679</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -7984,18 +8009,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SHREEJISPG</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>840.3</v>
+        <v>160</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>786.79</v>
+        <v>151.11</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -8007,7 +8032,7 @@
         <v>5.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7676250456370939</v>
+        <v>0.7607327127135024</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -8022,18 +8047,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>SONACOMS</t>
+          <t>NAZARA</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>879.45</v>
+        <v>405.4</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>819.54</v>
+        <v>373.3</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -8042,10 +8067,10 @@
         <v>5333</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.752354874041621</v>
+        <v>0.7680314386020276</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -8060,18 +8085,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SAILIFE</t>
+          <t>HYUNDAI</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1487.2</v>
+        <v>1922</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1389.76</v>
+        <v>1802.5</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -8083,7 +8108,7 @@
         <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7730497748570038</v>
+        <v>0.7329121139205554</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -8098,18 +8123,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>HYUNDAI</t>
+          <t>APLAPOLLO</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1866.9</v>
+        <v>2195</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>1756.89</v>
+        <v>2061.94</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -8118,10 +8143,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7296914932457101</v>
+        <v>0.7351287917636385</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -8136,18 +8161,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SIRCA</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>413.5</v>
+        <v>5105</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>389.69</v>
+        <v>4776.93</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -8156,10 +8181,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7393270049896555</v>
+        <v>0.7343513076407243</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -8174,18 +8199,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>INDGN</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>598.95</v>
+        <v>1911.7</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>559.5</v>
+        <v>1787.37</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -8194,10 +8219,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7552847754654984</v>
+        <v>0.7694027849000039</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -8212,18 +8237,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>VARROC</t>
+          <t>ZYDUSLIFE</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>807.5</v>
+        <v>1184.4</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>749.1</v>
+        <v>1122.81</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -8232,10 +8257,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7466745770962638</v>
+        <v>0.7407445465662104</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -8250,18 +8275,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>SOMANYCERA</t>
+          <t>CRAFTSMAN</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>543.8</v>
+        <v>10833</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>494.03</v>
+        <v>9887.709999999999</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -8270,10 +8295,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7637337227698674</v>
+        <v>0.7483860597215101</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -8288,18 +8313,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>SIRCA</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1080.2</v>
+        <v>415.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>1004.9</v>
+        <v>392.56</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -8308,10 +8333,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7378270658391139</v>
+        <v>0.7332738353516626</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -8326,18 +8351,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261028</v>
+        <v>20261029</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>VADILALIND</t>
+          <t>CHALET</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>7342</v>
+        <v>815.45</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>6894.07</v>
+        <v>762.63</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -8346,10 +8371,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7232688329073871</v>
+        <v>0.7316456944499231</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V5 daily refresh 2026-10-30
</commit_message>
<xml_diff>
--- a/V5_Live_Tracker.xlsx
+++ b/V5_Live_Tracker.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of Thu 29 Oct 2026</t>
+          <t>As of Fri 30 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>₹198,496</t>
+          <t>₹198,705</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>₹+700  (+0.35%)</t>
+          <t>₹+208  (+0.10%)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-0.65%</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-3.69%</t>
+          <t>-3.59%</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>₹87,357</t>
+          <t>₹87,565</t>
         </is>
       </c>
     </row>
@@ -693,11 +693,11 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
@@ -820,7 +820,7 @@
         <v>49.27</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3">
@@ -844,16 +844,16 @@
         <v>9126</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>810</v>
+        <v>811.65</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>10530</v>
+        <v>10551.45</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>1404</v>
+        <v>1425.45</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1561965811965812</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>683.88</v>
@@ -862,13 +862,13 @@
         <v>722.4071428571428</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>0.1081393298059965</v>
+        <v>0.1099523897527963</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>13.22</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -892,16 +892,16 @@
         <v>7587.6</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1911.7</v>
+        <v>1906.4</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>7646.8</v>
+        <v>7625.6</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>59.19999999999982</v>
+        <v>38</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.007802203595339741</v>
+        <v>0.005008171226738362</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>1777.36</v>
@@ -910,13 +910,13 @@
         <v>1777.36</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>0.07027253230109334</v>
+        <v>0.06768778850188847</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>56.89</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -940,31 +940,31 @@
         <v>7866.4</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>2244</v>
+        <v>2405.5</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>8976</v>
+        <v>9622</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>1109.6</v>
+        <v>1755.6</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0.1410556290043731</v>
+        <v>0.2231770568493848</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>1839.47</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>1987.228571428571</v>
+        <v>2108.642857142857</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>0.1144257703081233</v>
+        <v>0.1234076669537074</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>55</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -988,31 +988,31 @@
         <v>5025</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>352.9</v>
+        <v>349.35</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5293.5</v>
+        <v>5240.25</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>268.4999999999997</v>
+        <v>215.2500000000003</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.05343283582089545</v>
+        <v>0.04283582089552246</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>306.13</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>308.6428571428572</v>
+        <v>310.2285714285714</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>0.1254098692466501</v>
+        <v>0.1119834795231963</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>10.42</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
@@ -1036,16 +1036,16 @@
         <v>4249.2</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>2195</v>
+        <v>2165.1</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>4390</v>
+        <v>4330.2</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>140.8000000000002</v>
+        <v>81</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0.03313564906335315</v>
+        <v>0.01906241174809376</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>1983.64</v>
@@ -1054,13 +1054,13 @@
         <v>1983.64</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>0.09629157175398628</v>
+        <v>0.08381137129924707</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -1084,16 +1084,16 @@
         <v>3760</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>1962</v>
+        <v>2045</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3924</v>
+        <v>4090</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>164</v>
+        <v>330</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.04361702127659575</v>
+        <v>0.08776595744680851</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>1752.11</v>
@@ -1102,13 +1102,13 @@
         <v>1752.11</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.1069775739041795</v>
+        <v>0.1432224938875306</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>57.73</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1132,16 +1132,16 @@
         <v>5306</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>405.4</v>
+        <v>398.8</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5675.599999999999</v>
+        <v>5583.2</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>369.5999999999997</v>
+        <v>277.2000000000002</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0.06965699208443266</v>
+        <v>0.05224274406332457</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>353.13</v>
@@ -1150,13 +1150,13 @@
         <v>358.0214285714286</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>0.1168687011064908</v>
+        <v>0.102253188135836</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>14.18</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1180,31 +1180,31 @@
         <v>4143</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>1495.7</v>
+        <v>1557.5</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4487.1</v>
+        <v>4672.5</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>344.1000000000001</v>
+        <v>529.5</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.08305575669804492</v>
+        <v>0.1278059377262853</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>1285.37</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1310.214285714286</v>
+        <v>1365.157142857143</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.1240126457750313</v>
+        <v>0.123494611327677</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>51.67</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -1228,16 +1228,16 @@
         <v>4150</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>4235</v>
+        <v>4086.7</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>4235</v>
+        <v>4086.7</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>85</v>
+        <v>-63.30000000000018</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>0.02048192771084337</v>
+        <v>-0.01525301204819281</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>3879.27</v>
@@ -1246,13 +1246,13 @@
         <v>3879.27</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.08399763872491145</v>
+        <v>0.05075733476888439</v>
       </c>
       <c r="M11" s="13" t="n">
         <v>144.81</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1276,16 +1276,16 @@
         <v>4585.5</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>804.4</v>
+        <v>766.2</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4826.4</v>
+        <v>4597.200000000001</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>240.8999999999999</v>
+        <v>11.70000000000027</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.05253516519463523</v>
+        <v>0.002551521099116841</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>710.29</v>
@@ -1294,13 +1294,13 @@
         <v>710.29</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.1169940328194928</v>
+        <v>0.07297050378491265</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>27.71</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1324,16 +1324,16 @@
         <v>4984.5</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1011.8</v>
+        <v>997.3</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>5059</v>
+        <v>4986.5</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>74.49999999999989</v>
+        <v>1.999999999999886</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0.0149463336342662</v>
+        <v>0.0004012438559534329</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>949</v>
@@ -1342,13 +1342,13 @@
         <v>949</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.06206760229294322</v>
+        <v>0.04843076306026266</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>32.99</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1372,16 +1372,16 @@
         <v>4920</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1679.4</v>
+        <v>1673.2</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>5038.200000000001</v>
+        <v>5019.6</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>118.2000000000003</v>
+        <v>99.60000000000014</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.0240243902439025</v>
+        <v>0.02024390243902442</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>1536.33</v>
@@ -1390,13 +1390,13 @@
         <v>1536.33</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.0851911396927475</v>
+        <v>0.08180133875209186</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>54.19</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1420,16 +1420,16 @@
         <v>5319.6</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>1865</v>
+        <v>1871.8</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>5595</v>
+        <v>5615.4</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>275.3999999999999</v>
+        <v>295.7999999999997</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0.05177080983532593</v>
+        <v>0.05560568463794265</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>1647.97</v>
@@ -1438,13 +1438,13 @@
         <v>1647.97</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.1163699731903485</v>
+        <v>0.1195800833422374</v>
       </c>
       <c r="M15" s="13" t="n">
         <v>60.79</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -1468,16 +1468,16 @@
         <v>4102</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2217.4</v>
+        <v>2149.6</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>4434.8</v>
+        <v>4299.2</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>332.8000000000002</v>
+        <v>197.1999999999998</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0.08113115553388596</v>
+        <v>0.0480741101901511</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>1942.67</v>
@@ -1486,13 +1486,13 @@
         <v>1963.742857142857</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.1143939491553815</v>
+        <v>0.0864612685416556</v>
       </c>
       <c r="M16" s="13" t="n">
         <v>53.81</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -5390,7 +5390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7736,6 +7736,31 @@
         <v>-6348.9</v>
       </c>
       <c r="G93" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B94" s="20" t="n">
+        <v>198704.84</v>
+      </c>
+      <c r="C94" s="20" t="n">
+        <v>111139.44</v>
+      </c>
+      <c r="D94" s="20" t="n">
+        <v>87565.39999999999</v>
+      </c>
+      <c r="E94" s="20" t="n">
+        <v>82370.39999999999</v>
+      </c>
+      <c r="F94" s="20" t="n">
+        <v>-6348.9</v>
+      </c>
+      <c r="G94" s="14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7819,18 +7844,18 @@
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2244</v>
+        <v>9780</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>2115.61</v>
+        <v>9258.139999999999</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0.0267</v>
@@ -7839,10 +7864,10 @@
         <v>5333</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.8227190248905368</v>
+        <v>0.8338254736114659</v>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
@@ -7857,18 +7882,18 @@
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>LAURUSLABS</t>
         </is>
       </c>
       <c r="C3" s="14" t="n">
-        <v>47565</v>
+        <v>2405.5</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>45456.43</v>
+        <v>2257.07</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0.0267</v>
@@ -7877,10 +7902,10 @@
         <v>5333</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>0.8227645852234626</v>
+        <v>0.8094545768670283</v>
       </c>
       <c r="I3" s="14" t="inlineStr">
         <is>
@@ -7895,18 +7920,18 @@
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>SUNDRMFAST</t>
+          <t>ZYDUSLIFE</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1071.6</v>
+        <v>1245.5</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>992.47</v>
+        <v>1176.97</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0.0267</v>
@@ -7915,10 +7940,10 @@
         <v>5333</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.8377979172419234</v>
+        <v>0.8126853507203702</v>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
@@ -7933,18 +7958,18 @@
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>RADICO</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>4235</v>
+        <v>47200</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>3941.09</v>
+        <v>45107.14</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0.0267</v>
@@ -7953,10 +7978,10 @@
         <v>5333</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.7617774446767386</v>
+        <v>0.8088382434685937</v>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
@@ -7971,18 +7996,18 @@
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>SAILIFE</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>9664</v>
+        <v>1557.5</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>9150.139999999999</v>
+        <v>1461.33</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.0267</v>
@@ -7991,10 +8016,10 @@
         <v>5333</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.7634917754723679</v>
+        <v>0.8038211919534878</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
@@ -8009,18 +8034,18 @@
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>160</v>
+        <v>1681.4</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>151.11</v>
+        <v>1591.84</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0.0267</v>
@@ -8032,7 +8057,7 @@
         <v>5.8</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.7607327127135024</v>
+        <v>0.7794270089989935</v>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
@@ -8047,18 +8072,18 @@
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>NAZARA</t>
+          <t>INDGN</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>405.4</v>
+        <v>586.8</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>373.3</v>
+        <v>550.4</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0.0267</v>
@@ -8070,7 +8095,7 @@
         <v>5.7</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.7680314386020276</v>
+        <v>0.7826401304027762</v>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
@@ -8085,18 +8110,18 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>HYUNDAI</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>1922</v>
+        <v>1906.4</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1802.5</v>
+        <v>1780.36</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>0.0267</v>
@@ -8108,7 +8133,7 @@
         <v>5.7</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.7329121139205554</v>
+        <v>0.7720171116085512</v>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
@@ -8123,18 +8148,18 @@
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>APLAPOLLO</t>
+          <t>SHREEJISPG</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2195</v>
+        <v>843.3</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>2061.94</v>
+        <v>789.61</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>0.0267</v>
@@ -8143,10 +8168,10 @@
         <v>5333</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.7351287917636385</v>
+        <v>0.7376737076153418</v>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -8161,18 +8186,18 @@
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>APLAPOLLO</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>5105</v>
+        <v>2165.1</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>4776.93</v>
+        <v>2038.29</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0.0267</v>
@@ -8181,10 +8206,10 @@
         <v>5333</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.7343513076407243</v>
+        <v>0.7281597884710724</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -8199,18 +8224,18 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>CHALET</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1911.7</v>
+        <v>805.65</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>1787.37</v>
+        <v>751.0700000000001</v>
       </c>
       <c r="E12" s="14" t="n">
         <v>0.0267</v>
@@ -8219,10 +8244,10 @@
         <v>5333</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.7694027849000039</v>
+        <v>0.7543019395159474</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -8237,18 +8262,18 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>ZYDUSLIFE</t>
+          <t>KAJARIACER</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1184.4</v>
+        <v>1109.2</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1122.81</v>
+        <v>1041.51</v>
       </c>
       <c r="E13" s="14" t="n">
         <v>0.0267</v>
@@ -8257,10 +8282,10 @@
         <v>5333</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.7407445465662104</v>
+        <v>0.7374239442332827</v>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -8275,18 +8300,18 @@
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>CRAFTSMAN</t>
+          <t>KIRLFER</t>
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>10833</v>
+        <v>436.5</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>9887.709999999999</v>
+        <v>401.64</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>0.0267</v>
@@ -8295,10 +8320,10 @@
         <v>5333</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.7483860597215101</v>
+        <v>0.7491335276354731</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -8313,18 +8338,18 @@
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SIRCA</t>
+          <t>IPCALAB</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>415.8</v>
+        <v>1927.8</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>392.56</v>
+        <v>1779.83</v>
       </c>
       <c r="E15" s="14" t="n">
         <v>0.0267</v>
@@ -8333,10 +8358,10 @@
         <v>5333</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.7332738353516626</v>
+        <v>0.7272670252242237</v>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -8351,18 +8376,18 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>20261029</v>
+        <v>20261030</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>CHALET</t>
+          <t>SOMANYCERA</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>815.45</v>
+        <v>543</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>762.63</v>
+        <v>493.99</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.0267</v>
@@ -8371,10 +8396,10 @@
         <v>5333</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.7316456944499231</v>
+        <v>0.7298367711791836</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>

</xml_diff>